<commit_message>
før inn DM-03 og DM-04 og rett registerets påstand om prosjektene
Gjennomføringsnotatet for spor M, 1a beskriver DM-01–DM-04. DM-04:
ruteregistertesten ser ikke ruter deklarert med .get/.post, godtar de
utgåtte require_magic_link og require_entra_auth, og kontrollerer ikke
require_project_access. En ny rute uten autentisering ga grønn test; ingen
eksponert rute er funnet. DM-03: migrasjonene legger inn prosjektet oslobygg,
som er basens eneste prosjekt. AGENTS.md sier nå hva testen ikke dekker,
databaseauditen får en datert merknad om upsert_cached_models, og registeret
sier ikke lenger at POST /api/projects er en vei inn.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015fRXUU5uLqM3zyBx5hKfCy
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -847,7 +847,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>To veier: rutene `POST` og `PATCH /api/projects`, og databasefunksjonen `koe_register_project`, som drift kaller gjennom `scripts/catenda_admin.py`. Etter vedtaket i B-02 punkt 4 skal bare drift registrere prosjekter; det er ikke bygget (F1). En migrasjon legger inn prosjektet `oslobygg` som startrad.</t>
+          <t>Registreres av drift gjennom databasefunksjonen `koe_register_project` (`scripts/catenda_admin.py`). `POST /api/projects` svarer 403 utenfor utviklingsmodus. En prosjektadministrator kan endre navn, beskrivelse og innstillinger og deaktivere prosjektet (`PATCH`). At runtime-rollen heller ikke skal kunne kalle funksjonen, gjelder databaserettighetene og hører til F1 (B-02 punkt 4). En migrasjon legger inn prosjektet `oslobygg`, og det er i dag basens eneste prosjekt (DM-03).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -892,17 +892,17 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>backend/routes/project_routes.py; databasefunksjonen koe_register_project</t>
+          <t>databasefunksjonen koe_register_project; backend/routes/project_routes.py (PATCH; POST bare i utviklingsmodus); migrasjonen 20260911073600_projects.sql (startraden)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>MS-10, MS-12</t>
+          <t>MS-10, MS-12, DM-03</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>K 29.09: kolonnene og fremmednøklene i testbasen. L 29.09: rutene, migrasjonene og `scripts/catenda_admin.py`.</t>
+          <t>K 29.09: kolonnene og fremmednøklene i testbasen, startraden i testbasen og en telling i prosjektet. L 29.09: rutene, med vakten mot `POST` utenfor utviklingsmodus, migrasjonene og `scripts/catenda_admin.py`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
før inn oppdragsgivers valg for fila til IKT og arbeidsformen med spørsmål
Excel-fila til IKT har IKTs sju kolonner pluss lagring, type, status og
personopplysninger; belegg, funn og skrivere står bare i tabeller.md. Fila
sendes når 1b og 1c er med. AGENTS.md får regelen om at oppdragsgiver vil ha
konkrete spørsmål med spørsmålsverktøyet, ikke dokumenter å lese, og oppdraget
bruker den for tiltenkt atferd og bestemmelser.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015fRXUU5uLqM3zyBx5hKfCy
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -437,11 +437,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,27 +493,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Kan bygges opp igjen</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>Personopplysninger</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Skrives av</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Funn i hovedplanen</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Belegg</t>
         </is>
       </c>
     </row>
@@ -574,27 +550,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>nei. Journalen er kilden alt annet regnes fra.</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
           <t>`actorid` peker på en bruker. Fritekst i `data` og `comment` kan inneholde personopplysninger. Vurderingen hører til DPIA-en.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>backend/routes/event_routes.py; backend/services/sak_creation_service.py; backend/services/forsering_service.py; backend/services/endringsordre_service.py; backend/services/approval_service.py; backend/services/catenda_webhook_service.py (via sak_creation_service)</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>MS-01, MS-02, MS-03, AR-02</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene i testbasen og prosjektet, og skrankene (også CASCADE) i testbasen. L 29.09: kallerne av `append`/`append_batch` og `create_sak`.</t>
         </is>
       </c>
     </row>
@@ -651,27 +607,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
           <t>`aktor_id` peker på forfatteren. `tekst` og `kommentar` er fritekst.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>backend/routes/event_routes.py; backend/repositories/postgres/notat.py</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>MS-05</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøkkelen i testbasen. L 29.09: sletting i lageret. Skjermingen: AGENTS.md og `lib/auth/event_visibility.py`, ikke kontrollert på nytt 29.09.</t>
         </is>
       </c>
     </row>
@@ -728,27 +664,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>delvis. `cached_*` og `last_event_at` kan regnes ut av hendelsene. Om registerkolonnene også kan det, er ikke kontrollert.</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
           <t>`created_by` identifiserer den som opprettet saken (tre verdiformer, MG-04).</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/sak_creation_service.py; backend/services/endringsordre_service.py; backend/routes/event_routes.py (update_cache); backend/routes/forsering_routes.py (update_cache); backend/routes/approval_routes.py (update_cache)</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>MS-06, MS-07, DA-14, MG-04, DM-01</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene i testbasen og prosjektet, og kolonnekommentarene (DM-01). L 29.09: kallerne av `create` og `update_cache`.</t>
         </is>
       </c>
     </row>
@@ -805,27 +721,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>ikke kontrollert. Koblingene finnes trolig også som hendelser (`FORSERING_KOE_*`, `EO_KOE_*`), men det er ikke sjekket at de to alltid er like.</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/forsering_service.py; backend/services/endringsordre_service.py</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>DA-13, MS-08, DB-04</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fraværet av fremmednøkler i testbasen. L 29.09: kallerne av `add_relation`, `add_relations_batch` og `remove_relation`.</t>
         </is>
       </c>
     </row>
@@ -882,27 +778,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
           <t>`created_by` identifiserer den som opprettet prosjektet.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_register_project; backend/routes/project_routes.py (PATCH; POST bare i utviklingsmodus); migrasjonen 20260911073600_projects.sql (startraden)</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>MS-10, MS-12, DM-03</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøklene i testbasen, startraden i testbasen og en telling i prosjektet. L 29.09: rutene, med vakten mot `POST` utenfor utviklingsmodus, migrasjonene og `scripts/catenda_admin.py`.</t>
         </is>
       </c>
     </row>
@@ -959,27 +835,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>ikke relevant; tabellen skal fjernes.</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
           <t>`user_email`, `display_name`, `external_id`.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>triggerfunksjonen auto_create_project_membership</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>DA-10, MS-15, AR-07</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og triggeren i testbasen. D 20.09: ingen leser (databaseauditen).</t>
         </is>
       </c>
     </row>
@@ -1036,27 +892,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>nei. `id` må være stabil, fordi journalen viser til den.</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
           <t>`email` og `name`.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_resolve_identity</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>MG-02</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøklene i testbasen. L 29.09: funksjonen i migrasjonene og kallerne i `auth_service`, `catenda_webhook_service` og `koe_reconcile_memberships`.</t>
         </is>
       </c>
     </row>
@@ -1113,27 +949,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
           <t>`subject` er en ekstern identifikator for en person.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_resolve_identity</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>DA-07, MG-02</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøkkelen i testbasen. L 29.09: funksjonen i migrasjonene; søket etter tabellnavnet i Python-koden gir bare to docstringer.</t>
         </is>
       </c>
     </row>
@@ -1190,23 +1006,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>nei, men tapet betyr bare at brukerne må logge inn igjen.</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
           <t>Knyttet til en bruker gjennom `user_id`.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>backend/routes/auth_routes.py; backend/scripts/sync_catenda_memberships.py</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene i testbasen. L 29.09: rutene og skriptet.</t>
         </is>
       </c>
     </row>
@@ -1263,23 +1063,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>nei, men radene er kortlevde.</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>backend/routes/auth_routes.py</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene i testbasen. L 29.09: rutene.</t>
         </is>
       </c>
     </row>
@@ -1336,27 +1120,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>delvis. Fra Catenda, bortsett fra `viewer_override`.</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
           <t>`user_email`, `display_name` og `catenda_subject`.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_reconcile_memberships; backend/repositories/auth_repository.py (deactivate_user_projects, viewer_override); backend/routes/membership_routes.py</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>DB-05</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøklene i testbasen. L 29.09: funksjonen i migrasjonene og kallerne i `auth_service` og `membership_routes`.</t>
         </is>
       </c>
     </row>
@@ -1413,23 +1177,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>ja, ved neste synkronisering.</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_reconcile_memberships</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene i testbasen. L 29.09: funksjonen i migrasjonene.</t>
         </is>
       </c>
     </row>
@@ -1486,27 +1234,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_register_project</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>MS-12</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøklene i testbasen. L 29.09: funksjonen og skriptet.</t>
         </is>
       </c>
     </row>
@@ -1563,27 +1291,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_register_project</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>MS-12</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøkkelen i testbasen. L 29.09: funksjonen. Bruken ved webhook er ikke kontrollert 29.09.</t>
         </is>
       </c>
     </row>
@@ -1640,23 +1348,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>nei. Hvilket team som er hvilken side, er et valg drift gjør.</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>databasefunksjonen koe_set_contract_teams; databasefunksjonen koe_register_project</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøkkelen i testbasen. L 29.09: funksjonene og skriptet.</t>
         </is>
       </c>
     </row>
@@ -1713,27 +1405,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>ja, i prinsippet fra Catenda.</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Ingen funnet</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>DM-02, DA-15</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: lesere og skrivere i repoet og Git-historikken. K 29.09: ingen funksjon, trigger eller Edge Function i prosjektet nevner tabellen, og statistikken viser 0 rader.</t>
         </is>
       </c>
     </row>
@@ -1790,27 +1462,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
           <t>`linked_by` identifiserer den som koblet (e-post, lest i ruta).</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>backend/routes/bim_link_routes.py</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>DA-15, MS-13, MS-14</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøkkelen i testbasen. L 29.09: rutene.</t>
         </is>
       </c>
     </row>
@@ -1867,27 +1519,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>ikke relevant; tabellen skal fjernes.</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
           <t>`email`.</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>Ingen funnet</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>DA-09, MS-15</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene i testbasen. D 20.09: ingen lesere. L 29.09: `MagicLinkManager`.</t>
         </is>
       </c>
     </row>
@@ -1944,27 +1576,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>ikke relevant; tabellen skal fjernes.</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
           <t>`display_name`, `department` og koblingen til en bruker.</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Ingen funnet</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>DA-08, MS-15</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>K 29.09: kolonnene og fremmednøklene i testbasen. D 20.09: ingen kallere.</t>
         </is>
       </c>
     </row>
@@ -2021,27 +1633,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
           <t>`oppdatert_av` og fritekst i `innhold`.</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/utkast_registry.py</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>AR-03</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: tabelldefinisjonen og rutene.</t>
         </is>
       </c>
     </row>
@@ -2098,27 +1690,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
           <t>Godkjennere og saksbehandlere i JSON-dokumentet; ikke kontrollert i detalj.</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/approval_service.py</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>AR-03, MG-05</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: tabelldefinisjonen og `ApprovalService`.</t>
         </is>
       </c>
     </row>
@@ -2175,27 +1747,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/approval_service.py</t>
-        </is>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>AR-03</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: tabelldefinisjonen og `publish`/`deliver`.</t>
         </is>
       </c>
     </row>
@@ -2252,27 +1804,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
           <t>Godkjennere i JSON-dokumentet; ikke kontrollert i detalj.</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/eo_approval_service.py</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>AR-03</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: tabelldefinisjonen og `EOApprovalService`.</t>
         </is>
       </c>
     </row>
@@ -2329,27 +1861,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
           <t>Filinnholdet kan inneholde personopplysninger; ikke kontrollert.</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/vedlegg_registry.py</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>AR-03, MS-11</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: tabelldefinisjonen og modulheaderen.</t>
         </is>
       </c>
     </row>
@@ -2406,27 +1918,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
           <t>Ingen kjente.</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>backend/services/catenda_delivery_status.py</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>AR-03</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: tabelldefinisjonen og kallerne i `event_routes`.</t>
         </is>
       </c>
     </row>
@@ -2441,14 +1933,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2472,11 +1963,6 @@
           <t>Hvor fra appen lagres</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Belegg</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2499,11 +1985,6 @@
           <t>Forserings- og endringsordretjenesten (`create_topic`, `create_topic_relations`), webhook-tjenesten, synkroniseringstjenesten og hendelsesrutene (`create_comment`).</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: kallene i tjenestene og rutene. Hvilke hendelser som gir kommentar, er ikke kontrollert (fase 1c).</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2526,11 +2007,6 @@
           <t>Hendelses- og vedleggsrutene og webhook-tjenesten.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: kallene til `upload_document` og `create_document_reference`. Mappestrukturen og navngivingen er ikke kontrollert (B-03).</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2551,11 +2027,6 @@
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>`lib/security/webhook_security.py`, ved hver webhook.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>L 29.09: modulen. Om Redis brukes i et utrullet miljø, er ikke kontrollert.</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2676,60 +2147,24 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Belegg: K</t>
+          <t>Ikke kontrollert</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>kjørt og observert (med dato)</t>
+          <t>Står der påstanden ikke er kontrollert. Registeret bygges i runder.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Belegg: L</t>
+          <t>Detaljer</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>lest i kode eller migrasjonsfil (med dato)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Belegg: D</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>kontrollert i databasekatalogen tidligere (med dato)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Belegg: H</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>historisk dokumentert i en audit</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Ikke kontrollert</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Står der påstanden ikke er kontrollert. Registeret bygges i runder.</t>
+          <t>Hvem som skriver hver tabell, belegg og funn står i docs/datamodell/tabeller.md i repoet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
rett funnene fra code-review av spor M 1c
Kolonne 6 kunne si «Nei» og «fra Catenda» i samme celle. Fire vurderinger
fra 1a er rettet, kvitteringer regnes ikke lenger som data fra Catenda, og
verktøyet feiler på motsigelsen.

Katalogen leser unike indekser og følger bare NOT NULL i SQLite. Vakta for
nøkkelkolonner ser e-post, og vakta for dataflyten ser kall ved bart navn
importert fra klientlaget. ER-diagrammet merker bare koblinger som tegnes,
og tallene hentes fra katalogen. Hovedplanens endringslogg er oppdatert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P2KT8dP9GAxqJ7jn9b8SES
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
+          <t>Delvis. `aktor_rolle` og `aktor_team_id` er utledet av teammedlemskapet i Catenda da notatet ble skrevet. Innholdet kommer fra brukeren. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: fra Catenda i C10 (arket Dataflyt).</t>
+          <t>Delvis. En forsering opprettet gjennom `/api/forsering/opprett` får topicens GUID fra Catenda som sak-ID. Ellers er koblingene appens egne. Dataflyt: fra Catenda i C10 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Nei, ikke direkte. Koblingen til Catenda-prosjektet ligger i `catenda_project_configs`. Dataflyt: fra Catenda i C18, C20 (arket Dataflyt).</t>
+          <t>Delvis. Navnet kan hentes fra Catenda-prosjektet når drift registrerer prosjektet eller kjører `sync-name`. Koblingen til Catenda-prosjektet ligger i `catenda_project_configs`. Dataflyt: fra Catenda i C18, C20 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (sak_id, fag, COALESCE(model_id, ''::text), COALESCE(object_global_id, ''::text)). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Nei. Teamet er en Catenda-team-ID. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
+          <t>Delvis. Teamet og kontraktssiden er utledet av teammedlemskapet i Catenda. Innholdet kommer fra brukeren. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: fra Catenda i C07 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: kvittering for kall til Catenda i C07 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `catenda_item_id` er Catendas ID etter opplasting. Dataflyt: fra Catenda i C05, C08; til Catenda i C08 (arket Dataflyt).</t>
+          <t>Delvis. `catenda_item_id` er Catendas ID etter opplasting. Dataflyt: fra Catenda i C05, C08; til Catenda i C08; kvittering for kall til Catenda i C08 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Nei, men statusen gjelder et kall til Catenda. Dataflyt: fra Catenda i C06 (arket Dataflyt).</t>
+          <t>Nei, men statusen gjelder et kall til Catenda. Dataflyt: kvittering for kall til Catenda i C06 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
pensjoner saksrapporten som automatisk Catenda-vedlegg (B-03)
Bare et frosset brev blir PDF i Catenda. En hendelse uten brev får
kommentar og statussynk, og pdf_uploaded er false. POST /api/events
avviser pdf_base64 og pdf_filename. ReportLabPdfGenerator, lib/pdf_input.py
og testene som bare gjaldt dem er slettet.

Closes #140

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014gApZ93cV81EGy4iEHQe3P
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -5300,7 +5300,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>PDF av brevet eller saken. Et frosset brev i hendelsen gjøres til PDF og må komme gjennom; ellers lages PDF-en på serveren.</t>
+          <t>Det frosne brevet i hendelsen som PDF, og bare det. En hendelse uten brev laster ikke opp noe.</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>`pending` før hendelsen lagres. Så `delivered` bare når PDF, kommentar og status alle lyktes, ellers `failed`.</t>
+          <t>`pending` før hendelsen lagres. Så `delivered` når kommentar og status lyktes, og brevet er lastet opp når hendelsen har et; ellers `failed`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fjern SystemContext, CSV-prototypen og pensjonert Entra- og magic-link-kode
- Fjern /api/validate-user og beskrivelsen i OpenAPI-generatoren.
- Hent klienten i /api/health/catenda fra klientfabrikken; svarene er
  uendret og nå testet for deaktivert, ukonfigurert, tilkoblet og feilet.
- Fjern SystemContext, get_system, CSVRepository og fixtures som bare
  holdt prototypekjeden i live.
- Fjern Entra-dekoratører, MagicLinkManager, Entra-innstillinger og
  ubrukte manager-/generatorparametere. /api/magic-link/verify svarer
  fortsatt 410 og er beskrevet som pensjonert.
- Skriptene create_test_sak og test_full_flow bruker vanlige sakslenker.
- Fjern direkte PyJWT og cryptography; de hentes fortsatt transitivt.
- Oppdater C17 i dataflytregisteret.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A5ERykaPbjBVRQRpevmaVw
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -4115,7 +4115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6863,7 +6863,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>C17 Kontroll av tilkoblingen og en bruker</t>
+          <t>C17 Kontroll av tilkoblingen</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/health/catenda` og `POST /api/validate-user`.</t>
+          <t>`GET /api/health/catenda`.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -6905,12 +6905,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>C17.2</t>
+          <t>C18.1</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>C17 Kontroll av tilkoblingen og en bruker</t>
+          <t>C18 Prosjekt registreres av drift</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -6920,39 +6920,39 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/health/catenda` og `POST /api/validate-user`.</t>
+          <t>`scripts/catenda_admin.py register`.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Catenda: prosjektmedlemmer</t>
+          <t>Catenda: prosjekter</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Appen, lagres ikke</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>GET /v2/projects/{catenda_project_id}/members</t>
+          <t>GET /v2/projects/{catenda_project_id}</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>backend/routes/utility_routes.py:validate_user</t>
+          <t>backend/scripts/catenda_admin.py:cmd_register; backend/scripts/catenda_admin.py:fetch_catenda_project_name; backend/repositories/auth_repository.py:AuthRepository.register_project; databasefunksjon:koe_register_project</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Om en e-post er medlem i det globale Catenda-prosjektet.</t>
+          <t>Prosjektnavnet, når drift ikke har oppgitt det.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>C18.1</t>
+          <t>C18.2</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -6972,39 +6972,39 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Catenda: prosjekter</t>
+          <t>Catenda: team og teammedlemmer</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>GET /v2/projects/{catenda_project_id}</t>
+          <t>GET /v2/projects/{catenda_project_id}/teams</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/catenda_admin.py:cmd_register; backend/scripts/catenda_admin.py:fetch_catenda_project_name; backend/repositories/auth_repository.py:AuthRepository.register_project; databasefunksjon:koe_register_project</t>
+          <t>backend/scripts/catenda_admin.py:cmd_register; backend/repositories/auth_repository.py:AuthRepository.register_project; databasefunksjon:koe_register_project; databasefunksjon:koe_set_contract_teams</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Prosjektnavnet, når drift ikke har oppgitt det.</t>
+          <t>Kontroll av at teamene drift oppgir, finnes i Catenda-prosjektet. ID-ene kommer fra drift.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>C18.2</t>
+          <t>C19.1</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>C18 Prosjekt registreres av drift</t>
+          <t>C19 Kontraktsteam endres av drift</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py register`.</t>
+          <t>`scripts/catenda_admin.py contract-teams` med `--bh` og `--te`.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -7034,24 +7034,24 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/catenda_admin.py:cmd_register; backend/repositories/auth_repository.py:AuthRepository.register_project; databasefunksjon:koe_register_project; databasefunksjon:koe_set_contract_teams</t>
+          <t>backend/scripts/catenda_admin.py:cmd_contract_teams; backend/repositories/auth_repository.py:AuthRepository.set_contract_teams; databasefunksjon:koe_set_contract_teams</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Kontroll av at teamene drift oppgir, finnes i Catenda-prosjektet. ID-ene kommer fra drift.</t>
+          <t>Kontroll av at teamene drift oppgir, finnes i Catenda-prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>C19.1</t>
+          <t>C20.1</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>C19 Kontraktsteam endres av drift</t>
+          <t>C20 Prosjektnavn hentes på nytt av drift</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -7061,77 +7061,30 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py contract-teams` med `--bh` og `--te`.</t>
+          <t>`scripts/catenda_admin.py sync-name`.</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Catenda: team og teammedlemmer</t>
+          <t>Catenda: prosjekter</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>GET /v2/projects/{catenda_project_id}/teams</t>
+          <t>GET /v2/projects/{catenda_project_id}</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/catenda_admin.py:cmd_contract_teams; backend/repositories/auth_repository.py:AuthRepository.set_contract_teams; databasefunksjon:koe_set_contract_teams</t>
+          <t>backend/scripts/catenda_admin.py:fetch_catenda_project_name; backend/scripts/catenda_admin.py:cmd_sync_name</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>Kontroll av at teamene drift oppgir, finnes i Catenda-prosjektet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>C20.1</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>C20 Prosjektnavn hentes på nytt av drift</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>inn</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>`scripts/catenda_admin.py sync-name`.</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Catenda: prosjekter</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>projects</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>GET /v2/projects/{catenda_project_id}</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>backend/scripts/catenda_admin.py:fetch_catenda_project_name; backend/scripts/catenda_admin.py:cmd_sync_name</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>Prosjektnavnet i Catenda, for hvert registrert prosjekt.</t>
         </is>

</xml_diff>

<commit_message>
legg til frist-delen av regelmodulen og håndhev § 33.6.2 fjerde ledd
Regelmodulen får frist.py med testene fra fristDomain.test.ts oversatt.
«Godkjent» krever alle dagene (B-13), og 0 dager med hindring er
«avslått» (oppdragsgiver 04.10). Det subsidiære standpunktet bærer de
godkjente dagene.

Forretningsreglene avviser spesifisert_krav_ok=false på kravet som
besvarte forespørselen (REQUEST_ANSWERED), og krever feltet der
§ 33.6.1-spørsmålet stilles (SPECIFICATION_ASSESSED). Ruta krever det
ikke lenger, fordi skjemaet ikke sender det når spørsmålet er skjult.

Del av #63 og #172.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dsm3Kkz8oA1D8md54UAnn5
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -7637,7 +7637,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Versjonen øker, og kravet settes på nytt. Et spor som er `avslatt`, `under_forhandling` eller `delvis_godkjent`, går tilbake til `sendt`.</t>
+          <t>Versjonen øker, og kravet settes på nytt. Et spor som er `avslatt`, `under_forhandling` eller `delvis_godkjent`, går tilbake til `sendt`. Har kravet dager og venter en forespørsel på svar, merkes kravet som svaret på den (`foresporsel_besvart_krav_id`, § 33.6.2 fjerde ledd).</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Status følger `beregnings_resultat`: `godkjent`, `delvis_godkjent` eller `avslatt`. Godkjente dager, ny sluttdato, varselvurderinger, vilkåret og subsidiært standpunkt settes. Et svar på et krav uten dager avvises (§ 33.7, TFR-06); før det sendes `frist_innsigelse_sendt` eller `frist_foresporsel_sendt`.</t>
+          <t>Status følger `beregnings_resultat`: `godkjent`, `delvis_godkjent` eller `avslatt`. Godkjente dager, ny sluttdato, varselvurderinger, vilkåret og subsidiært standpunkt settes. Et svar på et krav uten dager avvises (§ 33.7, TFR-06); før det sendes `frist_innsigelse_sendt` eller `frist_foresporsel_sendt`. På kravet som besvarte forespørselen med dager, avvises `spesifisert_krav_ok=false` (§ 33.6.2 fjerde ledd, #172). En senere revisjon av kravet kan møtes med § 33.6.1 (oppdragsgiver 04.10). Der § 33.6.1-spørsmålet stilles, må `spesifisert_krav_ok` sendes; ellers ville modellens standardverdi `true` bli lagret som BHs vurdering.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Samme behandling som `respons_frist`, også sperren mot et krav uten dager. Uten `beregnings_resultat` står statusen.</t>
+          <t>Samme behandling som `respons_frist`, også sperren mot et krav uten dager og mot § 33.6.1 på kravet som besvarte forespørselen. Uten `beregnings_resultat` står statusen.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
krev den faste teksten i forespørselen og avvis forespørselsfeltene i fristsvaret
#173a: den faste teksten etter § 33.6.2 første ledd ligger i
backend/constants/frist_foresporsel.json, som modellen og
fristVarselDomain.ts leser. FristForesporselData avviser en forespørsel der
teksten mangler i begrunnelsen eller i brevet. Svarfristen står etter den
faste teksten.

#173b: grenene for varsel og begrunnelse_utsatt i BHs fristsvar er fjernet
fra FristForm, fristDomain.ts og fristBegrunnelse.ts, med testene som låste
dem. Speilet i backend/regler/ står.

#182: FristResponsData avviser har_bh_foresporsel og dato_bh_foresporsel, og
projeksjonen kopierer dem ikke. ResponsEvent velger datatypen etter spor, så
feilen fra riktig type når klienten.

REGELVERSJON økes til 3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YPW3a6EwXYBPQhDDqHk5Ku
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -7748,7 +7748,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>BH ber TE spesifisere fristkravet. TE må da uten ugrunnet opphold angi dager eller begrunne hvorfor grunnlaget mangler, ellers tapes kravet. En egen handling: den setter ikke resultat, gjør ikke sporet avslått og åpner ikke forsering. Forespørselen sendes per brev, så `brev` er påkrevd.</t>
+          <t>BH ber TE spesifisere fristkravet. TE må da uten ugrunnet opphold angi dager eller begrunne hvorfor grunnlaget mangler, ellers tapes kravet. En egen handling: den setter ikke resultat, gjør ikke sporet avslått og åpner ikke forsering. Forespørselen sendes per brev, så `brev` er påkrevd. Den faste teksten i `backend/constants/frist_foresporsel.json` må stå uendret i både `begrunnelse` og brevets begrunnelse (#173).</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>vedtak: nøytralt fristvarsel i 3.1 (23.09); oppdragsgiver, 2026-10-04</t>
+          <t>vedtak: nøytralt fristvarsel i 3.1 (23.09); oppdragsgiver, 2026-10-04 og 2026-10-05</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -8879,7 +8879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E372"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14081,12 +14081,12 @@
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>har_bh_foresporsel</t>
+          <t>begrunnelse_varsel</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>Har BH sendt forespørsel om spesifisering? (§33.6.2). Relevant kun hvis krav er sent.</t>
+          <t>BHs begrunnelse for vurdering av varsling</t>
         </is>
       </c>
     </row>
@@ -14108,12 +14108,12 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>dato_bh_foresporsel</t>
+          <t>vilkar_oppfylt</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>Dato BH sendte forespørsel om spesifisering (§33.6.2) - YYYY-MM-DD. Brukes for å beregne om TEs svar kom i tide.</t>
+          <t>Har forholdet medført en faktisk fremdriftshindring? (§33.1)</t>
         </is>
       </c>
     </row>
@@ -14135,12 +14135,12 @@
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse_varsel</t>
+          <t>beregnings_resultat</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse for vurdering av varsling</t>
+          <t>BHs vurdering av antall dager (ren beregning)</t>
         </is>
       </c>
     </row>
@@ -14162,12 +14162,12 @@
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>vilkar_oppfylt</t>
+          <t>godkjent_dager</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -14177,7 +14177,7 @@
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>Har forholdet medført en faktisk fremdriftshindring? (§33.1)</t>
+          <t>Godkjent antall dager. Innvilges kun hvis Grunnlag også godkjennes.</t>
         </is>
       </c>
     </row>
@@ -14189,12 +14189,12 @@
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>beregnings_resultat</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>BHs vurdering av antall dager (ren beregning)</t>
+          <t>BH-godkjent ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -14216,12 +14216,12 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>godkjent_dager</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -14231,7 +14231,7 @@
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>Godkjent antall dager. Innvilges kun hvis Grunnlag også godkjennes.</t>
+          <t>Samlet begrunnelse</t>
         </is>
       </c>
     </row>
@@ -14243,7 +14243,7 @@
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>frist_for_spesifisering</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
@@ -14258,7 +14258,7 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>BH-godkjent ny sluttdato (YYYY-MM-DD)</t>
+          <t>Frist for TE å levere ytterligere spesifikasjon/fremdriftsplan (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -14270,12 +14270,12 @@
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>subsidiaer_triggers</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av SubsidiaerTrigger</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -14285,7 +14285,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>Samlet begrunnelse</t>
+          <t>Liste over årsaker til subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14297,12 +14297,12 @@
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>frist_for_spesifisering</t>
+          <t>subsidiaer_resultat</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -14312,7 +14312,7 @@
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>Frist for TE å levere ytterligere spesifikasjon/fremdriftsplan (YYYY-MM-DD)</t>
+          <t>Subsidiært beregningsresultat</t>
         </is>
       </c>
     </row>
@@ -14324,12 +14324,12 @@
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_triggers</t>
+          <t>subsidiaer_godkjent_dager</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>liste av SubsidiaerTrigger</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -14339,7 +14339,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Liste over årsaker til subsidiær vurdering</t>
+          <t>Subsidiært godkjent antall dager</t>
         </is>
       </c>
     </row>
@@ -14351,12 +14351,12 @@
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_resultat</t>
+          <t>subsidiaer_begrunnelse</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -14366,7 +14366,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært beregningsresultat</t>
+          <t>BH's begrunnelse for subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14378,34 +14378,34 @@
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_godkjent_dager</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært godkjent antall dager</t>
+          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>respons_frist</t>
+          <t>respons_frist_oppdatert</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_begrunnelse</t>
+          <t>frist_krav_id</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
@@ -14420,34 +14420,34 @@
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>BH's begrunnelse for subsidiær vurdering</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>respons_frist</t>
+          <t>respons_frist_oppdatert</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>vedlegg_ids</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -14459,12 +14459,12 @@
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>frist_krav_id</t>
+          <t>regelversjon</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Versjonen av reglene klienten regnet med (B-13). Kontrolleres mot regler.REGELVERSJON</t>
         </is>
       </c>
     </row>
@@ -14486,12 +14486,12 @@
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_ids</t>
+          <t>brev</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>LetterSnapshot</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -14513,12 +14513,12 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>regelversjon</t>
+          <t>tilleggs_begrunnelse</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -14528,7 +14528,7 @@
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>Versjonen av reglene klienten regnet med (B-13). Kontrolleres mot regler.REGELVERSJON</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -14540,12 +14540,12 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>brev</t>
+          <t>original_respons_id</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>LetterSnapshot</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -14555,7 +14555,7 @@
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Event-ID til original respons som oppdateres (for RESPONS_*_OPPDATERT)</t>
         </is>
       </c>
     </row>
@@ -14567,12 +14567,12 @@
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>tilleggs_begrunnelse</t>
+          <t>respondert_versjon</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hvilken TE-versjon (0-indeksert) denne responsen gjelder. Settes automatisk av backend.</t>
         </is>
       </c>
     </row>
@@ -14594,12 +14594,12 @@
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>original_respons_id</t>
+          <t>frist_varsel_ok</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -14609,7 +14609,7 @@
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>Event-ID til original respons som oppdateres (for RESPONS_*_OPPDATERT)</t>
+          <t>Er varsel om fristforlengelse sendt i tide? (§33.4). None hvis ikke relevant.</t>
         </is>
       </c>
     </row>
@@ -14621,12 +14621,12 @@
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>respondert_versjon</t>
+          <t>spesifisert_krav_ok</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -14636,7 +14636,7 @@
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>Hvilken TE-versjon (0-indeksert) denne responsen gjelder. Settes automatisk av backend.</t>
+          <t>Er spesifisert krav sendt i tide? (§33.6)</t>
         </is>
       </c>
     </row>
@@ -14648,7 +14648,7 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>frist_varsel_ok</t>
+          <t>foresporsel_svar_ok</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
@@ -14663,7 +14663,7 @@
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>Er varsel om fristforlengelse sendt i tide? (§33.4). None hvis ikke relevant.</t>
+          <t>Er svar på forespørsel sendt i tide? (§33.6.2/§5). None hvis ikke relevant.</t>
         </is>
       </c>
     </row>
@@ -14675,12 +14675,12 @@
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>spesifisert_krav_ok</t>
+          <t>begrunnelse_varsel</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -14690,7 +14690,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>Er spesifisert krav sendt i tide? (§33.6)</t>
+          <t>BHs begrunnelse for vurdering av varsling</t>
         </is>
       </c>
     </row>
@@ -14702,7 +14702,7 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>foresporsel_svar_ok</t>
+          <t>vilkar_oppfylt</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
@@ -14717,7 +14717,7 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>Er svar på forespørsel sendt i tide? (§33.6.2/§5). None hvis ikke relevant.</t>
+          <t>Har forholdet medført en faktisk fremdriftshindring? (§33.1)</t>
         </is>
       </c>
     </row>
@@ -14729,12 +14729,12 @@
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>har_bh_foresporsel</t>
+          <t>beregnings_resultat</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -14744,7 +14744,7 @@
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>Har BH sendt forespørsel om spesifisering? (§33.6.2). Relevant kun hvis krav er sent.</t>
+          <t>BHs vurdering av antall dager (ren beregning)</t>
         </is>
       </c>
     </row>
@@ -14756,12 +14756,12 @@
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>dato_bh_foresporsel</t>
+          <t>godkjent_dager</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -14771,7 +14771,7 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>Dato BH sendte forespørsel om spesifisering (§33.6.2) - YYYY-MM-DD. Brukes for å beregne om TEs svar kom i tide.</t>
+          <t>Godkjent antall dager. Innvilges kun hvis Grunnlag også godkjennes.</t>
         </is>
       </c>
     </row>
@@ -14783,7 +14783,7 @@
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse_varsel</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse for vurdering av varsling</t>
+          <t>BH-godkjent ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -14810,12 +14810,12 @@
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>vilkar_oppfylt</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>Har forholdet medført en faktisk fremdriftshindring? (§33.1)</t>
+          <t>Samlet begrunnelse</t>
         </is>
       </c>
     </row>
@@ -14837,12 +14837,12 @@
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>beregnings_resultat</t>
+          <t>frist_for_spesifisering</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -14852,7 +14852,7 @@
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>BHs vurdering av antall dager (ren beregning)</t>
+          <t>Frist for TE å levere ytterligere spesifikasjon/fremdriftsplan (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -14864,12 +14864,12 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>godkjent_dager</t>
+          <t>subsidiaer_triggers</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>liste av SubsidiaerTrigger</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -14879,7 +14879,7 @@
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>Godkjent antall dager. Innvilges kun hvis Grunnlag også godkjennes.</t>
+          <t>Liste over årsaker til subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14891,12 +14891,12 @@
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>subsidiaer_resultat</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>BH-godkjent ny sluttdato (YYYY-MM-DD)</t>
+          <t>Subsidiært beregningsresultat</t>
         </is>
       </c>
     </row>
@@ -14918,12 +14918,12 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>subsidiaer_godkjent_dager</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>Samlet begrunnelse</t>
+          <t>Subsidiært godkjent antall dager</t>
         </is>
       </c>
     </row>
@@ -14945,7 +14945,7 @@
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>frist_for_spesifisering</t>
+          <t>subsidiaer_begrunnelse</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
@@ -14960,7 +14960,7 @@
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>Frist for TE å levere ytterligere spesifikasjon/fremdriftsplan (YYYY-MM-DD)</t>
+          <t>BH's begrunnelse for subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14972,39 +14972,39 @@
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_triggers</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>liste av SubsidiaerTrigger</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>Liste over årsaker til subsidiær vurdering</t>
+          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_oppdatert</t>
+          <t>te_aksepterer_respons</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_resultat</t>
+          <t>kommentar</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -15014,46 +15014,46 @@
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært beregningsresultat</t>
+          <t>Valgfri kommentar fra entreprenør</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_oppdatert</t>
+          <t>te_aksepterer_respons</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_godkjent_dager</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært godkjent antall dager</t>
+          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_oppdatert</t>
+          <t>forsering_varsel</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_begrunnelse</t>
+          <t>frist_krav_id</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
@@ -15063,29 +15063,29 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>BH's begrunnelse for subsidiær vurdering</t>
+          <t>Event-ID til fristkravet som ble avslått</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_oppdatert</t>
+          <t>forsering_varsel</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>respons_frist_id</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -15095,51 +15095,51 @@
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
+          <t>Event-ID til BH's frist-respons som utløste forseringen</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>te_aksepterer_respons</t>
+          <t>forsering_varsel</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>kommentar</t>
+          <t>estimert_kostnad</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t>Valgfri kommentar fra entreprenør</t>
+          <t>Estimert kostnad for forsering i NOK</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>te_aksepterer_respons</t>
+          <t>forsering_varsel</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -15149,7 +15149,7 @@
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
+          <t>Begrunnelse for forsering</t>
         </is>
       </c>
     </row>
@@ -15161,22 +15161,22 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>frist_krav_id</t>
+          <t>bekreft_30_prosent</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
         <is>
-          <t>Event-ID til fristkravet som ble avslått</t>
+          <t>TE bekrefter at estimert kostnad er innenfor dagmulkt + 30%</t>
         </is>
       </c>
     </row>
@@ -15188,7 +15188,7 @@
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_id</t>
+          <t>dato_iverksettelse</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="E234" s="2" t="inlineStr">
         <is>
-          <t>Event-ID til BH's frist-respons som utløste forseringen</t>
+          <t>Dato forsering iverksettes (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -15215,12 +15215,12 @@
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>estimert_kostnad</t>
+          <t>avslatte_dager</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -15230,7 +15230,7 @@
       </c>
       <c r="E235" s="2" t="inlineStr">
         <is>
-          <t>Estimert kostnad for forsering i NOK</t>
+          <t>Antall dager som ble avslått av BH</t>
         </is>
       </c>
     </row>
@@ -15242,12 +15242,12 @@
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>dagmulktsats</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -15257,7 +15257,7 @@
       </c>
       <c r="E236" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for forsering</t>
+          <t>Dagmulktsats i NOK per dag (påkrevd for 30%-beregning)</t>
         </is>
       </c>
     </row>
@@ -15269,7 +15269,7 @@
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>bekreft_30_prosent</t>
+          <t>grunnlag_avslag_trigger</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
@@ -15284,46 +15284,46 @@
       </c>
       <c r="E237" s="2" t="inlineStr">
         <is>
-          <t>TE bekrefter at estimert kostnad er innenfor dagmulkt + 30%</t>
+          <t>True hvis forsering utløses av grunnlagsavslag (ikke direkte frist-avslag)</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>forsering_varsel</t>
+          <t>forsering_respons</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>dato_iverksettelse</t>
+          <t>vurdering_per_sak</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av objekt</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>Dato forsering iverksettes (YYYY-MM-DD)</t>
+          <t>BHs vurdering av forseringsrett per sak</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>forsering_varsel</t>
+          <t>forsering_respons</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>avslatte_dager</t>
+          <t>dager_med_forseringsrett</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
@@ -15333,56 +15333,56 @@
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr">
         <is>
-          <t>Antall dager som ble avslått av BH</t>
+          <t>Antall dager BH mener TE har forseringsrett for</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>forsering_varsel</t>
+          <t>forsering_respons</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>dagmulktsats</t>
+          <t>grunnlag_fortsatt_gyldig</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>Dagmulktsats i NOK per dag (påkrevd for 30%-beregning)</t>
+          <t>BH bekrefter at frist-avslaget fortsatt står ved lag</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>forsering_varsel</t>
+          <t>forsering_respons</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>grunnlag_avslag_trigger</t>
+          <t>grunnlag_begrunnelse</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -15392,7 +15392,7 @@
       </c>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>True hvis forsering utløses av grunnlagsavslag (ikke direkte frist-avslag)</t>
+          <t>BHs begrunnelse hvis grunnlaget bestrides</t>
         </is>
       </c>
     </row>
@@ -15404,12 +15404,12 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>vurdering_per_sak</t>
+          <t>trettiprosent_overholdt</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>liste av objekt</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -15419,7 +15419,7 @@
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>BHs vurdering av forseringsrett per sak</t>
+          <t>BH vurderer om estimert kostnad er innenfor 30%-grensen</t>
         </is>
       </c>
     </row>
@@ -15431,12 +15431,12 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>dager_med_forseringsrett</t>
+          <t>trettiprosent_begrunnelse</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -15446,7 +15446,7 @@
       </c>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>Antall dager BH mener TE har forseringsrett for</t>
+          <t>BHs begrunnelse ved avvik fra 30%-regelen</t>
         </is>
       </c>
     </row>
@@ -15458,7 +15458,7 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>grunnlag_fortsatt_gyldig</t>
+          <t>aksepterer</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
@@ -15468,12 +15468,12 @@
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>BH bekrefter at frist-avslaget fortsatt står ved lag</t>
+          <t>BH aksepterer forsering</t>
         </is>
       </c>
     </row>
@@ -15485,12 +15485,12 @@
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>grunnlag_begrunnelse</t>
+          <t>godkjent_kostnad</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -15500,7 +15500,7 @@
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse hvis grunnlaget bestrides</t>
+          <t>BH's godkjente forseringskostnad (kan være lavere enn estimert)</t>
         </is>
       </c>
     </row>
@@ -15512,22 +15512,22 @@
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>trettiprosent_overholdt</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>BH vurderer om estimert kostnad er innenfor 30%-grensen</t>
+          <t>BH's begrunnelse for aksept/avslag</t>
         </is>
       </c>
     </row>
@@ -15539,12 +15539,12 @@
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>trettiprosent_begrunnelse</t>
+          <t>rigg_varslet_i_tide</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -15554,7 +15554,7 @@
       </c>
       <c r="E247" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse ved avvik fra 30%-regelen</t>
+          <t>Om rigg/drift-varslet var rettidig</t>
         </is>
       </c>
     </row>
@@ -15566,7 +15566,7 @@
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>aksepterer</t>
+          <t>produktivitet_varslet_i_tide</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
@@ -15576,12 +15576,12 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>BH aksepterer forsering</t>
+          <t>Om produktivitets-varslet var rettidig</t>
         </is>
       </c>
     </row>
@@ -15593,7 +15593,7 @@
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>godkjent_kostnad</t>
+          <t>godkjent_rigg_drift</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
@@ -15608,7 +15608,7 @@
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>BH's godkjente forseringskostnad (kan være lavere enn estimert)</t>
+          <t>Godkjent rigg/drift-beløp</t>
         </is>
       </c>
     </row>
@@ -15620,22 +15620,22 @@
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>godkjent_produktivitet</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>BH's begrunnelse for aksept/avslag</t>
+          <t>Godkjent produktivitetsbeløp</t>
         </is>
       </c>
     </row>
@@ -15647,12 +15647,12 @@
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>rigg_varslet_i_tide</t>
+          <t>subsidiaer_triggers</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>Om rigg/drift-varslet var rettidig</t>
+          <t>Triggere for subsidiær vurdering (f.eks. 'grunnlag_bestridt')</t>
         </is>
       </c>
     </row>
@@ -15674,12 +15674,12 @@
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>produktivitet_varslet_i_tide</t>
+          <t>subsidiaer_godkjent_belop</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -15689,7 +15689,7 @@
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>Om produktivitets-varslet var rettidig</t>
+          <t>Subsidiært godkjent beløp</t>
         </is>
       </c>
     </row>
@@ -15701,12 +15701,12 @@
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>godkjent_rigg_drift</t>
+          <t>subsidiaer_begrunnelse</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -15716,51 +15716,51 @@
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>Godkjent rigg/drift-beløp</t>
+          <t>Begrunnelse for subsidiært standpunkt</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>forsering_respons</t>
+          <t>forsering_stoppet</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>godkjent_produktivitet</t>
+          <t>dato_stoppet</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
         <is>
-          <t>Godkjent produktivitetsbeløp</t>
+          <t>Dato forsering ble stoppet (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>forsering_respons</t>
+          <t>forsering_stoppet</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_triggers</t>
+          <t>paalopte_kostnader</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -15770,24 +15770,24 @@
       </c>
       <c r="E255" s="2" t="inlineStr">
         <is>
-          <t>Triggere for subsidiær vurdering (f.eks. 'grunnlag_bestridt')</t>
+          <t>Påløpte kostnader ved stopp i NOK</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>forsering_respons</t>
+          <t>forsering_stoppet</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_godkjent_belop</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -15797,46 +15797,46 @@
       </c>
       <c r="E256" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært godkjent beløp</t>
+          <t>Begrunnelse for stopp</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>forsering_respons</t>
+          <t>forsering_kostnader_oppdatert</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_begrunnelse</t>
+          <t>paalopte_kostnader</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for subsidiært standpunkt</t>
+          <t>Påløpte kostnader i NOK</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>forsering_stoppet</t>
+          <t>forsering_kostnader_oppdatert</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>dato_stoppet</t>
+          <t>kommentar</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
@@ -15846,51 +15846,51 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>Dato forsering ble stoppet (YYYY-MM-DD)</t>
+          <t>Kommentar til kostnadsoppdatering</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>forsering_stoppet</t>
+          <t>forsering_koe_lagt_til</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>paalopte_kostnader</t>
+          <t>koe_sak_id</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t>Påløpte kostnader ved stopp i NOK</t>
+          <t>SAK-ID til KOE som legges til/fjernes</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>forsering_stoppet</t>
+          <t>forsering_koe_lagt_til</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>koe_tittel</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
@@ -15905,24 +15905,24 @@
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for stopp</t>
+          <t>Tittel på KOE for visning</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>forsering_kostnader_oppdatert</t>
+          <t>forsering_koe_fjernet</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>paalopte_kostnader</t>
+          <t>koe_sak_id</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -15932,19 +15932,19 @@
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
-          <t>Påløpte kostnader i NOK</t>
+          <t>SAK-ID til KOE som legges til/fjernes</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>forsering_kostnader_oppdatert</t>
+          <t>forsering_koe_fjernet</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>kommentar</t>
+          <t>koe_tittel</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
@@ -15959,19 +15959,19 @@
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>Kommentar til kostnadsoppdatering</t>
+          <t>Tittel på KOE for visning</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_lagt_til</t>
+          <t>sak_opprettet</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>koe_sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
@@ -15981,24 +15981,24 @@
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E263" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til KOE som legges til/fjernes</t>
+          <t>Prosjekt-ID</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_lagt_til</t>
+          <t>sak_opprettet</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>koe_tittel</t>
+          <t>sakstittel</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
@@ -16008,24 +16008,24 @@
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t>Tittel på KOE for visning</t>
+          <t>Sakstittel</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_fjernet</t>
+          <t>sak_opprettet</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>koe_sak_id</t>
+          <t>catenda_topic_id</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
@@ -16035,24 +16035,24 @@
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E265" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til KOE som legges til/fjernes</t>
+          <t>Catenda topic GUID</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_fjernet</t>
+          <t>sak_opprettet</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>koe_tittel</t>
+          <t>sakstype</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="E266" s="2" t="inlineStr">
         <is>
-          <t>Tittel på KOE for visning</t>
+          <t>Sakstype: 'standard' (KOE), 'endringsordre' (EO), eller 'forsering'</t>
         </is>
       </c>
     </row>
@@ -16079,7 +16079,7 @@
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>prosjekt_navn</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
@@ -16094,7 +16094,7 @@
       </c>
       <c r="E267" s="2" t="inlineStr">
         <is>
-          <t>Prosjekt-ID</t>
+          <t>Prosjektnavn fra Catenda</t>
         </is>
       </c>
     </row>
@@ -16106,7 +16106,7 @@
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>sakstittel</t>
+          <t>byggherre</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
@@ -16116,12 +16116,12 @@
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>Sakstittel</t>
+          <t>Byggherre (BH) - fra topic custom field</t>
         </is>
       </c>
     </row>
@@ -16133,7 +16133,7 @@
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_id</t>
+          <t>leverandor</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
@@ -16148,7 +16148,7 @@
       </c>
       <c r="E269" s="2" t="inlineStr">
         <is>
-          <t>Catenda topic GUID</t>
+          <t>Leverandør/Entreprenør (TE) - fra topic custom field</t>
         </is>
       </c>
     </row>
@@ -16160,12 +16160,12 @@
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>sakstype</t>
+          <t>forsering_data</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>objekt</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -16175,19 +16175,19 @@
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>Sakstype: 'standard' (KOE), 'endringsordre' (EO), eller 'forsering'</t>
+          <t>Forsering-data inkl. avslatte_fristkrav, dato_varslet, estimert_kostnad (kun for forsering-saker)</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>sak_opprettet</t>
+          <t>internt_notat</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_navn</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
@@ -16197,29 +16197,29 @@
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>Prosjektnavn fra Catenda</t>
+          <t>Notat-tekst</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>sak_opprettet</t>
+          <t>internt_notat</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>byggherre</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -16229,19 +16229,19 @@
       </c>
       <c r="E272" s="2" t="inlineStr">
         <is>
-          <t>Byggherre (BH) - fra topic custom field</t>
+          <t>Hvilket spor notatet gjelder</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>sak_opprettet</t>
+          <t>eo_opprettet</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>leverandor</t>
+          <t>eo_nummer</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
@@ -16251,83 +16251,83 @@
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>Leverandør/Entreprenør (TE) - fra topic custom field</t>
+          <t>Endringsordre-nummer</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>sak_opprettet</t>
+          <t>eo_opprettet</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>forsering_data</t>
+          <t>beskrivelse</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>objekt</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
-          <t>Forsering-data inkl. avslatte_fristkrav, dato_varslet, estimert_kostnad (kun for forsering-saker)</t>
+          <t>Beskrivelse av endringen</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>internt_notat</t>
+          <t>eo_opprettet</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>relaterte_koe_saker</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
-          <t>Notat-tekst</t>
+          <t>SAK-IDs til KOE-er som inngår</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>internt_notat</t>
+          <t>eo_opprettet</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>sakstittel</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -16337,7 +16337,7 @@
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
-          <t>Hvilket spor notatet gjelder</t>
+          <t>Sakstittel for EO-saken</t>
         </is>
       </c>
     </row>
@@ -16349,7 +16349,7 @@
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>eo_nummer</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
@@ -16359,12 +16359,12 @@
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
         <is>
-          <t>Endringsordre-nummer</t>
+          <t>Prosjekt-ID</t>
         </is>
       </c>
     </row>
@@ -16376,7 +16376,7 @@
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>beskrivelse</t>
+          <t>catenda_topic_id</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
@@ -16386,51 +16386,51 @@
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringen</t>
+          <t>Catenda topic GUID</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>eo_opprettet</t>
+          <t>eo_koe_lagt_til</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>relaterte_koe_saker</t>
+          <t>koe_sak_id</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>SAK-IDs til KOE-er som inngår</t>
+          <t>SAK-ID til KOE som legges til/fjernes</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>eo_opprettet</t>
+          <t>eo_koe_lagt_til</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>sakstittel</t>
+          <t>koe_tittel</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
@@ -16445,19 +16445,19 @@
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
-          <t>Sakstittel for EO-saken</t>
+          <t>Tittel på KOE for visning</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>eo_opprettet</t>
+          <t>eo_koe_fjernet</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>koe_sak_id</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
@@ -16467,24 +16467,24 @@
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>Prosjekt-ID</t>
+          <t>SAK-ID til KOE som legges til/fjernes</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>eo_opprettet</t>
+          <t>eo_koe_fjernet</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_id</t>
+          <t>koe_tittel</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
@@ -16499,19 +16499,19 @@
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>Catenda topic GUID</t>
+          <t>Tittel på KOE for visning</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_lagt_til</t>
+          <t>eo_utstedt</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>koe_sak_id</t>
+          <t>eo_nummer</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
@@ -16526,24 +16526,24 @@
       </c>
       <c r="E283" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til KOE som legges til/fjernes</t>
+          <t>Endringsordre-nummer</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_lagt_til</t>
+          <t>eo_utstedt</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>koe_tittel</t>
+          <t>revisjon_nummer</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -16553,19 +16553,19 @@
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
-          <t>Tittel på KOE for visning</t>
+          <t>Revisjonsnummer</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_fjernet</t>
+          <t>eo_utstedt</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>koe_sak_id</t>
+          <t>beskrivelse</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
@@ -16580,24 +16580,24 @@
       </c>
       <c r="E285" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til KOE som legges til/fjernes</t>
+          <t>Beskrivelse av endringen</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_fjernet</t>
+          <t>eo_utstedt</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>koe_tittel</t>
+          <t>vedlegg_ids</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>Tittel på KOE for visning</t>
+          <t>Vedlegg-IDer</t>
         </is>
       </c>
     </row>
@@ -16619,22 +16619,22 @@
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>eo_nummer</t>
+          <t>konsekvenser</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>EOKonsekvenser</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>Endringsordre-nummer</t>
+          <t>Konsekvenser av endringen</t>
         </is>
       </c>
     </row>
@@ -16646,12 +16646,12 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>revisjon_nummer</t>
+          <t>konsekvens_beskrivelse</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -16661,7 +16661,7 @@
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>Revisjonsnummer</t>
+          <t>Beskrivelse av konsekvensene</t>
         </is>
       </c>
     </row>
@@ -16673,22 +16673,22 @@
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>beskrivelse</t>
+          <t>vederlag</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>VederlagKompensasjon</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringen</t>
+          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
         </is>
       </c>
     </row>
@@ -16700,12 +16700,12 @@
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_ids</t>
+          <t>oppgjorsform</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -16715,7 +16715,7 @@
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>Vedlegg-IDer</t>
+          <t>DEPRECATED: Bruk vederlag.metode</t>
         </is>
       </c>
     </row>
@@ -16727,12 +16727,12 @@
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>konsekvenser</t>
+          <t>kompensasjon_belop</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>EOKonsekvenser</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
-          <t>Konsekvenser av endringen</t>
+          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>konsekvens_beskrivelse</t>
+          <t>fradrag_belop</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -16769,7 +16769,7 @@
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av konsekvensene</t>
+          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
         </is>
       </c>
     </row>
@@ -16781,12 +16781,12 @@
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>vederlag</t>
+          <t>er_estimat</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>VederlagKompensasjon</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -16796,7 +16796,7 @@
       </c>
       <c r="E293" s="2" t="inlineStr">
         <is>
-          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
+          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
         </is>
       </c>
     </row>
@@ -16808,12 +16808,12 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>oppgjorsform</t>
+          <t>frist_dager</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -16823,7 +16823,7 @@
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.metode</t>
+          <t>Fristforlengelse i dager</t>
         </is>
       </c>
     </row>
@@ -16835,12 +16835,12 @@
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>kompensasjon_belop</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -16850,7 +16850,7 @@
       </c>
       <c r="E295" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
+          <t>Ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -16862,12 +16862,12 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>fradrag_belop</t>
+          <t>relaterte_koe_saker</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -16877,7 +16877,7 @@
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
+          <t>SAK-IDs til KOE-er som inngår</t>
         </is>
       </c>
     </row>
@@ -16889,12 +16889,12 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>er_estimat</t>
+          <t>relaterte_sak_ids</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -16904,7 +16904,7 @@
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
+          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
         </is>
       </c>
     </row>
@@ -16916,22 +16916,22 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>frist_dager</t>
+          <t>netto_belop</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>Fristforlengelse i dager</t>
+          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
         </is>
       </c>
     </row>
@@ -16943,22 +16943,22 @@
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>har_priskonsekvens</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>Ny sluttdato (YYYY-MM-DD)</t>
+          <t>Sjekker om EO har priskonsekvens</t>
         </is>
       </c>
     </row>
@@ -16970,39 +16970,39 @@
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>relaterte_koe_saker</t>
+          <t>har_fristkonsekvens</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>SAK-IDs til KOE-er som inngår</t>
+          <t>Sjekker om EO har fristkonsekvens</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>eo_utstedt</t>
+          <t>eo_akseptert</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>relaterte_sak_ids</t>
+          <t>akseptert</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -17012,127 +17012,127 @@
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
-          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
+          <t>Om TE aksepterer</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>eo_utstedt</t>
+          <t>eo_akseptert</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>netto_belop</t>
+          <t>kommentar</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
+          <t>TEs kommentar</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>eo_utstedt</t>
+          <t>eo_bestridt</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>har_priskonsekvens</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har priskonsekvens</t>
+          <t>Begrunnelse for bestridelse</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>eo_utstedt</t>
+          <t>eo_bestridt</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>har_fristkonsekvens</t>
+          <t>nytt_koe_sak_id</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har fristkonsekvens</t>
+          <t>SAK-ID til nytt KOE som fremmes som alternativ</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>eo_akseptert</t>
+          <t>eo_revidert</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>akseptert</t>
+          <t>ny_revisjon_nummer</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>Om TE aksepterer</t>
+          <t>Nytt revisjonsnummer</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>eo_akseptert</t>
+          <t>eo_revidert</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>kommentar</t>
+          <t>endringer_beskrivelse</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
@@ -17142,56 +17142,56 @@
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>TEs kommentar</t>
+          <t>Beskrivelse av endringene</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>eo_bestridt</t>
+          <t>eo_revidert</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>oppdatert_data</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>EOUtstedtData</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for bestridelse</t>
+          <t>Oppdatert EO-data (hvis endret)</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>eo_bestridt</t>
+          <t>Delmodell EOKonsekvenser</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>nytt_koe_sak_id</t>
+          <t>sha</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -17201,78 +17201,78 @@
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til nytt KOE som fremmes som alternativ</t>
+          <t>SHA-konsekvenser</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>eo_revidert</t>
+          <t>Delmodell EOKonsekvenser</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>ny_revisjon_nummer</t>
+          <t>kvalitet</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>Nytt revisjonsnummer</t>
+          <t>Kvalitetskonsekvenser</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>eo_revidert</t>
+          <t>Delmodell EOKonsekvenser</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>endringer_beskrivelse</t>
+          <t>fremdrift</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringene</t>
+          <t>Fremdriftskonsekvenser</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>eo_revidert</t>
+          <t>Delmodell EOKonsekvenser</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>oppdatert_data</t>
+          <t>pris</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>EOUtstedtData</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>Oppdatert EO-data (hvis endret)</t>
+          <t>Priskonsekvenser</t>
         </is>
       </c>
     </row>
@@ -17294,7 +17294,7 @@
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>sha</t>
+          <t>annet</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
@@ -17309,51 +17309,51 @@
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>SHA-konsekvenser</t>
+          <t>Andre konsekvenser</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOKonsekvenser</t>
+          <t>Delmodell EOUtstedtData</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>kvalitet</t>
+          <t>eo_nummer</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>Kvalitetskonsekvenser</t>
+          <t>Endringsordre-nummer</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOKonsekvenser</t>
+          <t>Delmodell EOUtstedtData</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>fremdrift</t>
+          <t>revisjon_nummer</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -17363,51 +17363,51 @@
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>Fremdriftskonsekvenser</t>
+          <t>Revisjonsnummer</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOKonsekvenser</t>
+          <t>Delmodell EOUtstedtData</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>pris</t>
+          <t>beskrivelse</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
-          <t>Priskonsekvenser</t>
+          <t>Beskrivelse av endringen</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOKonsekvenser</t>
+          <t>Delmodell EOUtstedtData</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>annet</t>
+          <t>vedlegg_ids</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
@@ -17417,7 +17417,7 @@
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
-          <t>Andre konsekvenser</t>
+          <t>Vedlegg-IDer</t>
         </is>
       </c>
     </row>
@@ -17429,22 +17429,22 @@
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>eo_nummer</t>
+          <t>konsekvenser</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>EOKonsekvenser</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
         <is>
-          <t>Endringsordre-nummer</t>
+          <t>Konsekvenser av endringen</t>
         </is>
       </c>
     </row>
@@ -17456,12 +17456,12 @@
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>revisjon_nummer</t>
+          <t>konsekvens_beskrivelse</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
@@ -17471,7 +17471,7 @@
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>Revisjonsnummer</t>
+          <t>Beskrivelse av konsekvensene</t>
         </is>
       </c>
     </row>
@@ -17483,22 +17483,22 @@
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>beskrivelse</t>
+          <t>vederlag</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>VederlagKompensasjon</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringen</t>
+          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
         </is>
       </c>
     </row>
@@ -17510,12 +17510,12 @@
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_ids</t>
+          <t>oppgjorsform</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
@@ -17525,7 +17525,7 @@
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>Vedlegg-IDer</t>
+          <t>DEPRECATED: Bruk vederlag.metode</t>
         </is>
       </c>
     </row>
@@ -17537,12 +17537,12 @@
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>konsekvenser</t>
+          <t>kompensasjon_belop</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>EOKonsekvenser</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="E321" s="2" t="inlineStr">
         <is>
-          <t>Konsekvenser av endringen</t>
+          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
         </is>
       </c>
     </row>
@@ -17564,12 +17564,12 @@
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>konsekvens_beskrivelse</t>
+          <t>fradrag_belop</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -17579,7 +17579,7 @@
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av konsekvensene</t>
+          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
         </is>
       </c>
     </row>
@@ -17591,12 +17591,12 @@
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>vederlag</t>
+          <t>er_estimat</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>VederlagKompensasjon</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="E323" s="2" t="inlineStr">
         <is>
-          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
+          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>oppgjorsform</t>
+          <t>frist_dager</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -17633,7 +17633,7 @@
       </c>
       <c r="E324" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.metode</t>
+          <t>Fristforlengelse i dager</t>
         </is>
       </c>
     </row>
@@ -17645,12 +17645,12 @@
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>kompensasjon_belop</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
@@ -17660,7 +17660,7 @@
       </c>
       <c r="E325" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
+          <t>Ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -17672,12 +17672,12 @@
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>fradrag_belop</t>
+          <t>relaterte_koe_saker</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
@@ -17687,7 +17687,7 @@
       </c>
       <c r="E326" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
+          <t>SAK-IDs til KOE-er som inngår</t>
         </is>
       </c>
     </row>
@@ -17699,12 +17699,12 @@
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>er_estimat</t>
+          <t>relaterte_sak_ids</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -17714,7 +17714,7 @@
       </c>
       <c r="E327" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
+          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
         </is>
       </c>
     </row>
@@ -17726,22 +17726,22 @@
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>frist_dager</t>
+          <t>netto_belop</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>Fristforlengelse i dager</t>
+          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
         </is>
       </c>
     </row>
@@ -17753,22 +17753,22 @@
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>har_priskonsekvens</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
         <is>
-          <t>Ny sluttdato (YYYY-MM-DD)</t>
+          <t>Sjekker om EO har priskonsekvens</t>
         </is>
       </c>
     </row>
@@ -17780,39 +17780,39 @@
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>relaterte_koe_saker</t>
+          <t>har_fristkonsekvens</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>SAK-IDs til KOE-er som inngår</t>
+          <t>Sjekker om EO har fristkonsekvens</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOUtstedtData</t>
+          <t>Delmodell KonsekvensVarsler</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>relaterte_sak_ids</t>
+          <t>vederlag</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
@@ -17822,100 +17822,100 @@
       </c>
       <c r="E331" s="2" t="inlineStr">
         <is>
-          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOUtstedtData</t>
+          <t>Delmodell KonsekvensVarsler</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>netto_belop</t>
+          <t>rigg_drift</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOUtstedtData</t>
+          <t>Delmodell KonsekvensVarsler</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>har_priskonsekvens</t>
+          <t>produktivitet</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har priskonsekvens</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOUtstedtData</t>
+          <t>Delmodell KonsekvensVarsler</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>har_fristkonsekvens</t>
+          <t>frist</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har fristkonsekvens</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>Delmodell KonsekvensVarsler</t>
+          <t>Delmodell LetterParty</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>vederlag</t>
+          <t>navn</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
@@ -17925,7 +17925,7 @@
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -17937,12 +17937,12 @@
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>Delmodell KonsekvensVarsler</t>
+          <t>Delmodell LetterParty</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>rigg_drift</t>
+          <t>rolle</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -17964,12 +17964,12 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>Delmodell KonsekvensVarsler</t>
+          <t>Delmodell LetterParty</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>produktivitet</t>
+          <t>adresse</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
@@ -17991,12 +17991,12 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>Delmodell KonsekvensVarsler</t>
+          <t>Delmodell LetterParty</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>frist</t>
+          <t>orgnr</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
@@ -18018,12 +18018,12 @@
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterParty</t>
+          <t>Delmodell LetterReferences</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>navn</t>
+          <t>sakId</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
@@ -18045,12 +18045,12 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterParty</t>
+          <t>Delmodell LetterReferences</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>rolle</t>
+          <t>sakstittel</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
@@ -18072,12 +18072,12 @@
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterParty</t>
+          <t>Delmodell LetterReferences</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>adresse</t>
+          <t>eventId</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
@@ -18099,12 +18099,12 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterParty</t>
+          <t>Delmodell LetterReferences</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>orgnr</t>
+          <t>sporType</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
@@ -18131,7 +18131,7 @@
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>sakId</t>
+          <t>dato</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
@@ -18158,7 +18158,7 @@
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>sakstittel</t>
+          <t>kravDato</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
@@ -18168,7 +18168,7 @@
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -18180,12 +18180,12 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterReferences</t>
+          <t>Delmodell LetterSection</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>eventId</t>
+          <t>tittel</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
@@ -18207,12 +18207,12 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterReferences</t>
+          <t>Delmodell LetterSection</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>sporType</t>
+          <t>originalTekst</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
@@ -18234,12 +18234,12 @@
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterReferences</t>
+          <t>Delmodell LetterSection</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>dato</t>
+          <t>redigertTekst</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
@@ -18261,22 +18261,22 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterReferences</t>
+          <t>Delmodell LetterSections</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>kravDato</t>
+          <t>innledning</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterSection</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
@@ -18288,17 +18288,17 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSection</t>
+          <t>Delmodell LetterSections</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>tittel</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterSection</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
@@ -18315,17 +18315,17 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSection</t>
+          <t>Delmodell LetterSections</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>originalTekst</t>
+          <t>avslutning</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterSection</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -18342,12 +18342,12 @@
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSection</t>
+          <t>Delmodell LetterSnapshot</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>redigertTekst</t>
+          <t>tittel</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -18369,17 +18369,17 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSections</t>
+          <t>Delmodell LetterSnapshot</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>innledning</t>
+          <t>mottaker</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>LetterSection</t>
+          <t>LetterParty</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
@@ -18396,17 +18396,17 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSections</t>
+          <t>Delmodell LetterSnapshot</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>avsender</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>LetterSection</t>
+          <t>LetterParty</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
@@ -18423,17 +18423,17 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSections</t>
+          <t>Delmodell LetterSnapshot</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>avslutning</t>
+          <t>referanser</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>LetterSection</t>
+          <t>LetterReferences</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -18455,12 +18455,12 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>tittel</t>
+          <t>seksjoner</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterSections</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
@@ -18477,125 +18477,125 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSnapshot</t>
+          <t>Delmodell SaerskiltKrav</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>mottaker</t>
+          <t>rigg_drift</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>LetterParty</t>
+          <t>SaerskiltKravItem</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rigg/drift krav (§34.1.3 første ledd)</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSnapshot</t>
+          <t>Delmodell SaerskiltKrav</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>avsender</t>
+          <t>produktivitet</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>LetterParty</t>
+          <t>SaerskiltKravItem</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Produktivitetstap krav (§34.1.3 annet ledd)</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSnapshot</t>
+          <t>Delmodell SaerskiltKravItem</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>referanser</t>
+          <t>belop</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>LetterReferences</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Beløp for dette særskilte kravet</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSnapshot</t>
+          <t>Delmodell SaerskiltKravItem</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>seksjoner</t>
+          <t>dato_klar_over</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>LetterSections</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Når TE ble klar over at utgifter ville påløpe (YYYY-MM-DD). Brukes til 7-dagers varslingssjekk.</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKrav</t>
+          <t>Delmodell VarselInfo</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>rigg_drift</t>
+          <t>dato_sendt</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>SaerskiltKravItem</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -18605,24 +18605,24 @@
       </c>
       <c r="E360" s="2" t="inlineStr">
         <is>
-          <t>Rigg/drift krav (§34.1.3 første ledd)</t>
+          <t>Når varselet faktisk ble sendt til BH (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKrav</t>
+          <t>Delmodell VarselInfo</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>produktivitet</t>
+          <t>metode</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>SaerskiltKravItem</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
@@ -18632,51 +18632,51 @@
       </c>
       <c r="E361" s="2" t="inlineStr">
         <is>
-          <t>Produktivitetstap krav (§34.1.3 annet ledd)</t>
+          <t>Metoder brukt for å varsle (f.eks. ['epost', 'byggemote', 'telefon'])</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKravItem</t>
+          <t>Delmodell VederlagKompensasjon</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>belop</t>
+          <t>metode</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>VederlagsMetode</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
         <is>
-          <t>Beløp for dette særskilte kravet</t>
+          <t>Vederlagsmetode etter NS 8407 (§34)</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKravItem</t>
+          <t>Delmodell VederlagKompensasjon</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>dato_klar_over</t>
+          <t>belop_direkte</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
@@ -18686,24 +18686,24 @@
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>Når TE ble klar over at utgifter ville påløpe (YYYY-MM-DD). Brukes til 7-dagers varslingssjekk.</t>
+          <t>For ENHETSPRISER/FASTPRIS_TILBUD: Beløp i NOK</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>Delmodell VarselInfo</t>
+          <t>Delmodell VederlagKompensasjon</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>dato_sendt</t>
+          <t>kostnads_overslag</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -18713,24 +18713,24 @@
       </c>
       <c r="E364" s="2" t="inlineStr">
         <is>
-          <t>Når varselet faktisk ble sendt til BH (YYYY-MM-DD)</t>
+          <t>For REGNINGSARBEID (§30.2): Kostnadsoverslag i NOK</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>Delmodell VarselInfo</t>
+          <t>Delmodell VederlagKompensasjon</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>metode</t>
+          <t>fradrag_belop</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -18740,7 +18740,7 @@
       </c>
       <c r="E365" s="2" t="inlineStr">
         <is>
-          <t>Metoder brukt for å varsle (f.eks. ['epost', 'byggemote', 'telefon'])</t>
+          <t>Fradrag i NOK (§34.4) - reduksjon for besparelser</t>
         </is>
       </c>
     </row>
@@ -18752,22 +18752,22 @@
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>metode</t>
+          <t>er_estimat</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>VederlagsMetode</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
         <is>
-          <t>Vederlagsmetode etter NS 8407 (§34)</t>
+          <t>Om beløpet er et estimat (endelig oppgjør senere)</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18779,7 @@
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>belop_direkte</t>
+          <t>netto_belop</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
@@ -18789,12 +18789,12 @@
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>For ENHETSPRISER/FASTPRIS_TILBUD: Beløp i NOK</t>
+          <t>Beregner netto beløp basert på metode. For ENHETSPRISER/FASTPRIS_TILBUD: belop_direkte - fradrag For REGNINGSARBEID: kostnads_overslag - fradrag</t>
         </is>
       </c>
     </row>
@@ -18806,7 +18806,7 @@
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>kostnads_overslag</t>
+          <t>krevd_belop</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
@@ -18816,118 +18816,10 @@
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
-        <is>
-          <t>For REGNINGSARBEID (§30.2): Kostnadsoverslag i NOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" s="2" t="inlineStr">
-        <is>
-          <t>Delmodell VederlagKompensasjon</t>
-        </is>
-      </c>
-      <c r="B369" s="2" t="inlineStr">
-        <is>
-          <t>fradrag_belop</t>
-        </is>
-      </c>
-      <c r="C369" s="2" t="inlineStr">
-        <is>
-          <t>tall</t>
-        </is>
-      </c>
-      <c r="D369" s="2" t="inlineStr">
-        <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="E369" s="2" t="inlineStr">
-        <is>
-          <t>Fradrag i NOK (§34.4) - reduksjon for besparelser</t>
-        </is>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" s="2" t="inlineStr">
-        <is>
-          <t>Delmodell VederlagKompensasjon</t>
-        </is>
-      </c>
-      <c r="B370" s="2" t="inlineStr">
-        <is>
-          <t>er_estimat</t>
-        </is>
-      </c>
-      <c r="C370" s="2" t="inlineStr">
-        <is>
-          <t>ja/nei</t>
-        </is>
-      </c>
-      <c r="D370" s="2" t="inlineStr">
-        <is>
-          <t>nei</t>
-        </is>
-      </c>
-      <c r="E370" s="2" t="inlineStr">
-        <is>
-          <t>Om beløpet er et estimat (endelig oppgjør senere)</t>
-        </is>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" s="2" t="inlineStr">
-        <is>
-          <t>Delmodell VederlagKompensasjon</t>
-        </is>
-      </c>
-      <c r="B371" s="2" t="inlineStr">
-        <is>
-          <t>netto_belop</t>
-        </is>
-      </c>
-      <c r="C371" s="2" t="inlineStr">
-        <is>
-          <t>tall</t>
-        </is>
-      </c>
-      <c r="D371" s="2" t="inlineStr">
-        <is>
-          <t>beregnet</t>
-        </is>
-      </c>
-      <c r="E371" s="2" t="inlineStr">
-        <is>
-          <t>Beregner netto beløp basert på metode. For ENHETSPRISER/FASTPRIS_TILBUD: belop_direkte - fradrag For REGNINGSARBEID: kostnads_overslag - fradrag</t>
-        </is>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" s="2" t="inlineStr">
-        <is>
-          <t>Delmodell VederlagKompensasjon</t>
-        </is>
-      </c>
-      <c r="B372" s="2" t="inlineStr">
-        <is>
-          <t>krevd_belop</t>
-        </is>
-      </c>
-      <c r="C372" s="2" t="inlineStr">
-        <is>
-          <t>tall</t>
-        </is>
-      </c>
-      <c r="D372" s="2" t="inlineStr">
-        <is>
-          <t>beregnet</t>
-        </is>
-      </c>
-      <c r="E372" s="2" t="inlineStr">
         <is>
           <t>Alias for netto_belop - brukes i state-modellen. Returnerer det totale kravet/kompensasjonen.</t>
         </is>

</xml_diff>

<commit_message>
krev nytt grunnlagssvar ved endret underkategori, og la projeksjonen holde sakstype og svarfrist
#215 (B-13, vedtak 05.10): endrer TE underkategorien etter BHs svar på
grunnlaget, faller hele svaret i tilstanden: resultat, begrunnelse, § 32.2-
vurdering, låsing og TEs aksept. Grunnlaget er SENDT igjen. Vederlag og frist
som var besvart subsidiært, forblir subsidiære til grunnlaget er besvart på
nytt (subsidiaert_til_nytt_svar).

#233: sakstypen settes bare av sak_opprettet. eo_opprettet i en sak som ikke
er en endringsordresak, endrer ikke tilstanden, også ved gjenspilling.

#238: FristResponsData har ikke lenger frist_for_spesifisering, og et nytt
fristsvar med feltet avvises. Projeksjonen kopierer det ikke.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H8NHZL4Xe5wsYMp3ARGAJW
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -8879,7 +8879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14243,12 +14243,12 @@
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>frist_for_spesifisering</t>
+          <t>subsidiaer_triggers</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av SubsidiaerTrigger</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
@@ -14258,7 +14258,7 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>Frist for TE å levere ytterligere spesifikasjon/fremdriftsplan (YYYY-MM-DD)</t>
+          <t>Liste over årsaker til subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14270,12 +14270,12 @@
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_triggers</t>
+          <t>subsidiaer_resultat</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>liste av SubsidiaerTrigger</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -14285,7 +14285,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>Liste over årsaker til subsidiær vurdering</t>
+          <t>Subsidiært beregningsresultat</t>
         </is>
       </c>
     </row>
@@ -14297,12 +14297,12 @@
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_resultat</t>
+          <t>subsidiaer_godkjent_dager</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -14312,7 +14312,7 @@
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært beregningsresultat</t>
+          <t>Subsidiært godkjent antall dager</t>
         </is>
       </c>
     </row>
@@ -14324,12 +14324,12 @@
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_godkjent_dager</t>
+          <t>subsidiaer_begrunnelse</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -14339,7 +14339,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært godkjent antall dager</t>
+          <t>BH's begrunnelse for subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14351,49 +14351,49 @@
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_begrunnelse</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>BH's begrunnelse for subsidiær vurdering</t>
+          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>respons_frist</t>
+          <t>respons_frist_oppdatert</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>frist_krav_id</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -14405,12 +14405,12 @@
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>frist_krav_id</t>
+          <t>vedlegg_ids</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -14432,12 +14432,12 @@
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_ids</t>
+          <t>regelversjon</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Versjonen av reglene klienten regnet med (B-13). Kontrolleres mot regler.REGELVERSJON</t>
         </is>
       </c>
     </row>
@@ -14459,12 +14459,12 @@
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>regelversjon</t>
+          <t>brev</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>LetterSnapshot</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>Versjonen av reglene klienten regnet med (B-13). Kontrolleres mot regler.REGELVERSJON</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -14486,12 +14486,12 @@
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>brev</t>
+          <t>tilleggs_begrunnelse</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>LetterSnapshot</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -14513,7 +14513,7 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>tilleggs_begrunnelse</t>
+          <t>original_respons_id</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
@@ -14528,7 +14528,7 @@
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Event-ID til original respons som oppdateres (for RESPONS_*_OPPDATERT)</t>
         </is>
       </c>
     </row>
@@ -14540,12 +14540,12 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>original_respons_id</t>
+          <t>respondert_versjon</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -14555,7 +14555,7 @@
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>Event-ID til original respons som oppdateres (for RESPONS_*_OPPDATERT)</t>
+          <t>Hvilken TE-versjon (0-indeksert) denne responsen gjelder. Settes automatisk av backend.</t>
         </is>
       </c>
     </row>
@@ -14567,12 +14567,12 @@
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>respondert_versjon</t>
+          <t>frist_varsel_ok</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>Hvilken TE-versjon (0-indeksert) denne responsen gjelder. Settes automatisk av backend.</t>
+          <t>Er varsel om fristforlengelse sendt i tide? (§33.4). None hvis ikke relevant.</t>
         </is>
       </c>
     </row>
@@ -14594,7 +14594,7 @@
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>frist_varsel_ok</t>
+          <t>spesifisert_krav_ok</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
@@ -14609,7 +14609,7 @@
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>Er varsel om fristforlengelse sendt i tide? (§33.4). None hvis ikke relevant.</t>
+          <t>Er spesifisert krav sendt i tide? (§33.6)</t>
         </is>
       </c>
     </row>
@@ -14621,7 +14621,7 @@
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>spesifisert_krav_ok</t>
+          <t>foresporsel_svar_ok</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -14636,7 +14636,7 @@
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>Er spesifisert krav sendt i tide? (§33.6)</t>
+          <t>Er svar på forespørsel sendt i tide? (§33.6.2/§5). None hvis ikke relevant.</t>
         </is>
       </c>
     </row>
@@ -14648,12 +14648,12 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>foresporsel_svar_ok</t>
+          <t>begrunnelse_varsel</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -14663,7 +14663,7 @@
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>Er svar på forespørsel sendt i tide? (§33.6.2/§5). None hvis ikke relevant.</t>
+          <t>BHs begrunnelse for vurdering av varsling</t>
         </is>
       </c>
     </row>
@@ -14675,12 +14675,12 @@
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse_varsel</t>
+          <t>vilkar_oppfylt</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -14690,7 +14690,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse for vurdering av varsling</t>
+          <t>Har forholdet medført en faktisk fremdriftshindring? (§33.1)</t>
         </is>
       </c>
     </row>
@@ -14702,12 +14702,12 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>vilkar_oppfylt</t>
+          <t>beregnings_resultat</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -14717,7 +14717,7 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>Har forholdet medført en faktisk fremdriftshindring? (§33.1)</t>
+          <t>BHs vurdering av antall dager (ren beregning)</t>
         </is>
       </c>
     </row>
@@ -14729,12 +14729,12 @@
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>beregnings_resultat</t>
+          <t>godkjent_dager</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -14744,7 +14744,7 @@
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>BHs vurdering av antall dager (ren beregning)</t>
+          <t>Godkjent antall dager. Innvilges kun hvis Grunnlag også godkjennes.</t>
         </is>
       </c>
     </row>
@@ -14756,12 +14756,12 @@
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>godkjent_dager</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -14771,7 +14771,7 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>Godkjent antall dager. Innvilges kun hvis Grunnlag også godkjennes.</t>
+          <t>BH-godkjent ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -14783,7 +14783,7 @@
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>BH-godkjent ny sluttdato (YYYY-MM-DD)</t>
+          <t>Samlet begrunnelse</t>
         </is>
       </c>
     </row>
@@ -14810,12 +14810,12 @@
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>subsidiaer_triggers</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av SubsidiaerTrigger</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>Samlet begrunnelse</t>
+          <t>Liste over årsaker til subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14837,12 +14837,12 @@
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>frist_for_spesifisering</t>
+          <t>subsidiaer_resultat</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>FristBeregningResultat</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -14852,7 +14852,7 @@
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>Frist for TE å levere ytterligere spesifikasjon/fremdriftsplan (YYYY-MM-DD)</t>
+          <t>Subsidiært beregningsresultat</t>
         </is>
       </c>
     </row>
@@ -14864,12 +14864,12 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_triggers</t>
+          <t>subsidiaer_godkjent_dager</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>liste av SubsidiaerTrigger</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -14879,7 +14879,7 @@
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>Liste over årsaker til subsidiær vurdering</t>
+          <t>Subsidiært godkjent antall dager</t>
         </is>
       </c>
     </row>
@@ -14891,12 +14891,12 @@
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_resultat</t>
+          <t>subsidiaer_begrunnelse</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>FristBeregningResultat</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært beregningsresultat</t>
+          <t>BH's begrunnelse for subsidiær vurdering</t>
         </is>
       </c>
     </row>
@@ -14918,34 +14918,34 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_godkjent_dager</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært godkjent antall dager</t>
+          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_oppdatert</t>
+          <t>te_aksepterer_respons</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_begrunnelse</t>
+          <t>kommentar</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
@@ -14960,14 +14960,14 @@
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>BH's begrunnelse for subsidiær vurdering</t>
+          <t>Valgfri kommentar fra entreprenør</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_oppdatert</t>
+          <t>te_aksepterer_respons</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -14994,12 +14994,12 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>te_aksepterer_respons</t>
+          <t>forsering_varsel</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>kommentar</t>
+          <t>frist_krav_id</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
@@ -15009,29 +15009,29 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>Valgfri kommentar fra entreprenør</t>
+          <t>Event-ID til fristkravet som ble avslått</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>te_aksepterer_respons</t>
+          <t>forsering_varsel</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>respons_frist_id</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -15041,7 +15041,7 @@
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>Står på toppnivå i modellen og legges i `data` ved lagring.</t>
+          <t>Event-ID til BH's frist-respons som utløste forseringen</t>
         </is>
       </c>
     </row>
@@ -15053,12 +15053,12 @@
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>frist_krav_id</t>
+          <t>estimert_kostnad</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>Event-ID til fristkravet som ble avslått</t>
+          <t>Estimert kostnad for forsering i NOK</t>
         </is>
       </c>
     </row>
@@ -15080,7 +15080,7 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>respons_frist_id</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
@@ -15095,7 +15095,7 @@
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>Event-ID til BH's frist-respons som utløste forseringen</t>
+          <t>Begrunnelse for forsering</t>
         </is>
       </c>
     </row>
@@ -15107,22 +15107,22 @@
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>estimert_kostnad</t>
+          <t>bekreft_30_prosent</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t>Estimert kostnad for forsering i NOK</t>
+          <t>TE bekrefter at estimert kostnad er innenfor dagmulkt + 30%</t>
         </is>
       </c>
     </row>
@@ -15134,7 +15134,7 @@
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>dato_iverksettelse</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
@@ -15149,7 +15149,7 @@
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for forsering</t>
+          <t>Dato forsering iverksettes (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -15161,22 +15161,22 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>bekreft_30_prosent</t>
+          <t>avslatte_dager</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
         <is>
-          <t>TE bekrefter at estimert kostnad er innenfor dagmulkt + 30%</t>
+          <t>Antall dager som ble avslått av BH</t>
         </is>
       </c>
     </row>
@@ -15188,12 +15188,12 @@
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>dato_iverksettelse</t>
+          <t>dagmulktsats</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="E234" s="2" t="inlineStr">
         <is>
-          <t>Dato forsering iverksettes (YYYY-MM-DD)</t>
+          <t>Dagmulktsats i NOK per dag (påkrevd for 30%-beregning)</t>
         </is>
       </c>
     </row>
@@ -15215,66 +15215,66 @@
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>avslatte_dager</t>
+          <t>grunnlag_avslag_trigger</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
         <is>
-          <t>Antall dager som ble avslått av BH</t>
+          <t>True hvis forsering utløses av grunnlagsavslag (ikke direkte frist-avslag)</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>forsering_varsel</t>
+          <t>forsering_respons</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>dagmulktsats</t>
+          <t>vurdering_per_sak</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>liste av objekt</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
         <is>
-          <t>Dagmulktsats i NOK per dag (påkrevd for 30%-beregning)</t>
+          <t>BHs vurdering av forseringsrett per sak</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>forsering_varsel</t>
+          <t>forsering_respons</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>grunnlag_avslag_trigger</t>
+          <t>dager_med_forseringsrett</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       </c>
       <c r="E237" s="2" t="inlineStr">
         <is>
-          <t>True hvis forsering utløses av grunnlagsavslag (ikke direkte frist-avslag)</t>
+          <t>Antall dager BH mener TE har forseringsrett for</t>
         </is>
       </c>
     </row>
@@ -15296,12 +15296,12 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>vurdering_per_sak</t>
+          <t>grunnlag_fortsatt_gyldig</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>liste av objekt</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -15311,7 +15311,7 @@
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>BHs vurdering av forseringsrett per sak</t>
+          <t>BH bekrefter at frist-avslaget fortsatt står ved lag</t>
         </is>
       </c>
     </row>
@@ -15323,12 +15323,12 @@
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>dager_med_forseringsrett</t>
+          <t>grunnlag_begrunnelse</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="E239" s="2" t="inlineStr">
         <is>
-          <t>Antall dager BH mener TE har forseringsrett for</t>
+          <t>BHs begrunnelse hvis grunnlaget bestrides</t>
         </is>
       </c>
     </row>
@@ -15350,7 +15350,7 @@
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>grunnlag_fortsatt_gyldig</t>
+          <t>trettiprosent_overholdt</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
@@ -15365,7 +15365,7 @@
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>BH bekrefter at frist-avslaget fortsatt står ved lag</t>
+          <t>BH vurderer om estimert kostnad er innenfor 30%-grensen</t>
         </is>
       </c>
     </row>
@@ -15377,7 +15377,7 @@
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>grunnlag_begrunnelse</t>
+          <t>trettiprosent_begrunnelse</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
@@ -15392,7 +15392,7 @@
       </c>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse hvis grunnlaget bestrides</t>
+          <t>BHs begrunnelse ved avvik fra 30%-regelen</t>
         </is>
       </c>
     </row>
@@ -15404,7 +15404,7 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>trettiprosent_overholdt</t>
+          <t>aksepterer</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
@@ -15414,12 +15414,12 @@
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>BH vurderer om estimert kostnad er innenfor 30%-grensen</t>
+          <t>BH aksepterer forsering</t>
         </is>
       </c>
     </row>
@@ -15431,12 +15431,12 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>trettiprosent_begrunnelse</t>
+          <t>godkjent_kostnad</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -15446,7 +15446,7 @@
       </c>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>BHs begrunnelse ved avvik fra 30%-regelen</t>
+          <t>BH's godkjente forseringskostnad (kan være lavere enn estimert)</t>
         </is>
       </c>
     </row>
@@ -15458,12 +15458,12 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>aksepterer</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -15473,7 +15473,7 @@
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>BH aksepterer forsering</t>
+          <t>BH's begrunnelse for aksept/avslag</t>
         </is>
       </c>
     </row>
@@ -15485,12 +15485,12 @@
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>godkjent_kostnad</t>
+          <t>rigg_varslet_i_tide</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -15500,7 +15500,7 @@
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>BH's godkjente forseringskostnad (kan være lavere enn estimert)</t>
+          <t>Om rigg/drift-varslet var rettidig</t>
         </is>
       </c>
     </row>
@@ -15512,22 +15512,22 @@
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>produktivitet_varslet_i_tide</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>BH's begrunnelse for aksept/avslag</t>
+          <t>Om produktivitets-varslet var rettidig</t>
         </is>
       </c>
     </row>
@@ -15539,12 +15539,12 @@
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>rigg_varslet_i_tide</t>
+          <t>godkjent_rigg_drift</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -15554,7 +15554,7 @@
       </c>
       <c r="E247" s="2" t="inlineStr">
         <is>
-          <t>Om rigg/drift-varslet var rettidig</t>
+          <t>Godkjent rigg/drift-beløp</t>
         </is>
       </c>
     </row>
@@ -15566,12 +15566,12 @@
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>produktivitet_varslet_i_tide</t>
+          <t>godkjent_produktivitet</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -15581,7 +15581,7 @@
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>Om produktivitets-varslet var rettidig</t>
+          <t>Godkjent produktivitetsbeløp</t>
         </is>
       </c>
     </row>
@@ -15593,12 +15593,12 @@
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>godkjent_rigg_drift</t>
+          <t>subsidiaer_triggers</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -15608,7 +15608,7 @@
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>Godkjent rigg/drift-beløp</t>
+          <t>Triggere for subsidiær vurdering (f.eks. 'grunnlag_bestridt')</t>
         </is>
       </c>
     </row>
@@ -15620,7 +15620,7 @@
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>godkjent_produktivitet</t>
+          <t>subsidiaer_godkjent_belop</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
@@ -15635,7 +15635,7 @@
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>Godkjent produktivitetsbeløp</t>
+          <t>Subsidiært godkjent beløp</t>
         </is>
       </c>
     </row>
@@ -15647,12 +15647,12 @@
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_triggers</t>
+          <t>subsidiaer_begrunnelse</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -15662,51 +15662,51 @@
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>Triggere for subsidiær vurdering (f.eks. 'grunnlag_bestridt')</t>
+          <t>Begrunnelse for subsidiært standpunkt</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>forsering_respons</t>
+          <t>forsering_stoppet</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_godkjent_belop</t>
+          <t>dato_stoppet</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>Subsidiært godkjent beløp</t>
+          <t>Dato forsering ble stoppet (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>forsering_respons</t>
+          <t>forsering_stoppet</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>subsidiaer_begrunnelse</t>
+          <t>paalopte_kostnader</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -15716,7 +15716,7 @@
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for subsidiært standpunkt</t>
+          <t>Påløpte kostnader ved stopp i NOK</t>
         </is>
       </c>
     </row>
@@ -15728,7 +15728,7 @@
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>dato_stoppet</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
@@ -15738,19 +15738,19 @@
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
         <is>
-          <t>Dato forsering ble stoppet (YYYY-MM-DD)</t>
+          <t>Begrunnelse for stopp</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>forsering_stoppet</t>
+          <t>forsering_kostnader_oppdatert</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -15765,24 +15765,24 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
         <is>
-          <t>Påløpte kostnader ved stopp i NOK</t>
+          <t>Påløpte kostnader i NOK</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>forsering_stoppet</t>
+          <t>forsering_kostnader_oppdatert</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>kommentar</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
@@ -15797,24 +15797,24 @@
       </c>
       <c r="E256" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for stopp</t>
+          <t>Kommentar til kostnadsoppdatering</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>forsering_kostnader_oppdatert</t>
+          <t>forsering_koe_lagt_til</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>paalopte_kostnader</t>
+          <t>koe_sak_id</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -15824,19 +15824,19 @@
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t>Påløpte kostnader i NOK</t>
+          <t>SAK-ID til KOE som legges til/fjernes</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>forsering_kostnader_oppdatert</t>
+          <t>forsering_koe_lagt_til</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>kommentar</t>
+          <t>koe_tittel</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
@@ -15851,14 +15851,14 @@
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>Kommentar til kostnadsoppdatering</t>
+          <t>Tittel på KOE for visning</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_lagt_til</t>
+          <t>forsering_koe_fjernet</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -15885,7 +15885,7 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_lagt_til</t>
+          <t>forsering_koe_fjernet</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -15912,12 +15912,12 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_fjernet</t>
+          <t>sak_opprettet</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>koe_sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
@@ -15927,24 +15927,24 @@
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til KOE som legges til/fjernes</t>
+          <t>Prosjekt-ID</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>forsering_koe_fjernet</t>
+          <t>sak_opprettet</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>koe_tittel</t>
+          <t>sakstittel</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
@@ -15954,12 +15954,12 @@
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>Tittel på KOE for visning</t>
+          <t>Sakstittel</t>
         </is>
       </c>
     </row>
@@ -15971,7 +15971,7 @@
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>catenda_topic_id</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
@@ -15986,7 +15986,7 @@
       </c>
       <c r="E263" s="2" t="inlineStr">
         <is>
-          <t>Prosjekt-ID</t>
+          <t>Catenda topic GUID</t>
         </is>
       </c>
     </row>
@@ -15998,7 +15998,7 @@
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>sakstittel</t>
+          <t>sakstype</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
@@ -16008,12 +16008,12 @@
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t>Sakstittel</t>
+          <t>Sakstype: 'standard' (KOE), 'endringsordre' (EO), eller 'forsering'</t>
         </is>
       </c>
     </row>
@@ -16025,7 +16025,7 @@
       </c>
       <c r="B265" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_id</t>
+          <t>prosjekt_navn</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
@@ -16040,7 +16040,7 @@
       </c>
       <c r="E265" s="2" t="inlineStr">
         <is>
-          <t>Catenda topic GUID</t>
+          <t>Prosjektnavn fra Catenda</t>
         </is>
       </c>
     </row>
@@ -16052,7 +16052,7 @@
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>sakstype</t>
+          <t>byggherre</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="E266" s="2" t="inlineStr">
         <is>
-          <t>Sakstype: 'standard' (KOE), 'endringsordre' (EO), eller 'forsering'</t>
+          <t>Byggherre (BH) - fra topic custom field</t>
         </is>
       </c>
     </row>
@@ -16079,7 +16079,7 @@
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_navn</t>
+          <t>leverandor</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
@@ -16094,7 +16094,7 @@
       </c>
       <c r="E267" s="2" t="inlineStr">
         <is>
-          <t>Prosjektnavn fra Catenda</t>
+          <t>Leverandør/Entreprenør (TE) - fra topic custom field</t>
         </is>
       </c>
     </row>
@@ -16106,12 +16106,12 @@
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>byggherre</t>
+          <t>forsering_data</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>objekt</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -16121,19 +16121,19 @@
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>Byggherre (BH) - fra topic custom field</t>
+          <t>Forsering-data inkl. avslatte_fristkrav, dato_varslet, estimert_kostnad (kun for forsering-saker)</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>sak_opprettet</t>
+          <t>internt_notat</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>leverandor</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
@@ -16143,29 +16143,29 @@
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E269" s="2" t="inlineStr">
         <is>
-          <t>Leverandør/Entreprenør (TE) - fra topic custom field</t>
+          <t>Notat-tekst</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>sak_opprettet</t>
+          <t>internt_notat</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>forsering_data</t>
+          <t>spor</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>objekt</t>
+          <t>SporType</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -16175,26 +16175,26 @@
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>Forsering-data inkl. avslatte_fristkrav, dato_varslet, estimert_kostnad (kun for forsering-saker)</t>
+          <t>Hvilket spor notatet gjelder</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>internt_notat</t>
+          <t>eo_opprettet</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
+          <t>eo_nummer</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="C271" s="2" t="inlineStr">
-        <is>
-          <t>tekst</t>
-        </is>
-      </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
           <t>ja</t>
@@ -16202,34 +16202,34 @@
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>Notat-tekst</t>
+          <t>Endringsordre-nummer</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>internt_notat</t>
+          <t>eo_opprettet</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>spor</t>
+          <t>beskrivelse</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>SporType</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
         <is>
-          <t>Hvilket spor notatet gjelder</t>
+          <t>Beskrivelse av endringen</t>
         </is>
       </c>
     </row>
@@ -16241,22 +16241,22 @@
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>eo_nummer</t>
+          <t>relaterte_koe_saker</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>Endringsordre-nummer</t>
+          <t>SAK-IDs til KOE-er som inngår</t>
         </is>
       </c>
     </row>
@@ -16268,7 +16268,7 @@
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>beskrivelse</t>
+          <t>sakstittel</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
@@ -16278,12 +16278,12 @@
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringen</t>
+          <t>Sakstittel for EO-saken</t>
         </is>
       </c>
     </row>
@@ -16295,12 +16295,12 @@
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>relaterte_koe_saker</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -16310,7 +16310,7 @@
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
-          <t>SAK-IDs til KOE-er som inngår</t>
+          <t>Prosjekt-ID</t>
         </is>
       </c>
     </row>
@@ -16322,7 +16322,7 @@
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>sakstittel</t>
+          <t>catenda_topic_id</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
@@ -16337,19 +16337,19 @@
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
-          <t>Sakstittel for EO-saken</t>
+          <t>Catenda topic GUID</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>eo_opprettet</t>
+          <t>eo_koe_lagt_til</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>koe_sak_id</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
@@ -16359,24 +16359,24 @@
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
         <is>
-          <t>Prosjekt-ID</t>
+          <t>SAK-ID til KOE som legges til/fjernes</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>eo_opprettet</t>
+          <t>eo_koe_lagt_til</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_id</t>
+          <t>koe_tittel</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
@@ -16391,14 +16391,14 @@
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>Catenda topic GUID</t>
+          <t>Tittel på KOE for visning</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_lagt_til</t>
+          <t>eo_koe_fjernet</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
@@ -16425,7 +16425,7 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_lagt_til</t>
+          <t>eo_koe_fjernet</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -16452,12 +16452,12 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_fjernet</t>
+          <t>eo_utstedt</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>koe_sak_id</t>
+          <t>eo_nummer</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
@@ -16472,24 +16472,24 @@
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til KOE som legges til/fjernes</t>
+          <t>Endringsordre-nummer</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>eo_koe_fjernet</t>
+          <t>eo_utstedt</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>koe_tittel</t>
+          <t>revisjon_nummer</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -16499,7 +16499,7 @@
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>Tittel på KOE for visning</t>
+          <t>Revisjonsnummer</t>
         </is>
       </c>
     </row>
@@ -16511,7 +16511,7 @@
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>eo_nummer</t>
+          <t>beskrivelse</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
@@ -16526,7 +16526,7 @@
       </c>
       <c r="E283" s="2" t="inlineStr">
         <is>
-          <t>Endringsordre-nummer</t>
+          <t>Beskrivelse av endringen</t>
         </is>
       </c>
     </row>
@@ -16538,12 +16538,12 @@
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>revisjon_nummer</t>
+          <t>vedlegg_ids</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -16553,7 +16553,7 @@
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
-          <t>Revisjonsnummer</t>
+          <t>Vedlegg-IDer</t>
         </is>
       </c>
     </row>
@@ -16565,22 +16565,22 @@
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>beskrivelse</t>
+          <t>konsekvenser</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>EOKonsekvenser</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E285" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringen</t>
+          <t>Konsekvenser av endringen</t>
         </is>
       </c>
     </row>
@@ -16592,12 +16592,12 @@
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_ids</t>
+          <t>konsekvens_beskrivelse</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>Vedlegg-IDer</t>
+          <t>Beskrivelse av konsekvensene</t>
         </is>
       </c>
     </row>
@@ -16619,12 +16619,12 @@
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>konsekvenser</t>
+          <t>vederlag</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>EOKonsekvenser</t>
+          <t>VederlagKompensasjon</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -16634,7 +16634,7 @@
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>Konsekvenser av endringen</t>
+          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
         </is>
       </c>
     </row>
@@ -16646,7 +16646,7 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>konsekvens_beskrivelse</t>
+          <t>oppgjorsform</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
@@ -16661,7 +16661,7 @@
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av konsekvensene</t>
+          <t>DEPRECATED: Bruk vederlag.metode</t>
         </is>
       </c>
     </row>
@@ -16673,12 +16673,12 @@
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>vederlag</t>
+          <t>kompensasjon_belop</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>VederlagKompensasjon</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
+          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
         </is>
       </c>
     </row>
@@ -16700,12 +16700,12 @@
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>oppgjorsform</t>
+          <t>fradrag_belop</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -16715,7 +16715,7 @@
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.metode</t>
+          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
         </is>
       </c>
     </row>
@@ -16727,12 +16727,12 @@
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>kompensasjon_belop</t>
+          <t>er_estimat</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
+          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
         </is>
       </c>
     </row>
@@ -16754,12 +16754,12 @@
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>fradrag_belop</t>
+          <t>frist_dager</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -16769,7 +16769,7 @@
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
+          <t>Fristforlengelse i dager</t>
         </is>
       </c>
     </row>
@@ -16781,12 +16781,12 @@
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>er_estimat</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -16796,7 +16796,7 @@
       </c>
       <c r="E293" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
+          <t>Ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -16808,12 +16808,12 @@
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>frist_dager</t>
+          <t>relaterte_koe_saker</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -16823,7 +16823,7 @@
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>Fristforlengelse i dager</t>
+          <t>SAK-IDs til KOE-er som inngår</t>
         </is>
       </c>
     </row>
@@ -16835,12 +16835,12 @@
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>relaterte_sak_ids</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -16850,7 +16850,7 @@
       </c>
       <c r="E295" s="2" t="inlineStr">
         <is>
-          <t>Ny sluttdato (YYYY-MM-DD)</t>
+          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
         </is>
       </c>
     </row>
@@ -16862,22 +16862,22 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>relaterte_koe_saker</t>
+          <t>netto_belop</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>SAK-IDs til KOE-er som inngår</t>
+          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
         </is>
       </c>
     </row>
@@ -16889,22 +16889,22 @@
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>relaterte_sak_ids</t>
+          <t>har_priskonsekvens</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
-          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
+          <t>Sjekker om EO har priskonsekvens</t>
         </is>
       </c>
     </row>
@@ -16916,12 +16916,12 @@
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>netto_belop</t>
+          <t>har_fristkonsekvens</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -16931,19 +16931,19 @@
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
+          <t>Sjekker om EO har fristkonsekvens</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>eo_utstedt</t>
+          <t>eo_akseptert</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>har_priskonsekvens</t>
+          <t>akseptert</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
@@ -16953,78 +16953,78 @@
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har priskonsekvens</t>
+          <t>Om TE aksepterer</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>eo_utstedt</t>
+          <t>eo_akseptert</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>har_fristkonsekvens</t>
+          <t>kommentar</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har fristkonsekvens</t>
+          <t>TEs kommentar</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>eo_akseptert</t>
+          <t>eo_bestridt</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>akseptert</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
-          <t>Om TE aksepterer</t>
+          <t>Begrunnelse for bestridelse</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>eo_akseptert</t>
+          <t>eo_bestridt</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>kommentar</t>
+          <t>nytt_koe_sak_id</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
@@ -17039,24 +17039,24 @@
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>TEs kommentar</t>
+          <t>SAK-ID til nytt KOE som fremmes som alternativ</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>eo_bestridt</t>
+          <t>eo_revidert</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>ny_revisjon_nummer</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
@@ -17066,19 +17066,19 @@
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>Begrunnelse for bestridelse</t>
+          <t>Nytt revisjonsnummer</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>eo_bestridt</t>
+          <t>eo_revidert</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>nytt_koe_sak_id</t>
+          <t>endringer_beskrivelse</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
@@ -17088,12 +17088,12 @@
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>SAK-ID til nytt KOE som fremmes som alternativ</t>
+          <t>Beskrivelse av endringene</t>
         </is>
       </c>
     </row>
@@ -17105,66 +17105,66 @@
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>ny_revisjon_nummer</t>
+          <t>oppdatert_data</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>EOUtstedtData</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>Nytt revisjonsnummer</t>
+          <t>Oppdatert EO-data (hvis endret)</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>eo_revidert</t>
+          <t>Delmodell EOKonsekvenser</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>endringer_beskrivelse</t>
+          <t>sha</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringene</t>
+          <t>SHA-konsekvenser</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>eo_revidert</t>
+          <t>Delmodell EOKonsekvenser</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>oppdatert_data</t>
+          <t>kvalitet</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>EOUtstedtData</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -17174,7 +17174,7 @@
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
-          <t>Oppdatert EO-data (hvis endret)</t>
+          <t>Kvalitetskonsekvenser</t>
         </is>
       </c>
     </row>
@@ -17186,7 +17186,7 @@
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>sha</t>
+          <t>fremdrift</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>SHA-konsekvenser</t>
+          <t>Fremdriftskonsekvenser</t>
         </is>
       </c>
     </row>
@@ -17213,7 +17213,7 @@
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>kvalitet</t>
+          <t>pris</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
@@ -17228,7 +17228,7 @@
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>Kvalitetskonsekvenser</t>
+          <t>Priskonsekvenser</t>
         </is>
       </c>
     </row>
@@ -17240,7 +17240,7 @@
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>fremdrift</t>
+          <t>annet</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
@@ -17255,51 +17255,51 @@
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>Fremdriftskonsekvenser</t>
+          <t>Andre konsekvenser</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOKonsekvenser</t>
+          <t>Delmodell EOUtstedtData</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>pris</t>
+          <t>eo_nummer</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>Priskonsekvenser</t>
+          <t>Endringsordre-nummer</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOKonsekvenser</t>
+          <t>Delmodell EOUtstedtData</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>annet</t>
+          <t>revisjon_nummer</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
@@ -17309,7 +17309,7 @@
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>Andre konsekvenser</t>
+          <t>Revisjonsnummer</t>
         </is>
       </c>
     </row>
@@ -17321,7 +17321,7 @@
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>eo_nummer</t>
+          <t>beskrivelse</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
@@ -17336,7 +17336,7 @@
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>Endringsordre-nummer</t>
+          <t>Beskrivelse av endringen</t>
         </is>
       </c>
     </row>
@@ -17348,12 +17348,12 @@
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>revisjon_nummer</t>
+          <t>vedlegg_ids</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -17363,7 +17363,7 @@
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>Revisjonsnummer</t>
+          <t>Vedlegg-IDer</t>
         </is>
       </c>
     </row>
@@ -17375,22 +17375,22 @@
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>beskrivelse</t>
+          <t>konsekvenser</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>EOKonsekvenser</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av endringen</t>
+          <t>Konsekvenser av endringen</t>
         </is>
       </c>
     </row>
@@ -17402,12 +17402,12 @@
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_ids</t>
+          <t>konsekvens_beskrivelse</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
@@ -17417,7 +17417,7 @@
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
-          <t>Vedlegg-IDer</t>
+          <t>Beskrivelse av konsekvensene</t>
         </is>
       </c>
     </row>
@@ -17429,12 +17429,12 @@
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>konsekvenser</t>
+          <t>vederlag</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>EOKonsekvenser</t>
+          <t>VederlagKompensasjon</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -17444,7 +17444,7 @@
       </c>
       <c r="E317" s="2" t="inlineStr">
         <is>
-          <t>Konsekvenser av endringen</t>
+          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
         </is>
       </c>
     </row>
@@ -17456,7 +17456,7 @@
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>konsekvens_beskrivelse</t>
+          <t>oppgjorsform</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
@@ -17471,7 +17471,7 @@
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>Beskrivelse av konsekvensene</t>
+          <t>DEPRECATED: Bruk vederlag.metode</t>
         </is>
       </c>
     </row>
@@ -17483,12 +17483,12 @@
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>vederlag</t>
+          <t>kompensasjon_belop</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>VederlagKompensasjon</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
@@ -17498,7 +17498,7 @@
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>Vederlagskompensasjon (metode, beløp, fradrag) - konsistent med VederlagData</t>
+          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
         </is>
       </c>
     </row>
@@ -17510,12 +17510,12 @@
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>oppgjorsform</t>
+          <t>fradrag_belop</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
@@ -17525,7 +17525,7 @@
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.metode</t>
+          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
         </is>
       </c>
     </row>
@@ -17537,12 +17537,12 @@
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>kompensasjon_belop</t>
+          <t>er_estimat</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
@@ -17552,7 +17552,7 @@
       </c>
       <c r="E321" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.belop_direkte</t>
+          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
         </is>
       </c>
     </row>
@@ -17564,12 +17564,12 @@
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>fradrag_belop</t>
+          <t>frist_dager</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>heltall</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -17579,7 +17579,7 @@
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.fradrag_belop</t>
+          <t>Fristforlengelse i dager</t>
         </is>
       </c>
     </row>
@@ -17591,12 +17591,12 @@
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>er_estimat</t>
+          <t>ny_sluttdato</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="E323" s="2" t="inlineStr">
         <is>
-          <t>DEPRECATED: Bruk vederlag.er_estimat</t>
+          <t>Ny sluttdato (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -17618,12 +17618,12 @@
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>frist_dager</t>
+          <t>relaterte_koe_saker</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>heltall</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -17633,7 +17633,7 @@
       </c>
       <c r="E324" s="2" t="inlineStr">
         <is>
-          <t>Fristforlengelse i dager</t>
+          <t>SAK-IDs til KOE-er som inngår</t>
         </is>
       </c>
     </row>
@@ -17645,12 +17645,12 @@
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>ny_sluttdato</t>
+          <t>relaterte_sak_ids</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
@@ -17660,7 +17660,7 @@
       </c>
       <c r="E325" s="2" t="inlineStr">
         <is>
-          <t>Ny sluttdato (YYYY-MM-DD)</t>
+          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
         </is>
       </c>
     </row>
@@ -17672,22 +17672,22 @@
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>relaterte_koe_saker</t>
+          <t>netto_belop</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
         <is>
-          <t>SAK-IDs til KOE-er som inngår</t>
+          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
         </is>
       </c>
     </row>
@@ -17699,22 +17699,22 @@
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>relaterte_sak_ids</t>
+          <t>har_priskonsekvens</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
         <is>
-          <t>Alias for relaterte_koe_saker (for bakoverkompatibilitet)</t>
+          <t>Sjekker om EO har priskonsekvens</t>
         </is>
       </c>
     </row>
@@ -17726,12 +17726,12 @@
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>netto_belop</t>
+          <t>har_fristkonsekvens</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
@@ -17741,61 +17741,61 @@
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>Beregner netto beløp. Prioriterer vederlag-feltet, faller tilbake til legacy-felter.</t>
+          <t>Sjekker om EO har fristkonsekvens</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOUtstedtData</t>
+          <t>Delmodell KonsekvensVarsler</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>har_priskonsekvens</t>
+          <t>vederlag</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har priskonsekvens</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>Delmodell EOUtstedtData</t>
+          <t>Delmodell KonsekvensVarsler</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>har_fristkonsekvens</t>
+          <t>rigg_drift</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>beregnet</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>Sjekker om EO har fristkonsekvens</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -17807,7 +17807,7 @@
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>vederlag</t>
+          <t>produktivitet</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
@@ -17834,7 +17834,7 @@
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>rigg_drift</t>
+          <t>frist</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
@@ -17856,12 +17856,12 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>Delmodell KonsekvensVarsler</t>
+          <t>Delmodell LetterParty</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>produktivitet</t>
+          <t>navn</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
@@ -17871,7 +17871,7 @@
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -17883,12 +17883,12 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>Delmodell KonsekvensVarsler</t>
+          <t>Delmodell LetterParty</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>frist</t>
+          <t>rolle</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
@@ -17898,7 +17898,7 @@
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -17915,7 +17915,7 @@
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>navn</t>
+          <t>adresse</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
@@ -17925,7 +17925,7 @@
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -17942,7 +17942,7 @@
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>rolle</t>
+          <t>orgnr</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -17964,12 +17964,12 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterParty</t>
+          <t>Delmodell LetterReferences</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>adresse</t>
+          <t>sakId</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -17991,12 +17991,12 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterParty</t>
+          <t>Delmodell LetterReferences</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>orgnr</t>
+          <t>sakstittel</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
@@ -18006,7 +18006,7 @@
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
@@ -18023,7 +18023,7 @@
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>sakId</t>
+          <t>eventId</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
@@ -18050,7 +18050,7 @@
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>sakstittel</t>
+          <t>sporType</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
@@ -18077,7 +18077,7 @@
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>eventId</t>
+          <t>dato</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
@@ -18104,7 +18104,7 @@
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>sporType</t>
+          <t>kravDato</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
@@ -18126,12 +18126,12 @@
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterReferences</t>
+          <t>Delmodell LetterSection</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>dato</t>
+          <t>tittel</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
@@ -18153,12 +18153,12 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterReferences</t>
+          <t>Delmodell LetterSection</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>kravDato</t>
+          <t>originalTekst</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
@@ -18168,7 +18168,7 @@
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -18185,7 +18185,7 @@
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>tittel</t>
+          <t>redigertTekst</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
@@ -18207,17 +18207,17 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSection</t>
+          <t>Delmodell LetterSections</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>originalTekst</t>
+          <t>innledning</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterSection</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
@@ -18234,17 +18234,17 @@
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSection</t>
+          <t>Delmodell LetterSections</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>redigertTekst</t>
+          <t>begrunnelse</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterSection</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -18266,7 +18266,7 @@
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>innledning</t>
+          <t>avslutning</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
@@ -18288,17 +18288,17 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSections</t>
+          <t>Delmodell LetterSnapshot</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>begrunnelse</t>
+          <t>tittel</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>LetterSection</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
@@ -18315,17 +18315,17 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSections</t>
+          <t>Delmodell LetterSnapshot</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>avslutning</t>
+          <t>mottaker</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>LetterSection</t>
+          <t>LetterParty</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -18347,12 +18347,12 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>tittel</t>
+          <t>avsender</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>LetterParty</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -18374,12 +18374,12 @@
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>mottaker</t>
+          <t>referanser</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>LetterParty</t>
+          <t>LetterReferences</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
@@ -18401,12 +18401,12 @@
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>avsender</t>
+          <t>seksjoner</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>LetterParty</t>
+          <t>LetterSections</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
@@ -18423,71 +18423,71 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSnapshot</t>
+          <t>Delmodell SaerskiltKrav</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>referanser</t>
+          <t>rigg_drift</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>LetterReferences</t>
+          <t>SaerskiltKravItem</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rigg/drift krav (§34.1.3 første ledd)</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>Delmodell LetterSnapshot</t>
+          <t>Delmodell SaerskiltKrav</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>seksjoner</t>
+          <t>produktivitet</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>LetterSections</t>
+          <t>SaerskiltKravItem</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Produktivitetstap krav (§34.1.3 annet ledd)</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKrav</t>
+          <t>Delmodell SaerskiltKravItem</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>rigg_drift</t>
+          <t>belop</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>SaerskiltKravItem</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
@@ -18497,24 +18497,24 @@
       </c>
       <c r="E356" s="2" t="inlineStr">
         <is>
-          <t>Rigg/drift krav (§34.1.3 første ledd)</t>
+          <t>Beløp for dette særskilte kravet</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKrav</t>
+          <t>Delmodell SaerskiltKravItem</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>produktivitet</t>
+          <t>dato_klar_over</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>SaerskiltKravItem</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
@@ -18524,24 +18524,24 @@
       </c>
       <c r="E357" s="2" t="inlineStr">
         <is>
-          <t>Produktivitetstap krav (§34.1.3 annet ledd)</t>
+          <t>Når TE ble klar over at utgifter ville påløpe (YYYY-MM-DD). Brukes til 7-dagers varslingssjekk.</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKravItem</t>
+          <t>Delmodell VarselInfo</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>belop</t>
+          <t>dato_sendt</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>tekst</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
@@ -18551,24 +18551,24 @@
       </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
-          <t>Beløp for dette særskilte kravet</t>
+          <t>Når varselet faktisk ble sendt til BH (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>Delmodell SaerskiltKravItem</t>
+          <t>Delmodell VarselInfo</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>dato_klar_over</t>
+          <t>metode</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>liste av tekst</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
@@ -18578,51 +18578,51 @@
       </c>
       <c r="E359" s="2" t="inlineStr">
         <is>
-          <t>Når TE ble klar over at utgifter ville påløpe (YYYY-MM-DD). Brukes til 7-dagers varslingssjekk.</t>
+          <t>Metoder brukt for å varsle (f.eks. ['epost', 'byggemote', 'telefon'])</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>Delmodell VarselInfo</t>
+          <t>Delmodell VederlagKompensasjon</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>dato_sendt</t>
+          <t>metode</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>tekst</t>
+          <t>VederlagsMetode</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
         <is>
-          <t>Når varselet faktisk ble sendt til BH (YYYY-MM-DD)</t>
+          <t>Vederlagsmetode etter NS 8407 (§34)</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>Delmodell VarselInfo</t>
+          <t>Delmodell VederlagKompensasjon</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>metode</t>
+          <t>belop_direkte</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>liste av tekst</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
@@ -18632,7 +18632,7 @@
       </c>
       <c r="E361" s="2" t="inlineStr">
         <is>
-          <t>Metoder brukt for å varsle (f.eks. ['epost', 'byggemote', 'telefon'])</t>
+          <t>For ENHETSPRISER/FASTPRIS_TILBUD: Beløp i NOK</t>
         </is>
       </c>
     </row>
@@ -18644,22 +18644,22 @@
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>metode</t>
+          <t>kostnads_overslag</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>VederlagsMetode</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nei</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
         <is>
-          <t>Vederlagsmetode etter NS 8407 (§34)</t>
+          <t>For REGNINGSARBEID (§30.2): Kostnadsoverslag i NOK</t>
         </is>
       </c>
     </row>
@@ -18671,7 +18671,7 @@
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>belop_direkte</t>
+          <t>fradrag_belop</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
@@ -18686,7 +18686,7 @@
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>For ENHETSPRISER/FASTPRIS_TILBUD: Beløp i NOK</t>
+          <t>Fradrag i NOK (§34.4) - reduksjon for besparelser</t>
         </is>
       </c>
     </row>
@@ -18698,12 +18698,12 @@
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>kostnads_overslag</t>
+          <t>er_estimat</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>ja/nei</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -18713,7 +18713,7 @@
       </c>
       <c r="E364" s="2" t="inlineStr">
         <is>
-          <t>For REGNINGSARBEID (§30.2): Kostnadsoverslag i NOK</t>
+          <t>Om beløpet er et estimat (endelig oppgjør senere)</t>
         </is>
       </c>
     </row>
@@ -18725,7 +18725,7 @@
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>fradrag_belop</t>
+          <t>netto_belop</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
@@ -18735,12 +18735,12 @@
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
         <is>
-          <t>Fradrag i NOK (§34.4) - reduksjon for besparelser</t>
+          <t>Beregner netto beløp basert på metode. For ENHETSPRISER/FASTPRIS_TILBUD: belop_direkte - fradrag For REGNINGSARBEID: kostnads_overslag - fradrag</t>
         </is>
       </c>
     </row>
@@ -18752,74 +18752,20 @@
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>er_estimat</t>
+          <t>krevd_belop</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>ja/nei</t>
+          <t>tall</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>nei</t>
+          <t>beregnet</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
-        <is>
-          <t>Om beløpet er et estimat (endelig oppgjør senere)</t>
-        </is>
-      </c>
-    </row>
-    <row r="367">
-      <c r="A367" s="2" t="inlineStr">
-        <is>
-          <t>Delmodell VederlagKompensasjon</t>
-        </is>
-      </c>
-      <c r="B367" s="2" t="inlineStr">
-        <is>
-          <t>netto_belop</t>
-        </is>
-      </c>
-      <c r="C367" s="2" t="inlineStr">
-        <is>
-          <t>tall</t>
-        </is>
-      </c>
-      <c r="D367" s="2" t="inlineStr">
-        <is>
-          <t>beregnet</t>
-        </is>
-      </c>
-      <c r="E367" s="2" t="inlineStr">
-        <is>
-          <t>Beregner netto beløp basert på metode. For ENHETSPRISER/FASTPRIS_TILBUD: belop_direkte - fradrag For REGNINGSARBEID: kostnads_overslag - fradrag</t>
-        </is>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" s="2" t="inlineStr">
-        <is>
-          <t>Delmodell VederlagKompensasjon</t>
-        </is>
-      </c>
-      <c r="B368" s="2" t="inlineStr">
-        <is>
-          <t>krevd_belop</t>
-        </is>
-      </c>
-      <c r="C368" s="2" t="inlineStr">
-        <is>
-          <t>tall</t>
-        </is>
-      </c>
-      <c r="D368" s="2" t="inlineStr">
-        <is>
-          <t>beregnet</t>
-        </is>
-      </c>
-      <c r="E368" s="2" t="inlineStr">
         <is>
           <t>Alias for netto_belop - brukes i state-modellen. Returnerer det totale kravet/kompensasjonen.</t>
         </is>

</xml_diff>

<commit_message>
la aksepten vise til svaret TE godtar, og skriv kontrakten for flyten i språkprøven (#272)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HVhrnKD3RArSvZT8ckB5kh
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -14042,7 +14042,7 @@
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>Er spesifisert krav sendt i tide? (§33.6)</t>
+          <t>Er spesifisert krav sendt i tide? (§33.6). None hvis ikke vurdert (KA-U4).</t>
         </is>
       </c>
     </row>
@@ -14609,7 +14609,7 @@
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>Er spesifisert krav sendt i tide? (§33.6)</t>
+          <t>Er spesifisert krav sendt i tide? (§33.6). None hvis ikke vurdert (KA-U4).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
skill formatet kjernen leser fra formatet den skriver, legg bufferen i sak_metadata og prøv kompatibiliteten mellom TS-versjoner
Del av #316.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vBJt7WvjX53fzyU1er2Co
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: én rad per sak, med prosjekt, sakstype, hvem som opprettet den, og koblingen til topic, board og prosjekt i Catenda. I tillegg ti `cached_*`-kolonner og `last_event_at` med tall regnet ut av hendelsene, til lister og rapportering. Tabellen blander register og projeksjon; skillet er planlagt (MS-06, MS-07).</t>
+          <t>Saksregisteret: én rad per sak, med prosjekt, sakstype, hvem som opprettet den, og koblingen til topic, board og prosjekt i Catenda. I tillegg ti `cached_*`-kolonner og `last_event_at` med tall regnet ut av hendelsene, til lister og rapportering. Fem `kjerne_*`-kolonner er bufferen TS-kjernen regner ut av journalen: visningen og de fire versjonene den er regnet med (B-10, #316). Tabellen blander register og projeksjon; skillet er planlagt (MS-06, MS-07).</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Opprettes når en sak lages, gjennom `SakCreationService`: fra hendelsesrutene, for endringsordrer, og fra en ny topic i Catenda via webhook. Hvordan en forseringssak får sin rad, er ikke kontrollert. `cached_*` oppdateres etter lagrede hendelser (hendelsesrutene, forsering og godkjenning).</t>
+          <t>Opprettes når en sak lages, gjennom `SakCreationService`: fra hendelsesrutene, for endringsordrer, og fra en ny topic i Catenda via webhook. Hvordan en forseringssak får sin rad, er ikke kontrollert. `cached_*` oppdateres etter lagrede hendelser (hendelsesrutene, forsering og godkjenning). `kjerne_*` skrives bare av bufferen i TS-kjernen (`kjerne/buffer.ts`, lageret i `sprakprove/kjernelagring/bane.ts` til skrivestien i #310).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
bygg skiva: TS-serveren i server/, leveringsoppdraget og ruta for kjernen (#347)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kg7ueVuBhBfAmcGqguZji
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (event_id); unik (sak_id, versjon). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE); prosjekt_id → projects.id (uten fremmednøkkel); actorid → app_users.id (uten fremmednøkkel); actorteam → catenda_contract_teams.team_id (uten fremmednøkkel); referstoid → hendelse.event_id (uten fremmednøkkel); data → vedlegg_ids[] → vedlegg.vedlegg_id (uten fremmednøkkel). Vises til fra: approvals.body → items[].claimId (uten fremmednøkkel); approvals.body → packages[].eventIds[] (uten fremmednøkkel); catenda_delivery_status.event_id (uten fremmednøkkel); notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id); unik (event_id); unik (sak_id, versjon). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE); prosjekt_id → projects.id (uten fremmednøkkel); actorid → app_users.id (uten fremmednøkkel); actorteam → catenda_contract_teams.team_id (uten fremmednøkkel); referstoid → hendelse.event_id (uten fremmednøkkel); data → vedlegg_ids[] → vedlegg.vedlegg_id (uten fremmednøkkel). Vises til fra: approvals.body → items[].claimId (uten fremmednøkkel); approvals.body → packages[].eventIds[] (uten fremmednøkkel); catenda_delivery_status.event_id (uten fremmednøkkel); leveringsoppdrag.event_id (fremmednøkkel, ON DELETE CASCADE); notat.refererer_til_event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -561,12 +561,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>notat</t>
+          <t>leveringsoppdrag</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Interne notater i en sak. Synlige bare for forfatterens eget team, ikke for motparten og ikke for andre team på samme side. Ligger utenfor journalen: et notat er ikke et kontraktsvarsel og flytter ikke sakens versjon (MS-05).</t>
+          <t>Leveringsoppdraget for et brev TS-serveren skriver (LV-U1, B-03, dokumentet). Én rad per brev, og ett brev er ett dokument i Catenda. `innhold` fryser det som skal leveres: brevet slik det ble lagret, målet i Catenda, statusetiketten og versjonene. Raden er uforanderlig; et nytt leveringsforsøk sender samme innhold. Et lagret oppdrag beviser ikke at brevet er sendt eller mottatt. Forsøk, feil og kvitteringer er ikke bygget (#ISSUE-LEVERING). Bare testmiljøet skriver tabellen (#347).</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Når en bruker skriver et internt notat i en sak (hendelsesruta). Forfatteren kan slette notatet.</t>
+          <t>Når TS-serveren lagrer et brev: i samme transaksjon som hendelsen i `hendelse`. Slettes bare med saken eller hendelsen (kaskade).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -586,12 +586,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `aktor_rolle` og `aktor_team_id` er utledet av teammedlemskapet i Catenda da notatet ble skrevet. Innholdet kommer fra brukeren. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
+          <t>Nei. Målet (prosjekt, bibliotek, mappe og topic) leses fra prosjektets Catenda-konfigurasjon og saksregisteret når brevet lagres. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE); prosjekt_id → projects.id (uten fremmednøkkel); aktor_id → app_users.id (uten fremmednøkkel); aktor_team_id → catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE); event_id → hendelse.event_id (fremmednøkkel, ON DELETE CASCADE); prosjekt_id → projects.id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -611,44 +611,44 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på forfatteren. `tekst` og `kommentar` er fritekst.</t>
+          <t>`innhold` har avsenderens `aktor_id` og brevets fritekst.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>notat</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: én rad per sak, med prosjekt, sakstype, hvem som opprettet den, og koblingen til topic, board og prosjekt i Catenda. I tillegg ti `cached_*`-kolonner og `last_event_at` med tall regnet ut av hendelsene, til lister og rapportering. Fem `kjerne_*`-kolonner er bufferen TS-kjernen regner ut av journalen: visningen og de fire versjonene den er regnet med (B-10, #316). Tabellen blander register og projeksjon; skillet er planlagt (MS-06, MS-07).</t>
+          <t>Interne notater i en sak. Synlige bare for forfatterens eget team, ikke for motparten og ikke for andre team på samme side. Ligger utenfor journalen: et notat er ikke et kontraktsvarsel og flytter ikke sakens versjon (MS-05).</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Når en bruker skriver et internt notat i en sak (hendelsesruta). Forfatteren kan slette notatet.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Opprettes når en sak lages, gjennom `SakCreationService`: fra hendelsesrutene, for endringsordrer, og fra en ny topic i Catenda via webhook. Hvordan en forseringssak får sin rad, er ikke kontrollert. `cached_*` oppdateres etter lagrede hendelser (hendelsesrutene, forsering og godkjenning). `kjerne_*` skrives bare av bufferen i TS-kjernen (`kjerne/buffer.ts`, lageret i `sprakprove/kjernelagring/bane.ts` til skrivestien i #310).</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Delvis</t>
-        </is>
-      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `catenda_topic_id`, `catenda_board_id` og `catenda_project_id` er ID-er fra Catenda. Dataflyt: fra Catenda i C01, C15; til Catenda i C01, C15 (arket Dataflyt).</t>
+          <t>Delvis. `aktor_rolle` og `aktor_team_id` er utledet av teammedlemskapet i Catenda da notatet ble skrevet. Innholdet kommer fra brukeren. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: prosjekt_id → projects.id (uten fremmednøkkel); created_by → app_users.id (uten fremmednøkkel); catenda_project_id → catenda_project_configs.catenda_project_id (uten fremmednøkkel); catenda_board_id → catenda_topic_board_configs.topic_board_id (uten fremmednøkkel). Vises til fra: approval_outbox.case_id (uten fremmednøkkel); approvals.case_id (uten fremmednøkkel); catenda_delivery_status.case_id (uten fremmednøkkel); eo_approvals.body → packages[].sakId (uten fremmednøkkel); eo_approvals.body → packages[].request.koe_sak_ids[] (uten fremmednøkkel); hendelse.sak_id (fremmednøkkel, ON DELETE CASCADE); magic_links.sak_id (fremmednøkkel, ON DELETE CASCADE); notat.sak_id (fremmednøkkel, ON DELETE CASCADE); sak_bim_links.sak_id (fremmednøkkel, ON DELETE CASCADE); sak_relations.source_sak_id (uten fremmednøkkel); sak_relations.target_sak_id (uten fremmednøkkel); utkast.case_id (uten fremmednøkkel); vedlegg.case_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE); prosjekt_id → projects.id (uten fremmednøkkel); aktor_id → app_users.id (uten fremmednøkkel); aktor_team_id → catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>grunndata, avledet</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>`created_by` identifiserer den som opprettet saken (tre verdiformer, MG-04).</t>
+          <t>`aktor_id` peker på forfatteren. `tekst` og `kommentar` er fritekst.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>sak_relations</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Koblinger mellom saker, for eksempel hvilke KOE-er en forsering eller en endringsordre omfatter. Én rad per kobling, med type.</t>
+          <t>Saksregisteret: én rad per sak, med prosjekt, sakstype, hvem som opprettet den, og koblingen til topic, board og prosjekt i Catenda. I tillegg ti `cached_*`-kolonner og `last_event_at` med tall regnet ut av hendelsene, til lister og rapportering. Fem `kjerne_*`-kolonner er bufferen TS-kjernen regner ut av journalen: visningen og de fire versjonene den er regnet med (B-10, #316). Tabellen blander register og projeksjon; skillet er planlagt (MS-06, MS-07).</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -690,22 +690,22 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Når en forsering opprettes gjennom `/api/forsering/opprett`, og når en endringsordre opprettes eller KOE-er legges til eller fjernes fra den (forsering- og endringsordretjenesten). Å legge til eller fjerne KOE-er fra en forsering endrer bare Catenda, ikke denne tabellen (dataflyten, C11).</t>
+          <t>Opprettes når en sak lages, gjennom `SakCreationService`: fra hendelsesrutene, for endringsordrer, og fra en ny topic i Catenda via webhook. Hvordan en forseringssak får sin rad, er ikke kontrollert. `cached_*` oppdateres etter lagrede hendelser (hendelsesrutene, forsering og godkjenning). `kjerne_*` skrives bare av bufferen i TS-kjernen (`kjerne/buffer.ts`, lageret i `sprakprove/kjernelagring/bane.ts` til skrivestien i #310).</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Delvis</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Delvis. En forsering opprettet gjennom `/api/forsering/opprett` får topicens GUID fra Catenda som sak-ID. Ellers er koblingene appens egne. Dataflyt: fra Catenda i C10 (arket Dataflyt).</t>
+          <t>Delvis. `catenda_topic_id`, `catenda_board_id` og `catenda_project_id` er ID-er fra Catenda. Dataflyt: fra Catenda i C01, C15; til Catenda i C01, C15 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (source_sak_id, target_sak_id, relation_type). Viser til: source_sak_id → sak_metadata.sak_id (uten fremmednøkkel); target_sak_id → sak_metadata.sak_id (uten fremmednøkkel); prosjekt_id → projects.id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: prosjekt_id → projects.id (uten fremmednøkkel); created_by → app_users.id (uten fremmednøkkel); catenda_project_id → catenda_project_configs.catenda_project_id (uten fremmednøkkel); catenda_board_id → catenda_topic_board_configs.topic_board_id (uten fremmednøkkel). Vises til fra: approval_outbox.case_id (uten fremmednøkkel); approvals.case_id (uten fremmednøkkel); catenda_delivery_status.case_id (uten fremmednøkkel); eo_approvals.body → packages[].sakId (uten fremmednøkkel); eo_approvals.body → packages[].request.koe_sak_ids[] (uten fremmednøkkel); hendelse.sak_id (fremmednøkkel, ON DELETE CASCADE); leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE CASCADE); magic_links.sak_id (fremmednøkkel, ON DELETE CASCADE); notat.sak_id (fremmednøkkel, ON DELETE CASCADE); sak_bim_links.sak_id (fremmednøkkel, ON DELETE CASCADE); sak_relations.source_sak_id (uten fremmednøkkel); sak_relations.target_sak_id (uten fremmednøkkel); utkast.case_id (uten fremmednøkkel); vedlegg.case_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>grunndata, avledet</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -725,19 +725,19 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>`created_by` identifiserer den som opprettet saken (tre verdiformer, MG-04).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>sak_relations</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene i appen, med navn, beskrivelse, innstillinger, om prosjektet er aktivt, og organisasjonen det hører til (MS-10).</t>
+          <t>Koblinger mellom saker, for eksempel hvilke KOE-er en forsering eller en endringsordre omfatter. Én rad per kobling, med type.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -747,22 +747,22 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Registreres av drift gjennom databasefunksjonen `koe_register_project` (`scripts/catenda_admin.py`). `POST /api/projects` svarer 403 utenfor utviklingsmodus. En prosjektadministrator kan endre navn, beskrivelse og innstillinger og deaktivere prosjektet (`PATCH`). Driftsskriptet `catenda_admin.py sync-name` oppdaterer navnet direkte fra Catenda, utenom databasefunksjonen. At runtime-rollen heller ikke skal kunne kalle funksjonen, gjelder databaserettighetene og hører til F1 (B-02 punkt 4). En migrasjon legger inn prosjektet `oslobygg`, og det er i dag basens eneste prosjekt (DM-03).</t>
+          <t>Når en forsering opprettes gjennom `/api/forsering/opprett`, og når en endringsordre opprettes eller KOE-er legges til eller fjernes fra den (forsering- og endringsordretjenesten). Å legge til eller fjerne KOE-er fra en forsering endrer bare Catenda, ikke denne tabellen (dataflyten, C11).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Navnet kan hentes fra Catenda-prosjektet når drift registrerer prosjektet eller kjører `sync-name`. Koblingen til Catenda-prosjektet ligger i `catenda_project_configs`. Dataflyt: fra Catenda i C18, C20 (arket Dataflyt).</t>
+          <t>Delvis. En forsering opprettet gjennom `/api/forsering/opprett` får topicens GUID fra Catenda som sak-ID. Ellers er koblingene appens egne. Dataflyt: fra Catenda i C10 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: app_membership_sync.project_id (fremmednøkkel, ON DELETE CASCADE); app_project_memberships.project_id (fremmednøkkel, ON DELETE CASCADE); approval_outbox.project (uten fremmednøkkel); approvals.project (uten fremmednøkkel); catenda_delivery_status.project (uten fremmednøkkel); catenda_models_cache.prosjekt_id (uten fremmednøkkel); catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE); eo_approvals.project (uten fremmednøkkel); hendelse.prosjekt_id (uten fremmednøkkel); notat.prosjekt_id (uten fremmednøkkel); project_memberships.project_id (fremmednøkkel, ON DELETE CASCADE); sak_metadata.prosjekt_id (uten fremmednøkkel); sak_relations.prosjekt_id (uten fremmednøkkel); utkast.project (uten fremmednøkkel); vedlegg.project (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id); unik (source_sak_id, target_sak_id, relation_type). Viser til: source_sak_id → sak_metadata.sak_id (uten fremmednøkkel); target_sak_id → sak_metadata.sak_id (uten fremmednøkkel); prosjekt_id → projects.id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -782,19 +782,19 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>`created_by` identifiserer den som opprettet prosjektet.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>project_memberships</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Eldre medlemsliste per prosjekt, etter e-post. Erstattet av `app_project_memberships` og skal fjernes (MS-15) når `viewer` finnes der (DB-05).</t>
+          <t>Prosjektene i appen, med navn, beskrivelse, innstillinger, om prosjektet er aktivt, og organisasjonen det hører til (MS-10).</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `trg_auto_membership_on_project_create` legger inn en rad når et prosjekt opprettes. Koden som ser ut til å skrive tabellen, treffer en unik-skranke (AGENTS.md). Ingen leser den (DA-10).</t>
+          <t>Registreres av drift gjennom databasefunksjonen `koe_register_project` (`scripts/catenda_admin.py`). `POST /api/projects` svarer 403 utenfor utviklingsmodus. En prosjektadministrator kan endre navn, beskrivelse og innstillinger og deaktivere prosjektet (`PATCH`). Driftsskriptet `catenda_admin.py sync-name` oppdaterer navnet direkte fra Catenda, utenom databasefunksjonen. At runtime-rollen heller ikke skal kunne kalle funksjonen, gjelder databaserettighetene og hører til F1 (B-02 punkt 4). En migrasjon legger inn prosjektet `oslobygg`, og det er i dag basens eneste prosjekt (DM-03).</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Navnet kan hentes fra Catenda-prosjektet når drift registrerer prosjektet eller kjører `sync-name`. Koblingen til Catenda-prosjektet ligger i `catenda_project_configs`. Dataflyt: fra Catenda i C18, C20 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (project_id, user_email). Viser til: project_id → projects.id (fremmednøkkel, ON DELETE CASCADE).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: app_membership_sync.project_id (fremmednøkkel, ON DELETE CASCADE); app_project_memberships.project_id (fremmednøkkel, ON DELETE CASCADE); approval_outbox.project (uten fremmednøkkel); approvals.project (uten fremmednøkkel); catenda_delivery_status.project (uten fremmednøkkel); catenda_models_cache.prosjekt_id (uten fremmednøkkel); catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE); eo_approvals.project (uten fremmednøkkel); hendelse.prosjekt_id (uten fremmednøkkel); leveringsoppdrag.prosjekt_id (uten fremmednøkkel); notat.prosjekt_id (uten fremmednøkkel); project_memberships.project_id (fremmednøkkel, ON DELETE CASCADE); sak_metadata.prosjekt_id (uten fremmednøkkel); sak_relations.prosjekt_id (uten fremmednøkkel); utkast.project (uten fremmednøkkel); vedlegg.project (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -834,24 +834,24 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>rest</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>`user_email`, `display_name`, `external_id`.</t>
+          <t>`created_by` identifiserer den som opprettet prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>app_users</t>
+          <t>project_memberships</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Brukerne. Én rad per person, med e-post og navn. `id` er identiteten journalen bærer i `aktor_id`.</t>
+          <t>Eldre medlemsliste per prosjekt, etter e-post. Erstattet av `app_project_memberships` og skal fjernes (MS-15) når `viewer` finnes der (DB-05).</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Bare gjennom databasefunksjonen `koe_resolve_identity`. Den kalles ved innlogging, når en webhook fra Catenda har en forfatter, og for hvert medlem når medlemslisten synkroniseres. E-post og navn oppdateres fra Catenda hver gang.</t>
+          <t>Triggeren `trg_auto_membership_on_project_create` legger inn en rad når et prosjekt opprettes. Koden som ser ut til å skrive tabellen, treffer en unik-skranke (AGENTS.md). Ingen leser den (DA-10).</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -871,12 +871,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Ja. E-post og navn kommer fra Catenda-profilen og medlemslisten. Dataflyt: fra Catenda i C01, C03, C04 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: app_identities.user_id (fremmednøkkel, ON DELETE CASCADE); app_project_memberships.user_id (fremmednøkkel, ON DELETE CASCADE); app_sessions.user_id (fremmednøkkel, ON DELETE CASCADE); hendelse.actorid (uten fremmednøkkel); notat.aktor_id (uten fremmednøkkel); sak_metadata.created_by (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id); unik (project_id, user_email). Viser til: project_id → projects.id (fremmednøkkel, ON DELETE CASCADE).</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -891,24 +891,24 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>rest</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>`email` og `name`.</t>
+          <t>`user_email`, `display_name`, `external_id`.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>app_identities</t>
+          <t>app_users</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Kobler en bruker til en ekstern identitet: tilbyder, utsteder og subjekt i Catenda. Sørger for at samme person får samme brukerrad uansett vei inn.</t>
+          <t>Brukerne. Én rad per person, med e-post og navn. `id` er identiteten journalen bærer i `aktor_id`.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Bare gjennom `koe_resolve_identity`, som også er eneste leser. Ingen Python-kode leser eller skriver tabellen direkte (DA-07).</t>
+          <t>Bare gjennom databasefunksjonen `koe_resolve_identity`. Den kalles ved innlogging, når en webhook fra Catenda har en forfatter, og for hvert medlem når medlemslisten synkroniseres. E-post og navn oppdateres fra Catenda hver gang.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -928,12 +928,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Ja. Subjektet er Catenda-ID-en. Dataflyt: fra Catenda i C01, C03, C04 (arket Dataflyt).</t>
+          <t>Ja. E-post og navn kommer fra Catenda-profilen og medlemslisten. Dataflyt: fra Catenda i C01, C03, C04 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: user_id → app_users.id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: app_project_memberships.catenda_subject (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: app_identities.user_id (fremmednøkkel, ON DELETE CASCADE); app_project_memberships.user_id (fremmednøkkel, ON DELETE CASCADE); app_sessions.user_id (fremmednøkkel, ON DELETE CASCADE); hendelse.actorid (uten fremmednøkkel); notat.aktor_id (uten fremmednøkkel); sak_metadata.created_by (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -953,19 +953,19 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>`subject` er en ekstern identifikator for en person.</t>
+          <t>`email` og `name`.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>app_sessions</t>
+          <t>app_identities</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer en hash av sesjonstokenet, CSRF-tokenet og når sesjonen utløper.</t>
+          <t>Kobler en bruker til en ekstern identitet: tilbyder, utsteder og subjekt i Catenda. Sørger for at samme person får samme brukerrad uansett vei inn.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -975,22 +975,22 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Opprettes ved innlogging og slettes ved utlogging (innloggingsrutene). Utløpte rader ryddes av `scripts/sync_catenda_memberships.py`. Om skriptet kjører noe sted, er ikke kontrollert.</t>
+          <t>Bare gjennom `koe_resolve_identity`, som også er eneste leser. Ingen Python-kode leser eller skriver tabellen direkte (DA-07).</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja. Subjektet er Catenda-ID-en. Dataflyt: fra Catenda i C01, C03, C04 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → app_users.id (fremmednøkkel, ON DELETE CASCADE).</t>
+          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: user_id → app_users.id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: app_project_memberships.catenda_subject (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1010,19 +1010,19 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`.</t>
+          <t>`subject` er en ekstern identifikator for en person.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>app_oauth_attempts</t>
+          <t>app_sessions</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Påbegynte innlogginger mot Catenda (OAuth). Kortlevde rader som binder tilbakekallet til nettleseren som startet innloggingen.</t>
+          <t>Innloggingssesjoner. Lagrer en hash av sesjonstokenet, CSRF-tokenet og når sesjonen utløper.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Opprettes når innloggingen starter, og brukes opp når Catenda sender brukeren tilbake (innloggingsrutene).</t>
+          <t>Opprettes ved innlogging og slettes ved utlogging (innloggingsrutene). Utløpte rader ryddes av `scripts/sync_catenda_memberships.py`. Om skriptet kjører noe sted, er ikke kontrollert.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1042,12 +1042,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → app_users.id (fremmednøkkel, ON DELETE CASCADE).</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1067,19 +1067,19 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente; bare hasher og en returadresse.</t>
+          <t>Knyttet til en bruker gjennom `user_id`.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>app_project_memberships</t>
+          <t>app_oauth_attempts</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Hvem som er medlem av hvilket prosjekt, med rolle, og om medlemskapet er aktivt. En kopi av medlemslisten i Catenda, pluss appens egen `viewer_override`.</t>
+          <t>Påbegynte innlogginger mot Catenda (OAuth). Kortlevde rader som binder tilbakekallet til nettleseren som startet innloggingen.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1089,22 +1089,22 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Databasefunksjonen `koe_reconcile_memberships` synkroniserer mot Catenda ved innlogging, fra medlemsruta og fra skriptet `scripts/sync_catenda_memberships.py`. Medlemsruta setter `viewer_override`. Innloggingen kan også deaktivere medlemskap.</t>
+          <t>Opprettes når innloggingen starter, og brukes opp når Catenda sender brukeren tilbake (innloggingsrutene).</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Delvis</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Ja. Medlemslisten hentes fra Catenda-prosjektet. Dataflyt: fra Catenda i C03, C04 (arket Dataflyt).</t>
+          <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (project_id, catenda_subject); unik (project_id, user_id). Viser til: project_id → projects.id (fremmednøkkel, ON DELETE CASCADE); user_id → app_users.id (fremmednøkkel, ON DELETE CASCADE); catenda_subject → app_identities.subject (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>grunndata, kopi</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1124,19 +1124,19 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>`user_email`, `display_name` og `catenda_subject`.</t>
+          <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>app_membership_sync</t>
+          <t>app_project_memberships</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for et prosjekt sist ble synkronisert fra Catenda. Hindrer at en eldre synkronisering overskriver en nyere.</t>
+          <t>Hvem som er medlem av hvilket prosjekt, med rolle, og om medlemskapet er aktivt. En kopi av medlemslisten i Catenda, pluss appens egen `viewer_override`.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1146,22 +1146,22 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Av `koe_reconcile_memberships`, samtidig med medlemskapene.</t>
+          <t>Databasefunksjonen `koe_reconcile_memberships` synkroniserer mot Catenda ved innlogging, fra medlemsruta og fra skriptet `scripts/sync_catenda_memberships.py`. Medlemsruta setter `viewer_override`. Innloggingen kan også deaktivere medlemskap.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Delvis</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `catenda_project_id` er en Catenda-ID. Dataflyt: fra Catenda i C04 (arket Dataflyt).</t>
+          <t>Ja. Medlemslisten hentes fra Catenda-prosjektet. Dataflyt: fra Catenda i C03, C04 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → projects.id (fremmednøkkel, ON DELETE CASCADE); catenda_project_id → catenda_project_configs.catenda_project_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id); unik (project_id, catenda_subject); unik (project_id, user_id). Viser til: project_id → projects.id (fremmednøkkel, ON DELETE CASCADE); user_id → app_users.id (fremmednøkkel, ON DELETE CASCADE); catenda_subject → app_identities.subject (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata, kopi</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1181,19 +1181,19 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>`user_email`, `display_name` og `catenda_subject`.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>app_membership_sync</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Kobler et prosjekt i appen til prosjektet, dokumentbiblioteket og mappen i Catenda.</t>
+          <t>Når medlemslisten for et prosjekt sist ble synkronisert fra Catenda. Hindrer at en eldre synkronisering overskriver en nyere.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1203,22 +1203,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Av `koe_register_project`, som drift kaller gjennom `scripts/catenda_admin.py`.</t>
+          <t>Av `koe_reconcile_memberships`, samtidig med medlemskapene.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Ja. ID-ene er Catenda-ID-er, oppgitt ved registrering. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. `catenda_project_id` er en Catenda-ID. Dataflyt: fra Catenda i C04 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → projects.id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: app_membership_sync.catenda_project_id (uten fremmednøkkel); catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE CASCADE); catenda_models_cache.catenda_project_id (uten fremmednøkkel); catenda_topic_board_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE); sak_metadata.catenda_project_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → projects.id (fremmednøkkel, ON DELETE CASCADE); catenda_project_id → catenda_project_configs.catenda_project_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1245,12 +1245,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_board_configs</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Hvilke topic boards i Catenda som hører til et prosjekt. Brukes blant annet til å finne prosjektet når en webhook kommer.</t>
+          <t>Kobler et prosjekt i appen til prosjektet, dokumentbiblioteket og mappen i Catenda.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Ja. `topic_board_id` er en Catenda-ID. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja. ID-ene er Catenda-ID-er, oppgitt ved registrering. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (topic_board_id). Viser til: internal_project_id → catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: sak_metadata.catenda_board_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → projects.id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: app_membership_sync.catenda_project_id (uten fremmednøkkel); catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE CASCADE); catenda_models_cache.catenda_project_id (uten fremmednøkkel); catenda_topic_board_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE); sak_metadata.catenda_project_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1302,12 +1302,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>catenda_topic_board_configs</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Hvilke Catenda-team som representerer TE og BH i et prosjekt. Appen utleder en brukers kontraktsside og team herfra og fra medlemskapet i Catenda.</t>
+          <t>Hvilke topic boards i Catenda som hører til et prosjekt. Brukes blant annet til å finne prosjektet når en webhook kommer.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Av `koe_set_contract_teams` og `koe_register_project`, som drift kaller gjennom `scripts/catenda_admin.py`. Etter B-02 punkt 4 er det bare drift som skal gjøre dette.</t>
+          <t>Av `koe_register_project`, som drift kaller gjennom `scripts/catenda_admin.py`.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1327,12 +1327,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Ja. `team_id` er en Catenda-ID. Dataflyt: fra Catenda i C18, C19 (arket Dataflyt).</t>
+          <t>Ja. `topic_board_id` er en Catenda-ID. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: hendelse.actorteam (uten fremmednøkkel); notat.aktor_team_id (uten fremmednøkkel); utkast.team (uten fremmednøkkel); vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (topic_board_id). Viser til: internal_project_id → catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: sak_metadata.catenda_board_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1359,12 +1359,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>catenda_models_cache</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ment som kopi av BIM-modellene i Catenda per prosjekt, med fag. Tre BIM-ruter leser den og gir tomme lister når den er tom.</t>
+          <t>Hvilke Catenda-team som representerer TE og BH i et prosjekt. Appen utleder en brukers kontraktsside og team herfra og fra medlemskapet i Catenda.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1374,22 +1374,22 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Ikke funnet. Ingen kode, databasefunksjon eller trigger skriver tabellen, og `upsert_cached_models` har ingen kaller (DM-02, foreløpig).</t>
+          <t>Av `koe_set_contract_teams` og `koe_register_project`, som drift kaller gjennom `scripts/catenda_admin.py`. Etter B-02 punkt 4 er det bare drift som skal gjøre dette.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Ja, etter formålet. Hvordan den skulle fylles, er ikke kjent. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja. `team_id` er en Catenda-ID. Dataflyt: fra Catenda i C18, C19 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (catenda_project_id, model_id). Viser til: prosjekt_id → projects.id (uten fremmednøkkel); catenda_project_id → catenda_project_configs.catenda_project_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE CASCADE). Vises til fra: hendelse.actorteam (uten fremmednøkkel); notat.aktor_team_id (uten fremmednøkkel); utkast.team (uten fremmednøkkel); vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1399,12 +1399,12 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>kopi</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1416,22 +1416,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>sak_bim_links</t>
+          <t>catenda_models_cache</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Kobler en sak til et objekt i en BIM-modell, med modell, objekt-ID, IFC-type, egenskaper og hvem som koblet. Formålet er å se hvilke komponenter som fører til tvist (P2, P3).</t>
+          <t>Ment som kopi av BIM-modellene i Catenda per prosjekt, med fag. Tre BIM-ruter leser den og gir tomme lister når den er tom.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Når en bruker kobler et objekt til en sak eller fjerner koblingen (BIM-rutene).</t>
+          <t>Ikke funnet. Ingen kode, databasefunksjon eller trigger skriver tabellen, og `upsert_cached_models` har ingen kaller (DM-02, foreløpig).</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Modell- og objekt-ID-ene er fra Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, etter formålet. Hvordan den skulle fylles, er ikke kjent. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (sak_id, fag, COALESCE(model_id, ''::text), COALESCE(object_global_id, ''::text)). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE).</t>
+          <t>Nøkler: primærnøkkel (id); unik (catenda_project_id, model_id). Viser til: prosjekt_id → projects.id (uten fremmednøkkel); catenda_project_id → catenda_project_configs.catenda_project_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1456,54 +1456,54 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>kopi</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>`linked_by` identifiserer den som koblet (e-post, lest i ruta).</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>magic_links</t>
+          <t>sak_bim_links</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Etterlatenskap fra en eldre innlogging med lenke på e-post. Magic links utgår (P1), og tabellen skal fjernes (MS-15).</t>
+          <t>Kobler en sak til et objekt i en BIM-modell, med modell, objekt-ID, IFC-type, egenskaper og hvem som koblet. Formålet er å se hvilke komponenter som fører til tvist (P2, P3).</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Når en bruker kobler et objekt til en sak eller fjerner koblingen (BIM-rutene).</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Ingen kode leser eller skriver tabellen (DA-09). `MagicLinkManager` i `lib/auth/magic_link.py` lagrer i en JSON-fil, ikke her.</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Modell- og objekt-ID-ene er fra Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (sak_id, fag, COALESCE(model_id, ''::text), COALESCE(object_global_id, ''::text)). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE).</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1513,29 +1513,29 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>rest</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>`email`.</t>
+          <t>`linked_by` identifiserer den som koblet (e-post, lest i ruta).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>user_groups</t>
+          <t>magic_links</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Etterlatenskap: brukergrupper med roller og leder. Ingen kode bruker den, og den skal fjernes (MS-15).</t>
+          <t>Etterlatenskap fra en eldre innlogging med lenke på e-post. Magic links utgår (P1), og tabellen skal fjernes (MS-15).</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1545,12 +1545,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Ingen. To databasefunksjoner, `get_user_role` og `get_user_role_by_email`, leser tabellen, men ingen kaller dem (DA-08).</t>
+          <t>Ingen kode leser eller skriver tabellen (DA-09). `MagicLinkManager` i `lib/auth/magic_link.py` lagrer i en JSON-fil, ikke her.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (user_id). Viser til: manager_id → user_groups.id (fremmednøkkel, ON DELETE SET NULL); user_id → auth.users.id (fremmednøkkel, ON DELETE CASCADE).</t>
+          <t>Nøkler: primærnøkkel (token). Viser til: sak_id → sak_metadata.sak_id (fremmednøkkel, ON DELETE CASCADE).</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1580,19 +1580,19 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>`display_name`, `department` og koblingen til en bruker.</t>
+          <t>`email`.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>utkast</t>
+          <t>user_groups</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Teamets arbeidsutkast til et svar eller krav, per sak, spor og revisjon. Utkastet tilhører teamet, ikke personen, og er skjult for alle andre. `versjon` avviser samtidige lagringer.</t>
+          <t>Etterlatenskap: brukergrupper med roller og leder. Ingen kode bruker den, og den skal fjernes (MS-15).</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1602,64 +1602,64 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Når en bruker skriver i et skjema: utkastrutene (`GET`, `PUT` og `DELETE` på `/api/cases/&lt;sak_id&gt;/utkast/&lt;spor&gt;`).</t>
+          <t>Ingen. To databasefunksjoner, `get_user_role` og `get_user_role_by_email`, leser tabellen, men ingen kaller dem (DA-08).</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Teamet og kontraktssiden er utledet av teammedlemskapet i Catenda. Innholdet kommer fra brukeren. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project, case_id, spor, revisjon, team). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); team → catenda_contract_teams.team_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id); unik (user_id). Viser til: manager_id → user_groups.id (fremmednøkkel, ON DELETE SET NULL); user_id → auth.users.id (fremmednøkkel, ON DELETE CASCADE).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>PostgreSQL</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>rest</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>`oppdatert_av` og fritekst i `innhold`.</t>
+          <t>`display_name`, `department` og koblingen til en bruker.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>approvals</t>
+          <t>utkast</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Byggherrens interne godkjenning av svar i en sak: poster, godkjenningspakker og kommandoer, lagret som ett JSON-dokument per sak. Når en pakke er godkjent og publisert, skrives svarene til journalen.</t>
+          <t>Teamets arbeidsutkast til et svar eller krav, per sak, spor og revisjon. Utkastet tilhører teamet, ikke personen, og er skjult for alle andre. `versjon` avviser samtidige lagringer.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Godkjenningsrutene, gjennom `ApprovalService`.</t>
+          <t>Når en bruker skriver i et skjema: utkastrutene (`GET`, `PUT` og `DELETE` på `/api/cases/&lt;sak_id&gt;/utkast/&lt;spor&gt;`).</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Teamet og kontraktssiden er utledet av teammedlemskapet i Catenda. Innholdet kommer fra brukeren. Dataflyt: fra Catenda i C05 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project, case_id). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); body → items[].claimId → hendelse.event_id (uten fremmednøkkel); body → packages[].eventIds[] → hendelse.event_id (uten fremmednøkkel). Vises til fra: approval_outbox.id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project, case_id, spor, revisjon, team). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); team → catenda_contract_teams.team_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1694,44 +1694,44 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Godkjennere og saksbehandlere i JSON-dokumentet; ikke kontrollert i detalj.</t>
+          <t>`oppdatert_av` og fritekst i `innhold`.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>approval_outbox</t>
+          <t>approvals</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Kø for varsling etter at en godkjenningspakke er publisert. Én rad per pakke, med status (`pending`, `sending`, `delivered`, `failed`, `not_configured`).</t>
+          <t>Byggherrens interne godkjenning av svar i en sak: poster, godkjenningspakker og kommandoer, lagret som ett JSON-dokument per sak. Når en pakke er godkjent og publisert, skrives svarene til journalen.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Godkjenningsrutene, gjennom `ApprovalService`.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Av `ApprovalService` ved publisering og levering.</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: kvittering for kall til Catenda i C07 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Viser til: id → approvals.body → packages[].id (uten fremmednøkkel); project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project, case_id). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); body → items[].claimId → hendelse.event_id (uten fremmednøkkel); body → packages[].eventIds[] → hendelse.event_id (uten fremmednøkkel). Vises til fra: approval_outbox.id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1751,29 +1751,29 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Godkjennere og saksbehandlere i JSON-dokumentet; ikke kontrollert i detalj.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>eo_approvals</t>
+          <t>approval_outbox</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Godkjenning av endringsordrer før utstedelse, lagret som ett JSON-dokument per prosjekt.</t>
+          <t>Kø for varsling etter at en godkjenningspakke er publisert. Én rad per pakke, med status (`pending`, `sending`, `delivered`, `failed`, `not_configured`).</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Endringsordrerutene, gjennom `EOApprovalService`.</t>
+          <t>Av `ApprovalService` ved publisering og levering.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1783,12 +1783,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: kvittering for kall til Catenda i C07 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project). Viser til: project → projects.id (uten fremmednøkkel); body → packages[].sakId → sak_metadata.sak_id (uten fremmednøkkel); body → packages[].request.koe_sak_ids[] → sak_metadata.sak_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (id). Viser til: id → approvals.body → packages[].id (uten fremmednøkkel); project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1808,19 +1808,19 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Godkjennere i JSON-dokumentet; ikke kontrollert i detalj.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>vedlegg</t>
+          <t>eo_approvals</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Register over vedlegg i en sak, med status: `staged` (valgt, ikke sendt), `pending` (sendt i en lagret hendelse, venter på Catenda) og `delivered` (lastet opp og koblet i Catenda). Filinnholdet mellomlagres her fram til opplastingen.</t>
+          <t>Godkjenning av endringsordrer før utstedelse, lagret som ett JSON-dokument per prosjekt.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Vedleggsrutene og hendelsesrutene, gjennom `VedleggRegistry`.</t>
+          <t>Endringsordrerutene, gjennom `EOApprovalService`.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1840,12 +1840,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `catenda_item_id` er Catendas ID etter opplasting. Dataflyt: fra Catenda i C05, C08; til Catenda i C08; kvittering for kall til Catenda i C08 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project, case_id, vedlegg_id). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); lastet_opp_team → catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: hendelse.data → vedlegg_ids[] (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project). Viser til: project → projects.id (uten fremmednøkkel); body → packages[].sakId → sak_metadata.sak_id (uten fremmednøkkel); body → packages[].request.koe_sak_ids[] → sak_metadata.sak_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1865,62 +1865,119 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Filinnholdet kan inneholde personopplysninger; ikke kontrollert.</t>
+          <t>Godkjennere i JSON-dokumentet; ikke kontrollert i detalj.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>vedlegg</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Register over vedlegg i en sak, med status: `staged` (valgt, ikke sendt), `pending` (sendt i en lagret hendelse, venter på Catenda) og `delivered` (lastet opp og koblet i Catenda). Filinnholdet mellomlagres her fram til opplastingen.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Vedleggsrutene og hendelsesrutene, gjennom `VedleggRegistry`.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Delvis. `catenda_item_id` er Catendas ID etter opplasting. Dataflyt: fra Catenda i C05, C08; til Catenda i C08; kvittering for kall til Catenda i C08 (arket Dataflyt).</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (project, case_id, vedlegg_id). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); lastet_opp_team → catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: hendelse.data → vedlegg_ids[] (uten fremmednøkkel).</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>SQLite</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Filinnholdet kan inneholde personopplysninger; ikke kontrollert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>catenda_delivery_status</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Kvittering per hendelse for levering til Catenda (`pending`, `failed`, `delivered`), vist i banneret på saken. Ikke en kø for nye forsøk.</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Hendelsesrutene.</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Nei, men statusen gjelder et kall til Catenda. Dataflyt: kvittering for kall til Catenda i C06 (arket Dataflyt).</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (project, case_id, event_id). Viser til: project → projects.id (uten fremmednøkkel); case_id → sak_metadata.sak_id (uten fremmednøkkel); event_id → hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>SQLite</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente.</t>
         </is>
@@ -1937,7 +1994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2037,7 +2094,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>notat</t>
+          <t>leveringsoppdrag</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2072,29 +2129,29 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Saken notatet er skrevet i.</t>
+          <t>Saken brevet er sendt i. Slettes saken, slettes oppdraget med (ON DELETE CASCADE).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>sak_bim_links</t>
+          <t>leveringsoppdrag</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2104,7 +2161,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2114,14 +2171,14 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Saken BIM-objektet er koblet til.</t>
+          <t>Brevet oppdraget leverer. Unik, så hvert brev har ett oppdrag. Triggeren `leveringsoppdrag_vakt` avviser et oppdrag med en annen sak eller et annet prosjekt enn hendelsen.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>magic_links</t>
+          <t>notat</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -2156,29 +2213,29 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Saken lenken gjaldt. Tabellen er en rest (MS-15).</t>
+          <t>Saken notatet er skrevet i.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>sak_bim_links</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>internal_project_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2188,7 +2245,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2198,29 +2255,29 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet koblingen til Catenda gjelder. Én konfigurasjon per prosjekt.</t>
+          <t>Saken BIM-objektet er koblet til.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_board_configs</t>
+          <t>magic_links</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>internal_project_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>internal_project_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -2240,14 +2297,14 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet topic boardet hører til. Et prosjekt kan ha flere boards.</t>
+          <t>Saken lenken gjaldt. Tabellen er en rest (MS-15).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -2257,12 +2314,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>internal_project_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -2272,7 +2329,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2282,29 +2339,29 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet teamet representerer TE eller BH i.</t>
+          <t>Prosjektet koblingen til Catenda gjelder. Én konfigurasjon per prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>app_identities</t>
+          <t>catenda_topic_board_configs</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>app_users</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2324,29 +2381,29 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Brukeren den eksterne identiteten tilhører.</t>
+          <t>Prosjektet topic boardet hører til. Et prosjekt kan ha flere boards.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>app_sessions</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>app_users</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -2366,24 +2423,24 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Brukeren som er logget inn.</t>
+          <t>Prosjektet teamet representerer TE eller BH i.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>app_project_memberships</t>
+          <t>app_identities</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>project_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>app_users</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2408,14 +2465,14 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet medlemskapet gjelder.</t>
+          <t>Brukeren den eksterne identiteten tilhører.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>app_project_memberships</t>
+          <t>app_sessions</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2450,14 +2507,14 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Brukeren som er medlem. Én rad per prosjekt og bruker (UNIQUE).</t>
+          <t>Brukeren som er logget inn.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>app_membership_sync</t>
+          <t>app_project_memberships</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -2482,7 +2539,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2492,24 +2549,24 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet synkroniseringen gjelder. Én rad per prosjekt.</t>
+          <t>Prosjektet medlemskapet gjelder.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>project_memberships</t>
+          <t>app_project_memberships</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>project_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>app_users</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2534,24 +2591,24 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet i den eldre medlemslisten. Tabellen er en rest (MS-15).</t>
+          <t>Brukeren som er medlem. Én rad per prosjekt og bruker (UNIQUE).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>user_groups</t>
+          <t>app_membership_sync</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>manager_id</t>
+          <t>project_id</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>user_groups</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2566,34 +2623,34 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>SET NULL</t>
+          <t>CASCADE</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Lederen i brukergruppen. Tabellen er en rest (MS-15).</t>
+          <t>Prosjektet synkroniseringen gjelder. Én rad per prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>user_groups</t>
+          <t>project_memberships</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>project_id</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>auth.users</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2608,7 +2665,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2618,24 +2675,24 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Brukeren i Supabase-plattformens egen tabell, ikke `app_users`. Må løses om basen flyttes fra Supabase (B-12). Tabellen er en rest (MS-15).</t>
+          <t>Prosjektet i den eldre medlemslisten. Tabellen er en rest (MS-15).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>user_groups</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>manager_id</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>user_groups</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2645,7 +2702,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2653,27 +2710,31 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>SET NULL</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet hendelsen er skrevet i. Stemples av serveren fra autorisert kontekst, uten default (AGENTS.md, sikkerhetsinvariantene).</t>
+          <t>Lederen i brukergruppen. Tabellen er en rest (MS-15).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>user_groups</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>actorid</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>app_users</t>
+          <t>auth.users</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2683,18 +2744,22 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Den som sendte hendelsen. Verdien er `app_users.id` og aldri et navn (AGENTS.md). Kolonnen er `text`, `id` er `uuid`.</t>
+          <t>Brukeren i Supabase-plattformens egen tabell, ikke `app_users`. Må løses om basen flyttes fra Supabase (B-12). Tabellen er en rest (MS-15).</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2771,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>actorteam</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2732,7 +2797,7 @@
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, utledet fra teammedlemskapet i Catenda da hendelsen ble skrevet. Tom når teamet ikke var entydig. Lagres som 32 heksadesimaler uten bindestreker (`catenda_id`), mens `team_id` er `uuid`; en sammenstilling må normalisere.</t>
+          <t>Prosjektet hendelsen er skrevet i. Stemples av serveren fra autorisert kontekst, uten default (AGENTS.md, sikkerhetsinvariantene).</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2809,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>referstoid</t>
+          <t>actorid</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>app_users</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2770,7 +2835,7 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Kravet et svar gjelder (`refererer_til_event_id`), i samme sak. Forretningsreglene for svar sammenlikner den med sporets gjeldende krav.</t>
+          <t>Den som sendte hendelsen. Verdien er `app_users.id` og aldri et navn (AGENTS.md). Kolonnen er `text`, `id` er `uuid`.</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2847,17 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>data → vedlegg_ids[]</t>
+          <t>actorteam</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>vedlegg</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2802,35 +2867,35 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>mange til mange</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Vedleggene hendelsen sender. Leveringen til Catenda starter fra disse referansene etter at hendelsen er lagret. Sammenlikningen normaliserer med `catenda_id`. Går på tvers av lagene: journalen i PostgreSQL, registeret i SQLite.</t>
+          <t>Teamet avsenderen satt i, utledet fra teammedlemskapet i Catenda da hendelsen ble skrevet. Tom når teamet ikke var entydig. Lagres som 32 heksadesimaler uten bindestreker (`catenda_id`), mens `team_id` er `uuid`; en sammenstilling må normalisere.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>notat</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>referstoid</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2846,29 +2911,29 @@
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet notatet er skrevet i.</t>
+          <t>Kravet et svar gjelder (`refererer_til_event_id`), i samme sak. Forretningsreglene for svar sammenlikner den med sporets gjeldende krav.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>notat</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>data → vedlegg_ids[]</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>app_users</t>
+          <t>vedlegg</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2878,35 +2943,35 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>mange til mange</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Forfatteren.</t>
+          <t>Vedleggene hendelsen sender. Leveringen til Catenda starter fra disse referansene etter at hendelsen er lagret. Sammenlikningen normaliserer med `catenda_id`. Går på tvers av lagene: journalen i PostgreSQL, registeret i SQLite.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>notat</t>
+          <t>leveringsoppdrag</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2922,7 +2987,7 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Skjermingen går på denne verdien; uten den vises notatet til ingen (AGENTS.md). Samme verdiform som `hendelse.actorteam`.</t>
+          <t>Prosjektet brevet er sendt i. Triggeren krever at det er hendelsens prosjekt.</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2999,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2960,24 +3025,24 @@
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Hendelsen notatet kommenterer, om noen.</t>
+          <t>Prosjektet notatet er skrevet i.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>notat</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>app_users</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2998,29 +3063,29 @@
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet saken tilhører. Tilgangskontrollen holder hver forespørsel mot denne verdien.</t>
+          <t>Forfatteren.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>notat</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>app_users</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -3036,29 +3101,29 @@
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Den som opprettet saken. Bare delvis en kobling: verdien har tre former, og bare én av dem er `app_users.id` (MG-04).</t>
+          <t>Teamet som kan lese notatet. Skjermingen går på denne verdien; uten den vises notatet til ingen (AGENTS.md). Samme verdiform som `hendelse.actorteam`.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>notat</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3074,7 +3139,7 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Catenda-prosjektet saken ble opprettet i. Kolonnen er `text`, målet er `uuid`. Levering til Catenda bruker i dag den globale innstillingen, ikke denne verdien (INT-06).</t>
+          <t>Hendelsen notatet kommenterer, om noen.</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3151,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>catenda_board_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>catenda_topic_board_configs</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>topic_board_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3112,29 +3177,29 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Topic boardet sakens topic ligger på. Kolonnen er `text`, målet er `uuid`. Levering til Catenda leser boardet herfra.</t>
+          <t>Prosjektet saken tilhører. Tilgangskontrollen holder hver forespørsel mot denne verdien.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>sak_relations</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>source_sak_id</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>app_users</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3150,29 +3215,29 @@
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Forseringen eller endringsordren som omfatter en annen sak. Fremmednøkkelen mangler (DB-04); hvordan relasjoner skal lagres, er B-01. Opprettes en forsering gjennom `/api/forsering/opprett`, er verdien topicens GUID, og saken har da ingen rad i `sak_metadata`.</t>
+          <t>Den som opprettet saken. Bare delvis en kobling: verdien har tre former, og bare én av dem er `app_users.id` (MG-04).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>sak_relations</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>target_sak_id</t>
+          <t>catenda_project_id</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>catenda_project_id</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3188,29 +3253,29 @@
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>KOE-saken som inngår i forseringen eller endringsordren.</t>
+          <t>Catenda-prosjektet saken ble opprettet i. Kolonnen er `text`, målet er `uuid`. Levering til Catenda bruker i dag den globale innstillingen, ikke denne verdien (INT-06).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>sak_relations</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>catenda_board_id</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>catenda_topic_board_configs</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>topic_board_id</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3226,29 +3291,29 @@
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet relasjonen er skrevet i, stemplet fra autorisert kontekst.</t>
+          <t>Topic boardet sakens topic ligger på. Kolonnen er `text`, målet er `uuid`. Levering til Catenda leser boardet herfra.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>app_project_memberships</t>
+          <t>sak_relations</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>catenda_subject</t>
+          <t>source_sak_id</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>app_identities</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>subject</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3264,29 +3329,29 @@
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Personen i Catenda. `koe_reconcile_memberships` løser subjektet til `user_id` gjennom `koe_resolve_identity`, så de to kolonnene peker på samme person. Kontraktssiden slås opp med subjektet.</t>
+          <t>Forseringen eller endringsordren som omfatter en annen sak. Fremmednøkkelen mangler (DB-04); hvordan relasjoner skal lagres, er B-01. Opprettes en forsering gjennom `/api/forsering/opprett`, er verdien topicens GUID, og saken har da ingen rad i `sak_metadata`.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>app_membership_sync</t>
+          <t>sak_relations</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_id</t>
+          <t>target_sak_id</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3296,20 +3361,20 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Catenda-prosjektet synkroniseringen hentet fra. `ensure_fresh` godtar bare en synkronisering av prosjektets nåværende Catenda-prosjekt.</t>
+          <t>KOE-saken som inngår i forseringen eller endringsordren.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>catenda_models_cache</t>
+          <t>sak_relations</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3340,29 +3405,29 @@
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet modellene gjelder. BIM-rutene slår opp på denne. Tabellen fylles ikke (DM-02).</t>
+          <t>Prosjektet relasjonen er skrevet i, stemplet fra autorisert kontekst.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>catenda_models_cache</t>
+          <t>app_project_memberships</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_id</t>
+          <t>catenda_subject</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_configs</t>
+          <t>app_identities</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>catenda_project_id</t>
+          <t>subject</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -3378,29 +3443,29 @@
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Catenda-prosjektet modellene ligger i. Kolonnen er `text`, målet er `uuid`.</t>
+          <t>Personen i Catenda. `koe_reconcile_memberships` løser subjektet til `user_id` gjennom `koe_resolve_identity`, så de to kolonnene peker på samme person. Kontraktssiden slås opp med subjektet.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>utkast</t>
+          <t>app_membership_sync</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>catenda_project_id</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>catenda_project_id</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -3410,35 +3475,35 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet utkastet er skrevet i.</t>
+          <t>Catenda-prosjektet synkroniseringen hentet fra. `ensure_fresh` godtar bare en synkronisering av prosjektets nåværende Catenda-prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>utkast</t>
+          <t>catenda_models_cache</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>case_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -3454,29 +3519,29 @@
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Saken utkastet gjelder.</t>
+          <t>Prosjektet modellene gjelder. BIM-rutene slår opp på denne. Tabellen fylles ikke (DM-02).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>utkast</t>
+          <t>catenda_models_cache</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>team</t>
+          <t>catenda_project_id</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>catenda_project_configs</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>catenda_project_id</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -3492,14 +3557,14 @@
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Teamet som eier utkastet. Uten entydig team finnes det ikke noe utkast. Samme verdiform som `hendelse.actorteam`.</t>
+          <t>Catenda-prosjektet modellene ligger i. Kolonnen er `text`, målet er `uuid`.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>approvals</t>
+          <t>utkast</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3530,14 +3595,14 @@
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet godkjenningen hører til.</t>
+          <t>Prosjektet utkastet er skrevet i.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>approvals</t>
+          <t>utkast</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3562,35 +3627,35 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Saken. Ett dokument per prosjekt og sak.</t>
+          <t>Saken utkastet gjelder.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>approvals</t>
+          <t>utkast</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>body → items[].claimId</t>
+          <t>team</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -3606,7 +3671,7 @@
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Kravet en forberedt svarpost gjelder. Posten er ugyldig om et nyere krav eller en tilbaketrekking er kommet i sporet. Ved publisering blir verdien `refererer_til_event_id` i svaret.</t>
+          <t>Teamet som eier utkastet. Uten entydig team finnes det ikke noe utkast. Samme verdiform som `hendelse.actorteam`.</t>
         </is>
       </c>
     </row>
@@ -3618,17 +3683,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>body → packages[].eventIds[]</t>
+          <t>project</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -3638,35 +3703,35 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>mange til mange</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Hendelsene en publisert pakke ble til i journalen.</t>
+          <t>Prosjektet godkjenningen hører til.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>approval_outbox</t>
+          <t>approvals</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>approvals</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>body → packages[].id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -3682,29 +3747,29 @@
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Pakken varslingsjobben gjelder. Én jobb per pakke.</t>
+          <t>Saken. Ett dokument per prosjekt og sak.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>approval_outbox</t>
+          <t>approvals</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>body → items[].claimId</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -3720,29 +3785,29 @@
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet.</t>
+          <t>Kravet en forberedt svarpost gjelder. Posten er ugyldig om et nyere krav eller en tilbaketrekking er kommet i sporet. Ved publisering blir verdien `refererer_til_event_id` i svaret.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>approval_outbox</t>
+          <t>approvals</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>case_id</t>
+          <t>body → packages[].eventIds[]</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>hendelse</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3752,35 +3817,35 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>mange til mange</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Saken.</t>
+          <t>Hendelsene en publisert pakke ble til i journalen.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>eo_approvals</t>
+          <t>approval_outbox</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>approvals</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>body → packages[].id</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -3796,29 +3861,29 @@
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet. Ett dokument per prosjekt med alle endringsordrene til godkjenning.</t>
+          <t>Pakken varslingsjobben gjelder. Én jobb per pakke.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>eo_approvals</t>
+          <t>approval_outbox</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>body → packages[].sakId</t>
+          <t>project</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>sak_metadata</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -3828,25 +3893,25 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Saks-ID-en endringsordren er reservert under. Saken finnes først når ordren er utstedt; fram til da peker verdien på en sak som ikke finnes.</t>
+          <t>Prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>eo_approvals</t>
+          <t>approval_outbox</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>body → packages[].request.koe_sak_ids[]</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3866,20 +3931,20 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>mange til mange</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>KOE-sakene endringsordren skal omfatte.</t>
+          <t>Saken.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>vedlegg</t>
+          <t>eo_approvals</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3904,25 +3969,25 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet.</t>
+          <t>Prosjektet. Ett dokument per prosjekt med alle endringsordrene til godkjenning.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>vedlegg</t>
+          <t>eo_approvals</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>case_id</t>
+          <t>body → packages[].sakId</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3942,35 +4007,35 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Saken vedlegget er lastet opp i. Nedlasting krever at vedlegget står på nøyaktig denne saken.</t>
+          <t>Saks-ID-en endringsordren er reservert under. Saken finnes først når ordren er utstedt; fram til da peker verdien på en sak som ikke finnes.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>vedlegg</t>
+          <t>eo_approvals</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_team</t>
+          <t>body → packages[].request.koe_sak_ids[]</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>sak_metadata</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3980,20 +4045,20 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>mange til mange</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Teamet som lastet opp. Et vedlegg som ikke er sendt, er synlig bare for dette teamet. Samme verdiform som `hendelse.actorteam`.</t>
+          <t>KOE-sakene endringsordren skal omfatte.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>catenda_delivery_status</t>
+          <t>vedlegg</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4031,7 +4096,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>catenda_delivery_status</t>
+          <t>vedlegg</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4062,29 +4127,29 @@
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Saken banneret vises på.</t>
+          <t>Saken vedlegget er lastet opp i. Nedlasting krever at vedlegget står på nøyaktig denne saken.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>catenda_delivery_status</t>
+          <t>vedlegg</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>lastet_opp_team</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>hendelse</t>
+          <t>catenda_contract_teams</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -4094,11 +4159,125 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som lastet opp. Et vedlegg som ikke er sendt, er synlig bare for dette teamet. Samme verdiform som `hendelse.actorteam`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>catenda_delivery_status</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>projects</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>catenda_delivery_status</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>case_id</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>sak_metadata</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Saken banneret vises på.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>catenda_delivery_status</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>hendelse</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>Hendelsen kvitteringen gjelder. Kvitteringen skrives før hendelsen lagres; ved lesing teller bare kvitteringer for hendelser som finnes i journalen.</t>
         </is>

</xml_diff>

<commit_message>
rett PostgreSQL-forutsetningene i hovedplanen etter B-12, databasen, og B-19, og bytt ordet i B-13
Ordbyttet i B-13 og datamodellregistrene følger HF-U2 (#384). Radetiketten i
regler.json følger når #394 er merget.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmiNVm7sTS6jf2L3KkJp91
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>TE trekker ansvarsgrunnlaget, og med det kravene i saken.</t>
+          <t>TE trekker grunnlaget, og med det kravene i saken.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -8021,7 +8021,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>BH svarer på ansvarsgrunnlaget: godkjent, avslått eller frafalt pålegg, og om grunnlaget er varslet i tide.</t>
+          <t>BH svarer på grunnlaget: godkjent, avslått eller frafalt pålegg, og om grunnlaget er varslet i tide.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>BH endrer sitt svar på ansvarsgrunnlaget («snuoperasjon»).</t>
+          <t>BH endrer sitt svar på grunnlaget («snuoperasjon»).</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
før tabellene i SQL Server inn i datamodellregistrene
`SQL Server` er en ny lagring i `docs/verktoy/datamodell.py`, og katalog.json
får en del `sqlserver` med navn kvalifisert med skjemaet (`koe.app_users`).
Delen leses av `server/tester/katalog.ts` i en base runneren bygger fra
`database/migrasjoner/`, og `katalog.py` kjører den. `katalog.test.ts` holder
delen lik katalogen i CI-jobben `sqlserver`, og pytest-vaktene sammenlikner
registeret og katalog.json med `CREATE TABLE` i migrasjonene.

Closes #558

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017gWLQ6vS7pNq8wEBjdsx5F
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1983,6 +1983,576 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Én rad per person. `id` er aktøren i journalen og notatet (AGENTS.md). Svarer til `app_users` i PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en identitet sees.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Delvis. Navn og e-post kommer fra Catenda-identiteten. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>grunndata</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Navn og e-post.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_identities</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Identitetene til en bruker, unike på leverandør, issuer og subjekt. En Catenda-identitet har issueren og subjektformen basen kontrollerer, så samme person ikke får to brukerrader (AGENTS.md).</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>`koe.resolve_identity`, sammen med brukeren.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Ja, for leverandøren `catenda`: subjektet er Catenda-ID-en. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: app_identities.user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>grunndata</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Subjektet identifiserer en person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>koe.projects</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektene. `id` er prosjektgrensen i alle tabellene med saksdata, uten standardverdi (AGENTS.md).</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>ikke kontrollert Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>grunndata</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_project_memberships</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Delvis</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Ja, medlemslisten i Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: app_project_memberships.project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); app_project_memberships.user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>grunndata, kopi</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>E-post og visningsnavn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes i appen. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: catenda_contract_teams.internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel).</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>grunndata</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: sak_metadata.prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); sak_metadata.created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>`created_by` peker på en bruker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: hendelse.sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); hendelse.prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); hendelse.aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); hendelse.aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); hendelse.refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.event_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: notat.sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); notat.prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); notat.aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); notat.aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); notat.refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>koe.leveringsoppdrag</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: leveringsoppdrag.event_id → koe.hendelse.event_id (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag.sak_id → koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag.prosjekt_id → koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: kjernebuffer.sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); kjernebuffer.prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>avledet</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Som journalen den er regnet fra.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1994,7 +2564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4280,6 +4850,872 @@
       <c r="H58" s="2" t="inlineStr">
         <is>
           <t>Hendelsen kvitteringen gjelder. Kvitteringen skrives før hendelsen lagres; ved lesing teller bare kvitteringer for hendelser som finnes i journalen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_identities</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Brukeren identiteten hører til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_project_memberships</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>project_id</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>koe.projects</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet medlemskapet gjelder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_project_memberships</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Brukeren som er medlem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>internal_project_id</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>koe.projects</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet teamet er knyttet til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>koe.projects</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Brukeren som opprettet saken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>aktor_id</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>aktor_id</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Forfatteren, `app_users.id`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>koe.leveringsoppdrag</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Brevet oppdraget leverer. Unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>koe.leveringsoppdrag</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Saken, i den sammensatte nøkkelen mot brevet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>koe.leveringsoppdrag</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet, i den sammensatte nøkkelen mot brevet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>sak_id</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Saken bufferen er regnet for. Primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
rett kolonnenavnet i etikettene for tabellene i SQL Server
`partition('.')` delte ved første punktum, så etiketten i ER-diagrammet og
«Viser til» i tabellbeskrivelsen fikk med tabellnavnet for `koe.*`. Feilmeldingene
som viser til katalog.py, nevner nå begge variablene den krever.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmKxDdmp7yqXq9cSfFWzxu
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2073,7 +2073,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: app_identities.user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: app_project_memberships.project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); app_project_memberships.user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: catenda_contract_teams.internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: sak_metadata.prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); sak_metadata.created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: hendelse.sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); hendelse.prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); hendelse.aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); hendelse.aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); hendelse.refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.event_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.event_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: notat.sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); notat.prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); notat.aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); notat.aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); notat.refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: leveringsoppdrag.event_id → koe.hendelse.event_id (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag.sak_id → koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag.prosjekt_id → koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: event_id → koe.hendelse.event_id (fremmednøkkel, ON DELETE NO ACTION); sak_id → koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: kjernebuffer.sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); kjernebuffer.prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">

</xml_diff>

<commit_message>
sett koe.app_users og koe.app_identities til «uavklart»
Ingen inngang i server/ kaller `koe_api.catenda_identitet` ennå, så de to
tabellene har ingen skriver i appen, som de åtte andre (#53, del 3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BmKxDdmp7yqXq9cSfFWzxu
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en identitet sees.</t>
+          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en identitet sees. Ingen inngang i `server/` kaller den ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, sammen med brukeren.</t>
+          <t>`koe.resolve_identity`, sammen med brukeren. Ingen inngang i `server/` kaller den ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">

</xml_diff>

<commit_message>
før basens tidspunkt for transaksjonen i en tabell og godta bare det (DL-U3)
Grensen på 60 s faller bort. koe_api.skrivetidspunkt fører tidspunktet i
koe.skrivetidspunkt med transaksjonens ID som nøkkel, og skriv_hendelse godtar
bare det og sletter raden. Registrene i docs/datamodell kjenner tabellen og
skriverne for sak_metadata, hendelse og leveringsoppdrag.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WEQkdszCKkjDTn5TgPXoYU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. Ingen HTTP-inngang kaller dem ennå (#53).</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2499,55 +2499,112 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>koe.skrivetidspunkt</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med transaksjonens ID som nøkkel. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (transaksjon). Ingen relasjoner til andre tabeller.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>koe.kjernebuffer</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (sak_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>avledet</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>uavklart</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Som journalen den er regnet fra.</t>
         </is>

</xml_diff>

<commit_message>
bind tidspunktet til økta, så en rad fra før en omstart ikke kan brukes
CURRENT_TRANSACTION_ID() begynner på nytt etter en omstart. Raden i
koe.skrivetidspunkt gjelder nå også økta og når den logget inn, og
skriv_hendelse godtar den bare i samme økt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WEQkdszCKkjDTn5TgPXoYU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med transaksjonens ID som nøkkel. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med transaksjonens ID som nøkkel, og økta og når den logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` sletter den når transaksjons-ID-en brukes igjen.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">

</xml_diff>

<commit_message>
bruk økt-ID-en som nøkkel i koe.skrivetidspunkt, så en skriving bare leser og låser sin egen rad
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WEQkdszCKkjDTn5TgPXoYU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med transaksjonens ID som nøkkel, og økta og når den logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` sletter den neste gang samme økt-ID eller transaksjons-ID fører et tidspunkt.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (transaksjon). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">

</xml_diff>

<commit_message>
synkroniser medlemslisten i SQL Server og før DL-U8 (#53, del 3b)
Ny migrasjon med koblingen til Catenda-prosjektet, tidspunktet for
medlemslisten og prosedyren som skriver den, med en smal lesing av
listens alder. server/medlemskap.ts kaller prosedyrene, og testene
kjører mot SQL Server. DL-U8 er ført i vedtaksregisteret.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Z8zGnu6QfHdrA5LVtMQGh
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `deactivated_at` er når medlemskapet sist ble gjort inaktivt; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). Ingen inngang kaller modulen ennå.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -2271,37 +2271,37 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_project_configs</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Settes av driften. Ingen prosedyre skriver tabellen.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. ID-en til Catenda-prosjektet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2311,54 +2311,54 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>`created_by` peker på en bruker.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4). Svarer til `app_membership_sync` i PostgreSQL.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`. Ingen inngang kaller modulen ennå.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. Ingen HTTP-inngang kaller dem ennå (#53).</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.event_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2378,19 +2378,19 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2430,24 +2430,24 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
+          <t>`created_by` peker på en bruker.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
+          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. Ingen HTTP-inngang kaller dem ennå (#53).</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2467,12 +2467,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: event_id → koe.hendelse.event_id (fremmednøkkel, ON DELETE NO ACTION); sak_id → koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.event_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2492,36 +2492,36 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2539,72 +2539,186 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>koe.leveringsoppdrag</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: event_id → koe.hendelse.event_id (fremmednøkkel, ON DELETE NO ACTION); sak_id → koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>koe.skrivetidspunkt</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>koe.kjernebuffer</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (sak_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>avledet</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>uavklart</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Som journalen den er regnet fra.</t>
         </is>
@@ -2621,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5039,7 +5153,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.catenda_project_configs</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -5064,7 +5178,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -5074,19 +5188,19 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet teamet er knyttet til.</t>
+          <t>Prosjektet i appen som er koblet til Catenda-prosjektet. Settes av driften (arbeidsvalget 16.10 i #53).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>project_id</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5106,7 +5220,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -5116,24 +5230,24 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
+          <t>Prosjektet medlemslisten ble skrevet for (DL-U7).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -5158,29 +5272,29 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Brukeren som opprettet saken.</t>
+          <t>Prosjektet teamet er knyttet til.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -5200,29 +5314,29 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
+          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -5242,7 +5356,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+          <t>Brukeren som opprettet saken.</t>
         </is>
       </c>
     </row>
@@ -5254,17 +5368,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -5284,19 +5398,19 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
+          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5306,7 +5420,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -5326,29 +5440,29 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`.</t>
+          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -5368,7 +5482,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -5380,17 +5494,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -5410,29 +5524,29 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Forfatteren, `app_users.id`.</t>
+          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -5442,7 +5556,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -5452,29 +5566,29 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Brevet oppdraget leverer. Unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`.</t>
+          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -5494,7 +5608,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Saken, i den sammensatte nøkkelen mot brevet.</t>
+          <t>Forfatteren, `app_users.id`.</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5620,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -5516,7 +5630,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -5526,7 +5640,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -5536,14 +5650,14 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot brevet.</t>
+          <t>Brevet oppdraget leverer. Unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5553,7 +5667,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -5568,7 +5682,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -5578,14 +5692,14 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. Primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Saken, i den sammensatte nøkkelen mot brevet.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5595,7 +5709,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -5620,72 +5734,76 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+          <t>Prosjektet, i den sammensatte nøkkelen mot brevet.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken bufferen er regnet for. Primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -5693,17 +5811,21 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -5734,14 +5856,14 @@
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -5771,6 +5893,82 @@
       </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
regenerer tabeller.md og tabellbeskrivelse.xlsx etter de sammensatte nøklene (#590)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019gQrntcR5RouGDL4UdzGdG
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2415,7 +2415,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.event_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.sak_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: event_id → koe.hendelse.event_id (fremmednøkkel, ON DELETE NO ACTION); sak_id → koe.hendelse.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.hendelse.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: sak_id → koe.sak_metadata.sak_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_id → koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -5410,17 +5410,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -5440,29 +5440,29 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
+          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`, så notatet står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
@@ -5494,17 +5494,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -5524,29 +5524,29 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`.</t>
+          <t>Forfatteren, `app_users.id`.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -5556,7 +5556,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -5566,29 +5566,29 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
+          <t>Brevet oppdraget leverer. `event_id` er unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`, så oppdraget står i brevets sak og prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -5608,61 +5608,57 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Forfatteren, `app_users.id`.</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr"/>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Brevet oppdraget leverer. Unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -5672,12 +5668,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -5685,41 +5681,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Saken, i den sammensatte nøkkelen mot brevet.</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -5727,248 +5719,46 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot brevet.</t>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>Saken bufferen er regnet for. Primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>koe.kjernebuffer</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>prosjekt_id</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>koe.sak_metadata</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>prosjekt_id</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>Prosjektet, i den sammensatte nøkkelen mot saken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>koe.hendelse</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>aktor_team_id</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>koe.catenda_contract_teams</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>team_id</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Uten fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>koe.hendelse</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>refererer_til_event_id</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>koe.hendelse</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>event_id</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>Uten fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="inlineStr"/>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>koe.notat</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>aktor_team_id</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>koe.catenda_contract_teams</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>team_id</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>Uten fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr"/>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>koe.notat</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>refererer_til_event_id</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>koe.hendelse</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>event_id</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>Uten fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G81" s="2" t="inlineStr"/>
-      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
før innloggingens fravær per prosjekt, så en eldre medlemsliste ikke gir nytt medlemskap (DL-U9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxqLpccMARhdp6s6uM5ajt
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). Ingen inngang kaller modulen ennå.</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Ingen inngang kaller modulen ennå.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2328,12 +2328,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_sync</t>
+          <t>koe.app_membership_absences</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4). Svarer til `app_membership_sync` i PostgreSQL.</t>
+          <t>Prosjektene der innloggingens liste over brukerens Catenda-prosjekter viste at brukeren ikke er med, for en bruker uten medlemskap der (DL-U9). `observed_at` er når innloggingens liste ble hentet, etter basens klokke. En medlemsliste hentet samtidig eller før gir ikke brukeren et nytt medlemskap. Har ingen tabell i PostgreSQL.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`. Ingen inngang kaller modulen ennå.</t>
+          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Ingen inngang kaller modulen ennå.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id, user_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2385,37 +2385,37 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4). Svarer til `app_membership_sync` i PostgreSQL.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`. Ingen inngang kaller modulen ennå.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2435,19 +2435,19 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>`created_by` peker på en bruker.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. Ingen HTTP-inngang kaller dem ennå (#53).</t>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2492,19 +2492,19 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
+          <t>`created_by` peker på en bruker.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
+          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. Ingen HTTP-inngang kaller dem ennå (#53).</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2544,24 +2544,24 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
+          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2601,49 +2601,49 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2663,62 +2663,119 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>koe.skrivetidspunkt</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>koe.kjernebuffer</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>avledet</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>uavklart</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Som journalen den er regnet fra.</t>
         </is>
@@ -2735,7 +2792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5195,7 +5252,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_sync</t>
+          <t>koe.app_membership_absences</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5220,7 +5277,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -5230,24 +5287,24 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet medlemslisten ble skrevet for (DL-U7).</t>
+          <t>Prosjektet innloggingen viste at brukeren ikke er med i (DL-U9).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_membership_absences</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>internal_project_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -5272,19 +5329,19 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet teamet er knyttet til.</t>
+          <t>Brukeren som logget inn.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>project_id</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5304,7 +5361,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -5314,24 +5371,24 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
+          <t>Prosjektet medlemslisten ble skrevet for (DL-U7).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5356,29 +5413,29 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Brukeren som opprettet saken.</t>
+          <t>Prosjektet teamet er knyttet til.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -5398,19 +5455,19 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
+          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5440,14 +5497,14 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
+          <t>Brukeren som opprettet saken.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -5482,14 +5539,14 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`, så notatet står i sakens prosjekt.</t>
+          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5524,29 +5581,29 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Forfatteren, `app_users.id`.</t>
+          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -5556,7 +5613,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -5566,29 +5623,29 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Brevet oppdraget leverer. `event_id` er unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`, så oppdraget står i brevets sak og prosjekt.</t>
+          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`, så notatet står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -5598,7 +5655,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -5608,90 +5665,98 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Forfatteren, `app_users.id`.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
+          <t>koe.leveringsoppdrag</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>(event_id, sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
           <t>koe.hendelse</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>aktor_team_id</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>koe.catenda_contract_teams</t>
-        </is>
-      </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Brevet oppdraget leverer. `event_id` er unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`, så oppdraget står i brevets sak og prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5722,14 +5787,14 @@
       <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -5759,6 +5824,82 @@
       </c>
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
legg sesjonen og innloggingsforsøket i SQL Server
Tabellene koe.app_sessions og koe.app_oauth_attempts med prosedyrene i
koe_api for å opprette, lese, slette og bruke dem og rydde utløpte, og
server/sesjon.ts som kaller dem (B-19, #656). Basen lagrer bare SHA-256
av tokenene, og kjøretiden har bare EXECUTE på prosedyrene.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ggs6bQ2GYUY8kyn76e7jRk
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2778,6 +2778,120 @@
       <c r="K41" s="2" t="inlineStr">
         <is>
           <t>Som journalen den er regnet fra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`; ingen HTTP-inngang kaller modulen ennå (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_oauth_attempts</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`; ingen HTTP-inngang kaller modulen ennå (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5336,17 +5450,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_sync</t>
+          <t>koe.app_sessions</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>project_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -5361,7 +5475,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -5371,19 +5485,19 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet medlemslisten ble skrevet for (DL-U7).</t>
+          <t>Brukeren sesjonen er logget inn som.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>internal_project_id</t>
+          <t>project_id</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -5403,7 +5517,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -5413,19 +5527,19 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet teamet er knyttet til.</t>
+          <t>Prosjektet medlemslisten ble skrevet for (DL-U7).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>internal_project_id</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5455,7 +5569,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
+          <t>Prosjektet teamet er knyttet til.</t>
         </is>
       </c>
     </row>
@@ -5467,12 +5581,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -5497,29 +5611,29 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Brukeren som opprettet saken.</t>
+          <t>Prosjektet saken hører til, uten standardverdi (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -5539,7 +5653,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
+          <t>Brukeren som opprettet saken.</t>
         </is>
       </c>
     </row>
@@ -5551,17 +5665,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -5581,29 +5695,29 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
+          <t>Saken brevet hører til. Sammensatt med `prosjekt_id`, så brevet står i sakens prosjekt. Kaskaderer ikke.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -5623,7 +5737,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`, så notatet står i sakens prosjekt.</t>
+          <t>Avsenderen, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -5635,17 +5749,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -5665,29 +5779,29 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Forfatteren, `app_users.id`.</t>
+          <t>Saken notatet er skrevet i. Sammensatt med `prosjekt_id`, så notatet står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -5697,7 +5811,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -5707,29 +5821,29 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Brevet oppdraget leverer. `event_id` er unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`, så oppdraget står i brevets sak og prosjekt.</t>
+          <t>Forfatteren, `app_users.id`.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -5749,45 +5863,49 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Brevet oppdraget leverer. `event_id` er unik, så hvert brev har ett oppdrag. Sammensatt med `sak_id` og `prosjekt_id`, så oppdraget står i brevets sak og prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
@@ -5799,17 +5917,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -5825,29 +5943,29 @@
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -5863,7 +5981,7 @@
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
@@ -5875,17 +5993,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -5900,6 +6018,44 @@
       </c>
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
mål returstien i UTF-16-enheter og rund ikke ryddeklokka fram
Funn fra /code-review high i reviewøkta for #683: LEN slapp gjennom en
retursti over 2048 enheter med mellomrom til slutt eller tegn utenfor BMP,
og ryddingen kunne slette en sesjon les_sesjon ennå godtok. Registeret
nevner innloggingstidspunktet som personopplysning.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yDYgktsVRmuhKpCSm1fdZ
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -1067,7 +1067,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`.</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med tidspunktet for innloggingen (`created_at`, `expires_at`).</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`.</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med tidspunktet for innloggingen (`created_at`, `expires_at`).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
avkort utløpet til millisekundet og send returstien uten driverens grense
Funn fra kontrollen av rettingene i #683: en retursti over 4000 enheter
feilet i driveren i stedet for i basens kontroll, og utløpet ble rundet
opp i stedet for avkortet som tidspunktene i kommandoene. Grensetester
for en godtatt sti på 2048 enheter.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yDYgktsVRmuhKpCSm1fdZ
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -1067,7 +1067,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med tidspunktet for innloggingen (`created_at`, `expires_at`).</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med tidspunktet for innloggingen (`created_at`, `expires_at`).</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
før tilgangsoppslagene i registeret for medlemskapstabellene
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RTXiK5H5KPCic6HHJFKsa7
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL.</t>
+          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658).</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen.</t>
+          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen. `server/autorisasjon.ts` leser prosjektets kontraktsteam med `koe_api.kontraktsteam`, bare for en aktør med aktivt medlemskap uten leserollen (#658).</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt.</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/autorisasjon.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658).</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4). Svarer til `app_membership_sync` i PostgreSQL.</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2). Svarer til `app_membership_sync` i PostgreSQL.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">

</xml_diff>

<commit_message>
legg innloggingsinngangene til i TS-serveren
Login, tilbakekall, sesjon, utlogging og CSRF-token med samme stier, svar
og kapsler som Python. Tilbakekallet løser identiteten gjennom
koe_api.catenda_identitet og oppretter ingen sesjon når den ikke kan
avgjøres. Registeret får inngangene uten sesjon og uten prosjekt, med
begrunnelse og lukkede lister i testen.

Closes #659

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CBNM2dUxfPacrv8rpS5sjj
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en identitet sees. Ingen inngang i `server/` kaller den ennå (#53, del 3).</t>
+          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, sammen med brukeren. Ingen inngang i `server/` kaller den ennå (#53, del 3).</t>
+          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`; ingen HTTP-inngang kaller modulen ennå (F0b-5a, #659).</t>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`; ingen HTTP-inngang kaller modulen ennå (F0b-5a, #659).</t>
+          <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">

</xml_diff>

<commit_message>
start TS-serveren med Catenda fra miljøet og kontroll av migrasjonene, og send innloggingen og prosjektene dit fra vite
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012yx1ERUmwrUQ7Cs8Gf673K
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Ingen inngang kaller modulen ennå.</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10).</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/autorisasjon.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658).</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10). Den tomme Catenda-ID-en er ikke lov; den merker synkroniseringsraden etter en slik endring.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Ingen inngang kaller modulen ennå.</t>
+          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Innloggingen kaller modulen fra tilbakekallet i `server/innlogging.ts` (F0b-5b).</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2). Svarer til `app_membership_sync` i PostgreSQL.</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden den tomme Catenda-ID-en og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10).</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`. Ingen inngang kaller modulen ennå.</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, og triggeren `koe.catenda_project_configs_kobling_endret` når koblingen endres.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">

</xml_diff>

<commit_message>
før lesingen fra prosjektinngangene i registeret for medlemskapet, koblingen og synkroniseringen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012D4TzTeVMXqkaWWFJRQmqm
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658).</t>
+          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660).</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/autorisasjon.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658).</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/autorisasjon.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658). `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660).</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2). Svarer til `app_membership_sync` i PostgreSQL.</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">

</xml_diff>

<commit_message>
flytt journalen og leveringsoppdraget for kommandoinngangene til SQL Server, og ta pg ut av server/
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qj48eobHTRCFNxrhabuiAU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. Ingen HTTP-inngang kaller dem ennå (#53).</t>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661); ingen HTTP-inngang oppretter saker ennå (#370).</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
+          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661).</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">

</xml_diff>

<commit_message>
legg sakens topic i Catenda i en egen tabell, og krev bibliotek i koblingen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qj48eobHTRCFNxrhabuiAU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2670,12 +2670,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661).</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2685,22 +2685,22 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Ingen prosedyre skriver den ennå (#370, #371).</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2710,29 +2710,29 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2767,29 +2767,29 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2824,72 +2824,129 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -2906,7 +2963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5870,7 +5927,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5905,45 +5962,49 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
@@ -5955,17 +6016,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -5981,29 +6042,29 @@
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -6019,7 +6080,7 @@
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
@@ -6031,17 +6092,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -6056,6 +6117,44 @@
       </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
rett skriverne av journalen og oppdraget i PostgreSQL i tabellregisteret
server/lager.ts skriver ikke lenger i PostgreSQL, så hendelse mister skriveren
og leveringsoppdrag i PostgreSQL blir rest. Tilgangsreglene sier hvor låsen og
prosjektkontrollen i skrivingen ligger (review av #738).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014PDAEC33vXpuRFU1eu64bP
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Leveringsoppdraget for et brev TS-serveren skriver (LV-U1, B-03, dokumentet). Én rad per brev, og ett brev er ett dokument i Catenda. `innhold` fryser det som skal leveres: brevet slik det ble lagret, målet i Catenda, statusetiketten og versjonene. Raden er uforanderlig; et nytt leveringsforsøk sender samme innhold. Et lagret oppdrag beviser ikke at brevet er sendt eller mottatt. Forsøk, feil og kvitteringer er ikke bygget (#371). Bare testmiljøet skriver tabellen (#347).</t>
+          <t>Leveringsoppdraget for et brev TS-serveren skriver (LV-U1, B-03, dokumentet). Én rad per brev, og ett brev er ett dokument i Catenda. `innhold` fryser det som skal leveres: brevet slik det ble lagret, målet i Catenda, statusetiketten og versjonene. Raden er uforanderlig; et nytt leveringsforsøk sender samme innhold. Et lagret oppdrag beviser ikke at brevet er sendt eller mottatt. Forsøk, feil og kvitteringer er ikke bygget (#371). Ingen skriver tabellen lenger: TS-serveren skriver oppdraget i `koe.leveringsoppdrag` i SQL Server (F0b-7, #661).</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Når TS-serveren lagrer et brev: i samme transaksjon som hendelsen i `hendelse`. Slettes bare med saken eller hendelsen (kaskade).</t>
+          <t>Ingen steder etter F0b-7 (#661). Fram til da skrev TS-serveren oppdraget i samme transaksjon som hendelsen i `hendelse`. Slettes bare med saken eller hendelsen (kaskade).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>rest</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
legg til inngangen som oppretter en KOE-sak, og avvis BH også i skrivelaget
Closes #370

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMf9Vi59xgT9G8A2fM4BWK
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`. Ingen HTTP-inngang kaller den ennå (#53).</t>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370).</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661); ingen HTTP-inngang oppretter saker ennå (#370).</t>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661), og `koe_api.opprett_sak` fra `POST /api/kjerne/saker` (#370).</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Ingen prosedyre skriver den ennå (#370, #371).</t>
+          <t>Ingen prosedyre skriver den ennå (#741, #371).</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">

</xml_diff>

<commit_message>
lever brevet til Catenda med leveringsforsøk og en kvittering per operasjon
Leveringsoppdraget får en jobb av typen levering i samme transaksjon som
brevet. Kjøreren laster opp dokumentet med dokumentnøkkelen i navnet og
failOnDocumentExists, setter referansen på topicen og kvitterer hver
operasjon for seg. Hvert steg avstemmes først mot Catenda (B-03).

Tar også punkter fra #778: varig avvisning og ukjent jobbtype parkeres som
avvist, tidsavbrudd ved tilkobling og TLS-feil regnes som ikke sendt,
omstarten nullstiller antall forsøk, leasekontrollen står ett sted, den
ene UsikkertUtfall heter nå UsikkertCatendautfall, og testbasen gir
kjøreveien rettigheter bare mens en testsetning kjører.

Del av #371. Del av #778.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TVMWuj5SeWT72tkipmuCHa
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2618,7 +2618,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
+          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak`, og endres av `koe_api.hent_jobb`, `koe_api.kvitter_topic`, `koe_api.registrer_jobbfeil` og driftsverktøyet `koe_api.start_jobb_paa_nytt`.</t>
+          <t>`koe_api.opprett_sak` og triggeren `koe.leveringsoppdrag_levering`, og endres av `koe_api.hent_jobb`, `koe_api.kvitter_topic`, `koe_api.kvitter_levering`, `koe_api.registrer_jobbfeil` og driftsverktøyet `koe_api.start_jobb_paa_nytt`.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `kobling_endret` eller `startet_paa_nytt`, med innloggingen som startet jobben på nytt. Raden endres ikke.</t>
+          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med innloggingen som startet jobben på nytt. Raden endres ikke.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobb.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2784,29 +2784,29 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2824,12 +2824,12 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -2841,12 +2841,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2856,22 +2856,22 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2881,29 +2881,29 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2938,29 +2938,29 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2995,72 +2995,129 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3077,7 +3134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6167,22 +6224,22 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.jobb</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>leveringsoppdrag_id</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -6202,29 +6259,29 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Oppdraget en jobb `levering` leverer (#371). Hvert oppdrag har høyst én jobb.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>leveringsoppdrag_id</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -6234,7 +6291,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -6244,67 +6301,71 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(leveringsoppdrag_id, forutsetning)</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(leveringsoppdrag_id, operasjon)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Referansen på topicen forutsetter at dokumentet er kvittert for samme oppdrag.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -6320,81 +6381,241 @@
       <c r="G81" s="2" t="inlineStr"/>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Leasen kvitteringen ble skrevet med. Forsøket med samme ID lagres når forsøket er over, etter kvitteringen for dokumentet, så det er ingen fremmednøkkel.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
           <t>koe.notat</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>refererer_til_event_id</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>koe.hendelse</t>
         </is>
       </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>event_id</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E87" s="2" t="inlineStr">
         <is>
           <t>Uten fremmednøkkel</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr"/>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
lagre en kvittering per kommando i samme transaksjon som brevet
Klienten gir hver kommando en kommando_id. koe_api.skriv_hendelse og
koe_api.opprett_sak lagrer kvitteringen i koe.kvittering, og serveren leser
den med koe_api.kvittering før skrivingen. Samme ID og samme innhold gir
brevet fra kvitteringen, også etter et usikkert utfall av COMMIT; samme ID
med et annet innhold avvises med 422.

Del av #418.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PehjB9kGSJ5wyozWf4egor
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2784,12 +2784,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.kvittering</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen per kommando (invariant 4, #418): kommando-ID-en klienten gir, summen av innholdet serveren regner ut, og saken og brevet kommandoen ga. Lagres i samme transaksjon som brevet. Nøkkelen er prosjektet, aktøren og kommando-ID-en, så kvitteringen gjelder aktøren. Samme ID med samme sum gir brevet fra kvitteringen, og samme ID med en annen sum avvises (51410).</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2834,36 +2834,36 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Aktørens `app_users.id`.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2881,12 +2881,12 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -2898,12 +2898,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2913,22 +2913,22 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2938,29 +2938,29 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2995,29 +2995,29 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3037,12 +3037,12 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3052,72 +3052,129 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3134,7 +3191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6098,27 +6155,27 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>koe.jobb</t>
+          <t>koe.kvittering</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -6126,36 +6183,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G75" s="2" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Saken jobben gjelder. Sammensatt med `prosjekt_id`, så jobben står i sakens prosjekt. En sak har høyst én jobb `catenda_topic` (#741).</t>
+          <t>Aktøren som sendte kommandoen, `app_users.id`. Triggeren `koe.kvittering_samme_transaksjon` krever at den er lik `aktor_id` i brevet, så det er ingen egen fremmednøkkel.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>koe.jobbforsoek</t>
+          <t>koe.kvittering</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>jobb_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>koe.jobb</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>jobb_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -6165,7 +6218,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -6175,7 +6228,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Jobben forsøket gjelder. Fremmednøkkelen hindrer også TRUNCATE av jobbene (#582).</t>
+          <t>Brevet kommandoen ga (#418). `event_id` er unik, så hvert brev har høyst én kvittering. Sammensatt med `sak_id` og `prosjekt_id`, så kvitteringen står i brevets sak og prosjekt.</t>
         </is>
       </c>
     </row>
@@ -6187,17 +6240,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>siste_forsoek</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>koe.jobbforsoek</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>forsoek_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -6207,7 +6260,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -6217,29 +6270,29 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Det siste forsøket på jobben. Fremmednøkkelen hindrer også TRUNCATE av forsøkene (#582).</t>
+          <t>Saken jobben gjelder. Sammensatt med `prosjekt_id`, så jobben står i sakens prosjekt. En sak har høyst én jobb `catenda_topic` (#741).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
+          <t>koe.jobbforsoek</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>jobb_id</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
           <t>koe.jobb</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>leveringsoppdrag_id</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>koe.leveringsoppdrag</t>
-        </is>
-      </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>jobb_id</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -6249,7 +6302,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -6259,29 +6312,29 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget en jobb `levering` leverer (#371). Hvert oppdrag har høyst én jobb.</t>
+          <t>Jobben forsøket gjelder. Fremmednøkkelen hindrer også TRUNCATE av jobbene (#582).</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.jobb</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>leveringsoppdrag_id</t>
+          <t>siste_forsoek</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -6291,7 +6344,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -6301,29 +6354,29 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371).</t>
+          <t>Det siste forsøket på jobben. Fremmednøkkelen hindrer også TRUNCATE av forsøkene (#582).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.jobb</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>(leveringsoppdrag_id, forutsetning)</t>
+          <t>leveringsoppdrag_id</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>(leveringsoppdrag_id, operasjon)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -6343,7 +6396,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Referansen på topicen forutsetter at dokumentet er kvittert for samme oppdrag.</t>
+          <t>Oppdraget en jobb `levering` leverer (#371). Hvert oppdrag har høyst én jobb.</t>
         </is>
       </c>
     </row>
@@ -6355,22 +6408,22 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>forsoek_id</t>
+          <t>leveringsoppdrag_id</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>koe.jobbforsoek</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>forsoek_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -6378,32 +6431,36 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Leasen kvitteringen ble skrevet med. Forsøket med samme ID lagres når forsøket er over, etter kvitteringen for dokumentet, så det er ingen fremmednøkkel.</t>
+          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(leveringsoppdrag_id, forutsetning)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(leveringsoppdrag_id, operasjon)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -6423,132 +6480,136 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Referansen på topicen forutsetter at dokumentet er kvittert for samme oppdrag.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Leasen kvitteringen ble skrevet med. Forsøket med samme ID lagres når forsøket er over, etter kvitteringen for dokumentet, så det er ingen fremmednøkkel.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -6579,14 +6640,14 @@
       <c r="G86" s="2" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -6616,6 +6677,82 @@
       </c>
       <c r="G87" s="2" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
lever brevet som PDF lagret én gang per oppdrag, og la et registrert brev være uten dokument
Del av #371 (L-1c1), #783.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019cnzgz3nZG7Vz3xBqwg4Hr
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.forsoek_id (uten fremmednøkkel); koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobb.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2841,12 +2841,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.brevdokument</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>PDF-en av brevet i et leveringsoppdrag (#371 del 2, merknaden 12.10): bytene og SHA-256 av dem, lagret én gang per oppdrag før første opplasting. Kjøreren har kontrollert at PDF-en gjengir den frosne brevteksten tro (LV-U2), og laster opp den lagrede. Basen regner summen etter. Raden endres ikke, og bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2866,12 +2866,12 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2891,36 +2891,36 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Brevteksten kan ha navn på personer i prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2955,12 +2955,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2970,22 +2970,22 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2995,29 +2995,29 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3052,29 +3052,29 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -3094,12 +3094,12 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3109,72 +3109,129 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3191,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6403,7 +6460,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.brevdokument</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -6428,7 +6485,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -6438,49 +6495,45 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371).</t>
+          <t>Oppdraget PDF-en gjengir. Det er én PDF per oppdrag (#371 del 2).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.brevdokument</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>(leveringsoppdrag_id, forutsetning)</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>(leveringsoppdrag_id, operasjon)</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Referansen på topicen forutsetter at dokumentet er kvittert for samme oppdrag.</t>
+          <t>Leasen PDF-en ble lagret med. Forsøket med samme ID lagres når forsøket er over, så det er ingen fremmednøkkel.</t>
         </is>
       </c>
     </row>
@@ -6492,22 +6545,22 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>forsoek_id</t>
+          <t>leveringsoppdrag_id</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>koe.jobbforsoek</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>forsoek_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -6515,32 +6568,36 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Leasen kvitteringen ble skrevet med. Forsøket med samme ID lagres når forsøket er over, etter kvitteringen for dokumentet, så det er ingen fremmednøkkel.</t>
+          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(leveringsoppdrag_id, forutsetning)</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(leveringsoppdrag_id, operasjon)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -6560,132 +6617,136 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Referansen på topicen forutsetter at dokumentet er kvittert for samme oppdrag.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>forsoek_id</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr"/>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Leasen kvitteringen ble skrevet med. Forsøket med samme ID lagres når forsøket er over, etter kvitteringen for dokumentet, så det er ingen fremmednøkkel.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G86" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -6716,14 +6777,14 @@
       <c r="G88" s="2" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -6753,6 +6814,82 @@
       </c>
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>koe.notat</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>refererer_til_event_id</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>event_id</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>

</xml_diff>

<commit_message>
vis «levert» fra kvitteringen og bygg inn Noto Sans i brev-PDF-en
- lesOppdrag leser kvitteringen for dokumentreferansen, og GET-svaret og
  visningen viser «levert», «ikke levert ennå» eller «sendt utenfor appen»
  (L-1c2, #764, LV-U11)
- brev-PDF-en har Noto Sans (OFL) bygd inn som delmengde med Identity-H,
  og lesBrevPdf dekoder gjennom ToUnicode (#799)
- kjøreren henter en lagret PDF før den lager en ny (#795 punkt 4), og
  avvisningene fra PDF-en er presise (#795 punkt 2, 3 og 5)
- kommandosum bruker sjekksum fra levering.ts (#792 punkt 4)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NabhhAsF1Z8VaevDjtKupx
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2856,7 +2856,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts` når `koe_api.lagret_brevdokument` ikke gir noen PDF for oppdraget (#795 punkt 4).</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
legg til mellomlagring og opplasting av vedlegg i TS-serveren
Del av #790 (V-1): tabellen koe.vedlegg med radsikkerhet, prosedyrene
lagre_vedlegg og slett_vedlegg, og inngangene for opplasting, liste,
nedlasting og sletting under /api/kjerne/saker/<sak>/vedlegg.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3RVW9MNHPRoSa1XNJ6DZY
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel); koe.vedlegg.(bundet_av_event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2898,12 +2898,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. Bindingen kommer i V-2 og slettingen av innholdet etter levering i V-3.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2923,12 +2923,12 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2948,36 +2948,36 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Filen og filnavnet kan ha navn på personer i prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2995,12 +2995,12 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3012,12 +3012,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3027,22 +3027,22 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3052,29 +3052,29 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3109,29 +3109,29 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -3151,12 +3151,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3166,72 +3166,129 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3248,7 +3305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6892,6 +6949,170 @@
       <c r="H91" s="2" t="inlineStr">
         <is>
           <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>koe.vedlegg</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>koe.vedlegg</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>lastet_opp_av</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>koe.vedlegg</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>(event_id, sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>koe.vedlegg</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>lastet_opp_team</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
legg til fullmaktene, godkjenningspakkene og fullmaktsberegningen i TS
Del av #818 (S-1a): migrasjonen med teamvern og radsikkerhet, datalaget i
server/godkjenning.ts, beregningen i server/fullmakt.ts mot kjernens krav og
utregning, testene mot SQL Server og registrene i docs/datamodell.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DugQie7NSvo4MEEqZK7N1
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningshandling.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningspakke.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.godkjenner_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.aktor_team_id (uten fremmednøkkel); koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2955,37 +2955,37 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (runde 7 i #764). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, bruker_id); unik (prosjekt_id, plass). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3005,19 +3005,19 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Hvem som har fullmakt, med tittel og beløpsgrense.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp som fullmaktene.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
+          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3037,12 +3037,12 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3057,49 +3057,49 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -3119,44 +3119,44 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Godkjennerne i en pakke i kjedens rekkefølge, regnet av `server/fullmakt.ts` da pakken ble laget. Endres ikke.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3166,46 +3166,46 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Godkjennerne (`godkjenner_id`).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser tittelen og grensen godkjenneren hadde da den ble gitt, så den står om fullmakten endres senere (B-04 punkt 2). Endres ikke.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3233,62 +3233,347 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
+          <t>koe.leveringskvittering</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>transaksjon</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Nei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_catenda_topic</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>grunndata</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Nei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>koe.skrivetidspunkt</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Ingen kjente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>avledet</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Som journalen den er regnet fra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3305,7 +3590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7113,6 +7398,506 @@
       <c r="H95" s="2" t="inlineStr">
         <is>
           <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>koe.fullmakt</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>koe.projects</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (runde 7 i #764).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>koe.fullmakt</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>bruker_id</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Personen som har fullmakten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>koe.dagmulktssats</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>prosjekt_id</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>koe.projects</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>forrige_pakke_id</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>pakke_id</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>aktor_id</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>godkjenner_id</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Godkjenneren i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>aktor_id</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
lag datamodelleksporten på nytt for medlemsinngangene
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012bnrbeihcVLxYe62LESXDr
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660).</t>
+          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660). `koe_api.medlemmer`, også kalt derfra, leser de aktive medlemmene for en aktør med aktivt medlemskap (#820).</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10).</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10). `koe_api.sett_leserolle`, kalt fra `server/prosjekter.ts`, setter `viewer_override` for et annet aktivt medlem når aktøren er aktiv admin uten leserolle (#820).</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
bind vedleggene i brevet til hendelsen og frys dem i leveringsoppdraget
- `dokumentasjon` i hendelsen er `{vedlegg_id, filnavn, innhold_sha256}`: klienten
  oppgir ID-en, serveren fyller inn filnavn og sum fra mellomlageret (LV-U14)
- `vurder` får vedleggsoppslaget; et vedlegg serveren ikke fant, avvises med
  VEDLEGG_FINNES_IKKE; et registrert varsel krever brevet som vedlegg (OV-U4)
- `koe_api.bind_vedlegg` binder i skrivetransaksjonen, og `koe.vedlegg_uten_endring`
  slipper bare gjennom `bundet_av_event_id` fra NULL; et gjentak binder ikke (KT-U5)
- vedleggene i leveringsoppdraget (OPPDRAGSFORMAT 5), filnavnene i brevteksten
- én eksportert UUID-regex med små bokstaver (#815 punkt 3)
- REGELVERSJON 21, PROJEKSJONSVERSJON 31, feilinnføringene F287–F291

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013iwghGpu4GPmYSrDnR5QCw
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. Bindingen kommer i V-2 og slettingen av innholdet etter levering i V-3.</t>
+          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. `koe_api.bind_vedlegg` binder vedleggene hendelsen viser til, i samme transaksjon som hendelsen (V-2); bindingen er den eneste endringen triggeren `koe.vedlegg_uten_endring` slipper gjennom. Slettingen av innholdet etter levering kommer i V-3.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`.</t>
+          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`, og `koe_api.bind_vedlegg`, kalt fra `server/kommandoer.ts`.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
vis til GFK-U1 i datamodellregistrene
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BeUoEiFvPxprVmxLukSqYw
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (runde 7 i #764). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
+          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (GFK-U1). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (runde 7 i #764).</t>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
legg til driftsskriptet for registreringen og kontraktsteamene i TS
Del av #820 (F-1). Prosedyrene i koe_drift kan bare kjøres av koe_driftsrolle.
Har prosjektet saker, kan kontraktsteamene bare få nye team.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBv5X7Ga3vQaEX9FBeLS4H
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>ikke kontrollert Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Navnet oppgis av driften; i Python kan det hentes fra Catenda-prosjektet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764).</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes i appen. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Settes av driften. Ingen prosedyre skriver tabellen.</t>
+          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet, biblioteket, mappen og boardet og gjør koblingen aktiv.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3354,12 +3354,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3411,12 +3411,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3451,29 +3451,29 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3493,12 +3493,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3508,72 +3508,129 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3590,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7046,22 +7103,22 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -7081,45 +7138,49 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
@@ -7131,17 +7192,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -7157,29 +7218,29 @@
       <c r="G89" s="2" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -7195,7 +7256,7 @@
       <c r="G90" s="2" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
@@ -7207,17 +7268,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -7233,34 +7294,34 @@
       <c r="G91" s="2" t="inlineStr"/>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -7268,14 +7329,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G92" s="2" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
+          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>
       </c>
     </row>
@@ -7287,17 +7344,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_av</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -7317,7 +7374,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
+          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
@@ -7329,17 +7386,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
+          <t>lastet_opp_av</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -7359,7 +7416,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
+          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -7371,22 +7428,22 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_team</t>
+          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -7394,37 +7451,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
+          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>lastet_opp_team</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -7432,14 +7493,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
+          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -7451,12 +7508,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -7481,24 +7538,24 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Personen som har fullmakten.</t>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>bruker_id</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -7523,29 +7580,29 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+          <t>Personen som har fullmakten.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -7565,7 +7622,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
         </is>
       </c>
     </row>
@@ -7577,17 +7634,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -7607,7 +7664,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
         </is>
       </c>
     </row>
@@ -7619,17 +7676,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>forrige_pakke_id</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>pakke_id</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -7649,7 +7706,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
         </is>
       </c>
     </row>
@@ -7661,22 +7718,22 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -7684,37 +7741,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -7722,14 +7783,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G103" s="2" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -7741,17 +7798,17 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>godkjenner_id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -7771,29 +7828,29 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>godkjenner_id</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -7813,7 +7870,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Godkjenneren i steget.</t>
         </is>
       </c>
     </row>
@@ -7825,17 +7882,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -7855,7 +7912,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
         </is>
       </c>
     </row>
@@ -7867,35 +7924,77 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
           <t>aktor_id</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C108" s="2" t="inlineStr">
         <is>
           <t>koe.app_users</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D108" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E107" s="2" t="inlineStr">
+      <c r="E108" s="2" t="inlineStr">
         <is>
           <t>Fremmednøkkel</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr">
+      <c r="F108" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G107" s="2" t="inlineStr">
+      <c r="G108" s="2" t="inlineStr">
         <is>
           <t>NO ACTION</t>
         </is>
       </c>
-      <c r="H107" s="2" t="inlineStr">
+      <c r="H108" s="2" t="inlineStr">
         <is>
           <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>

</xml_diff>

<commit_message>
avvis bytte av Catenda-prosjekt med saker og stram inn registreringsskriptet
Del av #836. Arbeidsvalget 18.10 i #764: har prosjektet saker, avvises
bytte av Catenda-prosjekt; uten saker må kontraktsteamene oppgis på nytt,
og mappen og boardet beholdes bare for samme Catenda-prosjekt. Skriptet
sier fra om uendret virksomhet, manglende board og inaktiv kobling,
avviser registreringsflagg i kontraktsteam og godtar `--bh a b`.
Vakta for skriverne ser `DROP` og oppføringer uten formen `fil (…)`.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015T1t5VAsyBb5dkKT3DLMmw
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2115,7 +2115,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten.</t>
+          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten; skriptet sier fra når `--organisasjon` er en annen (#836).</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764).</t>
+          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764). Byttes Catenda-prosjektet, må teamene oppgis på nytt (#836).</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet, biblioteket og mappen og gjør koblingen aktiv. Boardet skrives over når det er oppgitt. Ellers står det hvis Catenda-prosjektet er det samme, og fjernes hvis det er byttet.</t>
+          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet og biblioteket og gjør koblingen aktiv. Mappen og boardet skrives over når de er oppgitt. Ellers står de hvis Catenda-prosjektet er det samme, og fjernes hvis det er byttet. Har prosjektet saker, avvises bytte av Catenda-prosjekt, og uten saker krever et bytte nye kontraktsteam (#836).</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
erstatt RTRIM-kontrollene med en tegnklasse og vern de uforanderlige tabellene mot TRUNCATE
- 20261019210000_tegnklasse.sql: de 31 kontrollene `*_uten_mellomrom`, som
  bare stoppet U+0020, blir `*_tegnklasse`, med bare U+0021–U+007E under den
  binære sorteringen (#609).
- 20261019211000_toemmingsvern.sql: `koe.toemmingsvern` har fremmednøkler til
  de åtte uforanderlige tabellene ingen annen nøkkel viste til, og kan ikke ha
  rader (#582).
- mellomrom.test.ts: vakten følger funksjonene `koe_sikkerhet` leser
  rekursivt, `fremmednoekkel` krever fast lengde på målet, og
  `verdiene_fyller_kolonnen` regner i byte i kolonnens koding (#673 p3–5). Ny
  vakt for den binære sorteringen på hver tekstkolonne (#609, #704 p2).
- journal.test.ts: TRUNCATE prøves mot hver tabell med triggeren, jobbene og
  vedleggene.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BcLWmkJoLWjEuGG9jR4pF6
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (provider, issuer, subject). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.app_identities_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3468,12 +3468,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3508,29 +3508,29 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3550,12 +3550,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3565,72 +3565,129 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3647,7 +3704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7061,22 +7118,22 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>app_identities_id</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_identities</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -7086,7 +7143,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -7096,29 +7153,29 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>brevdokument_id</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.brevdokument</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>leveringsoppdrag_id</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -7128,7 +7185,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -7138,29 +7195,29 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(godkjenningshandling_pakke_id, godkjenningshandling_loepenr)</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(pakke_id, loepenr)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -7170,7 +7227,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -7180,34 +7237,34 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id)</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.kvittering</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(prosjekt_id, aktor_id, kommando_id)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -7215,37 +7272,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>(leveringskvittering_oppdrag_id, leveringskvittering_operasjon)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>(leveringsoppdrag_id, operasjon)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -7253,37 +7314,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>prosjekt_med_saker_id</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -7291,37 +7356,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>sak_catenda_topic_sak_id</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -7329,32 +7398,36 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
+          <t>koe.toemmingsvern</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>vedlegg_id</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
           <t>koe.vedlegg</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>(sak_id, prosjekt_id)</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>koe.sak_metadata</t>
-        </is>
-      </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -7374,29 +7447,29 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_av</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -7406,7 +7479,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -7416,29 +7489,29 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -7448,7 +7521,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -7458,72 +7531,76 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
+          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_team</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G96" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -7531,41 +7608,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G97" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G97" s="2" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -7573,41 +7646,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Personen som har fullmakten.</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -7615,41 +7684,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G99" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G99" s="2" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -7657,36 +7722,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G100" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G100" s="2" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -7706,19 +7767,19 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>lastet_opp_av</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -7748,34 +7809,34 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -7783,37 +7844,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>lastet_opp_team</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -7821,31 +7886,27 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>godkjenner_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -7870,29 +7931,29 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>bruker_id</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -7912,29 +7973,29 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Personen som har fullmakten.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -7954,47 +8015,379 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>(sak_id, prosjekt_id)</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>forrige_pakke_id</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>pakke_id</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>aktor_id</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>aktor_team_id</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>koe.catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>team_id</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Uten fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr"/>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>godkjenner_id</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Godkjenneren i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
           <t>koe.godkjenningshandling</t>
         </is>
       </c>
-      <c r="B108" s="2" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>aktor_id</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="C116" s="2" t="inlineStr">
         <is>
           <t>koe.app_users</t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="D116" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E108" s="2" t="inlineStr">
+      <c r="E116" s="2" t="inlineStr">
         <is>
           <t>Fremmednøkkel</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr">
+      <c r="F116" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G108" s="2" t="inlineStr">
+      <c r="G116" s="2" t="inlineStr">
         <is>
           <t>NO ACTION</t>
         </is>
       </c>
-      <c r="H108" s="2" t="inlineStr">
+      <c r="H116" s="2" t="inlineStr">
         <is>
           <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>

</xml_diff>

<commit_message>
gi låsefeil på leserollen 503, logg årsaken i medlemsinngangene og fjern markøren i synkroniseringsraden
- prosjekter.ts: MedlemskapetLaast fra sett_leserolle gir 503 SYNC_UNAVAILABLE (#825 p2);
  fangene i lista og synkroniseringen logger feilen (#724 p2)
- prosjekter.test.ts: synced_at 30 s tilbake i prosjektMed, så testen ikke avhenger av
  klokka (#830); tester for låsen, loggingen og synkroniseringsraden
- migrasjon 20261019180000: catenda_project_id i app_membership_sync er NULL etter
  endret kobling, ikke den tomme GUID-en, og den tomme avvises (#726 p6)
- datamodellregisteret og katalog.json oppdatert

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019nS5wKJYGPLT2wvCcvd4z2
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660). Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10). Den tomme Catenda-ID-en er ikke lov; den merker synkroniseringsraden etter en slik endring. `topic_board_id` er boardet for saker som opprettes i appen (KT-U4); uten det avviser `koe_api.opprett_sak` saken (#741). Triggeren `koe.catenda_project_configs_endret` setter `updated_at` ved hver endring (#618).</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660). Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10), og setter Catenda-ID-en i synkroniseringsraden til NULL. Den tomme Catenda-ID-en er ikke lov. `topic_board_id` er boardet for saker som opprettes i appen (KT-U4); uten det avviser `koe_api.opprett_sak` saken (#741). Triggeren `koe.catenda_project_configs_endret` setter `updated_at` ved hver endring (#618).</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også gjennom `ferskeMedlemmer` for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden den tomme Catenda-ID-en og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10).</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også gjennom `ferskeMedlemmer` for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden ingen Catenda-ID (NULL) og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10, #726). Den tomme Catenda-ID-en er ikke lov.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">

</xml_diff>

<commit_message>
samle innloggingens Catenda-klient og kontroller boardet ved registrering
- tilbakekallet sletter den nye sesjonen når den gamle ikke kan slettes (#854 p1)
- hodekontrollen prøver navnene og rutens hoder (#854 p2)
- tilbakekallsadressen normaliseres som frontenden (#854 p4)
- innloggingen bruker integrasjonens CatendaOAuth (#726 p4)
- tokensvaret, subjektregelen og erObjekt på ett sted (#686 p1–p3)
- --board kontrolleres mot Catenda-prosjektet (#836 p2)
- bytte med saker avvises før Catenda-kallet (#868 p2)
- C18 i dataflyt.toml beskriver TS-skriptet (#868 p4)
- BARE_REGISTRER utledes av VALG (#868 p5)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFc1mgudee5cPaLFBuKYXm
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -8667,7 +8667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11551,12 +11551,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>C19.1</t>
+          <t>C18.3</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>C19 Kontraktsteam endres av drift</t>
+          <t>C18 Prosjekt registreres av drift</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -11566,77 +11566,124 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py contract-teams` med `--bh` og `--te`.</t>
+          <t>`scripts/catenda_admin.py register`.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Catenda: team og teammedlemmer</t>
+          <t>Catenda: topic board</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>Appen, lagres ikke</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>GET /v2/projects/{catenda_project_id}/teams</t>
+          <t>GET /opencde/bcf/3.0/projects?bimsync_project_id={catenda_project_id}</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/catenda_admin.py:cmd_contract_teams; backend/repositories/auth_repository.py:AuthRepository.set_contract_teams; databasefunksjon:koe_set_contract_teams</t>
+          <t>server/registrering.ts:kjoer; server/catenda.ts:CatendaOAuth</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Kontroll av at teamene drift oppgir, finnes i Catenda-prosjektet.</t>
+          <t>Kontroll av at boardet drift oppgir, hører til Catenda-prosjektet. Bare TS-skriptet kontrollerer det (#836).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>C19.1</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>C19 Kontraktsteam endres av drift</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>`scripts/catenda_admin.py contract-teams` med `--bh` og `--te`.</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: team og teammedlemmer</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>catenda_contract_teams</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>GET /v2/projects/{catenda_project_id}/teams</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>backend/scripts/catenda_admin.py:cmd_contract_teams; backend/repositories/auth_repository.py:AuthRepository.set_contract_teams; databasefunksjon:koe_set_contract_teams</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Kontroll av at teamene drift oppgir, finnes i Catenda-prosjektet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
           <t>C20.1</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>C20 Prosjektnavn hentes på nytt av drift</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>inn</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>`scripts/catenda_admin.py sync-name`.</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>Catenda: prosjekter</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>projects</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>GET /v2/projects/{catenda_project_id}</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>backend/scripts/catenda_admin.py:fetch_catenda_project_name; backend/scripts/catenda_admin.py:cmd_sync_name</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>Prosjektnavnet i Catenda, for hvert registrert prosjekt.</t>
         </is>

</xml_diff>

<commit_message>
kontroller boardet med detaljoppslaget og varsle når innloggingen mangler Catenda
Board-kontrollen leser bimsync_project_id i boardets detaljer, som Python,
i stedet for listen, der feltet ikke er dokumentert. Et ukjent board (404)
gir «Boardet finnes ikke», og et svar for et annet board avvises.
start.ts varsler at innloggingen ikke er satt opp når Catenda mangler.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzPvT1WMBVtiVWdawgpjSG
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -11581,7 +11581,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>GET /opencde/bcf/3.0/projects?bimsync_project_id={catenda_project_id}</t>
+          <t>GET /opencde/bcf/3.0/projects/{topic_board_id}</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -11591,7 +11591,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Kontroll av at boardet drift oppgir, hører til Catenda-prosjektet. Bare TS-skriptet kontrollerer det (#836).</t>
+          <t>`bimsync_project_id` for boardet drift oppgir, kontrollert mot Catenda-prosjektet. Bare TS-skriptet kontrollerer det (#836).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
la porten i opprett_sak være predikatet, kutt tidsstandardene og bind oppdraget til prosjektet
- koe_api.opprett_sak bruker koe_sikkerhet.oppretter som port (#877 punkt 22)
- standardene med SYSUTCDATETIME() kutter til millisekunder (#778 punkt 7)
- koe_api.start_jobb_paa_nytt lagrer SID-en, ikke innloggingsnavnet (#778)
- jobben, PDF-en og kvitteringene viser til oppdraget med prosjekt_id (#783)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZTGnpSGxxQdX6SJd7BDSR
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2643,7 +2643,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id); unik (id, prosjekt_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); leveringsoppdrag_id → koe.leveringsoppdrag.id (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>leveringsoppdrag_id</t>
+          <t>(leveringsoppdrag_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget en jobb `levering` leverer (#371). Hvert oppdrag har høyst én jobb.</t>
+          <t>Oppdraget en jobb `levering` leverer (#371). Hvert oppdrag har høyst én jobb. Sammensatt med `prosjekt_id`, så jobben står i oppdragets prosjekt (#783).</t>
         </is>
       </c>
     </row>
@@ -6978,7 +6978,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>leveringsoppdrag_id</t>
+          <t>(leveringsoppdrag_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget PDF-en gjengir. Det er én PDF per oppdrag (#371 del 2).</t>
+          <t>Oppdraget PDF-en gjengir. Det er én PDF per oppdrag (#371 del 2). Sammensatt med `prosjekt_id`, så PDF-en står i oppdragets prosjekt (#783).</t>
         </is>
       </c>
     </row>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>leveringsoppdrag_id</t>
+          <t>(leveringsoppdrag_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -7068,7 +7068,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371).</t>
+          <t>Oppdraget kvitteringen gjelder: én rad for dokumentet og én for referansen på topicen (B-03, #371). Sammensatt med `prosjekt_id`, så kvitteringen står i oppdragets prosjekt (#783).</t>
         </is>
       </c>
     </row>
@@ -7264,7 +7264,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>leveringsoppdrag_id</t>
+          <t>(leveringsoppdrag_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Oppdraget som leverte vedlegget. Et senere oppdrag som viser til samme vedlegg, får ingen ny rad.</t>
+          <t>Oppdraget som leverte vedlegget. Et senere oppdrag som viser til samme vedlegg, får ingen ny rad. Sammensatt med `prosjekt_id`, så kvitteringen står i oppdragets prosjekt (#783).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
la runneren lese identiteten før oppryddingen, og les biblioteket før kallet i testene
Oppryddingen etter migreringen avgjøres nå av USER_NAME() i forbindelsen, ikke av
feiltypen, så en sats som bytter identitet og avvises av en annen kontroll først,
ryddes heller ikke (#885 punkt 6). Bibliotektestene leser biblioteket før kallet
starter. Modulheaderen og jobbforsoek i datamodellen viser til de nye
definisjonene.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHJyt5r6ujksCooTRJKUU8
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med innloggingen som startet jobben på nytt. Raden endres ikke.</t>
+          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med SID-en til innloggingen som startet jobben på nytt (`sid:0x…`, eller `driften uten SID`). Raden endres ikke.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Prosedyrene for jobbkjøreren og driftsverktøyet i `database/migrasjoner/20261018100000_jobber.sql`.</t>
+          <t>Prosedyrene for jobbkjøreren i `database/migrasjoner/20261018100000_jobber.sql`, og driftsverktøyet `koe_api.start_jobb_paa_nytt`, sist definert i `20261020121000_oppretter_tid_og_oppdragsnoekkel.sql`.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">

</xml_diff>

<commit_message>
ta imot webhooken fra Catenda i TS med innboks i SQL Server (W-1a)
Den hemmelige stien sammenlignes i konstant tid (INT-01), og hendelsen
lagres i koe.innkommende_hendelse før svaret 200, én gang per event.id
(INT-02). Behandlingen kommer i W-1b.

Del av #819.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017BrjZNFzBYatGy2S2MJKWz
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3411,12 +3411,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Behandlingen kommer i W-1b.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3436,12 +3436,12 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3461,19 +3461,19 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3493,12 +3493,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3525,12 +3525,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3575,19 +3575,19 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3622,29 +3622,29 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3679,72 +3679,129 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="J59" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr">
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3761,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7554,17 +7611,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_med_saker_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -7596,17 +7653,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>sak_catenda_topic_sak_id</t>
+          <t>prosjekt_med_saker_id</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -7638,17 +7695,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>sak_catenda_topic_sak_id</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -7680,17 +7737,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>(vedlegg_id, operasjon)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -7717,22 +7774,22 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon)</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(vedlegg_id, operasjon)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -7742,7 +7799,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -7752,29 +7809,29 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -7794,29 +7851,29 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -7836,45 +7893,49 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G102" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
@@ -7886,17 +7947,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -7912,29 +7973,29 @@
       <c r="G103" s="2" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -7950,7 +8011,7 @@
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
@@ -7962,17 +8023,17 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -7988,34 +8049,34 @@
       <c r="G105" s="2" t="inlineStr"/>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -8023,14 +8084,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
+          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>
       </c>
     </row>
@@ -8042,17 +8099,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_av</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -8072,7 +8129,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
+          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
@@ -8084,17 +8141,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
+          <t>lastet_opp_av</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -8114,7 +8171,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
+          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -8126,22 +8183,22 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_team</t>
+          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -8149,37 +8206,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
+          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>lastet_opp_team</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -8187,14 +8248,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
+          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -8206,12 +8263,12 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -8236,24 +8293,24 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Personen som har fullmakten.</t>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>bruker_id</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -8278,29 +8335,29 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+          <t>Personen som har fullmakten.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -8320,7 +8377,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
         </is>
       </c>
     </row>
@@ -8332,17 +8389,17 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -8362,7 +8419,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
         </is>
       </c>
     </row>
@@ -8374,17 +8431,17 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>forrige_pakke_id</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>pakke_id</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -8404,7 +8461,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
         </is>
       </c>
     </row>
@@ -8416,22 +8473,22 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -8439,37 +8496,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -8477,14 +8538,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G117" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G117" s="2" t="inlineStr"/>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -8496,17 +8553,17 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>godkjenner_id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -8526,29 +8583,29 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>godkjenner_id</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -8568,7 +8625,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Godkjenneren i steget.</t>
         </is>
       </c>
     </row>
@@ -8580,17 +8637,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -8610,7 +8667,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
         </is>
       </c>
     </row>
@@ -8622,35 +8679,77 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
           <t>aktor_id</t>
         </is>
       </c>
-      <c r="C121" s="2" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>koe.app_users</t>
         </is>
       </c>
-      <c r="D121" s="2" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E121" s="2" t="inlineStr">
+      <c r="E122" s="2" t="inlineStr">
         <is>
           <t>Fremmednøkkel</t>
         </is>
       </c>
-      <c r="F121" s="2" t="inlineStr">
+      <c r="F122" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G121" s="2" t="inlineStr">
+      <c r="G122" s="2" t="inlineStr">
         <is>
           <t>NO ACTION</t>
         </is>
       </c>
-      <c r="H121" s="2" t="inlineStr">
+      <c r="H122" s="2" t="inlineStr">
         <is>
           <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>
@@ -8667,7 +8766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11686,6 +11785,53 @@
       <c r="I64" s="2" t="inlineStr">
         <is>
           <t>Prosjektnavnet i Catenda, for hvert registrert prosjekt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>C21.1</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>C21 Webhooken fra Catenda til innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Webhook fra Catenda til `POST /webhook/catenda/&lt;hemmelig sti&gt;` i TS-serveren (W-1a, #819). Alle hendelsestyper tas imot, også `bcf.*`.</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>koe.innkommende_hendelse</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Innkommende POST fra Catenda</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>server/webhook.ts:taImot; server/webhook.ts:mottaHendelse</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Hele kroppen, med `event.id` og `event.type` i egne kolonner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
behandle hendelsene i innboksen fra webhooken i jobbløkka (W-1b.1)
En topic laget av TE gir en sak med topicens tittel, koblet til topicen i
samme transaksjon (KT-U6). En topic fra BH (KT-U7), en topic av en annen
type (arbeidsvalget i #819), en topic som alt hører til en sak eller er
laget av integrasjonen (#741 punkt 17) og en forfatter uten entydig side
(INT-04) gir ingen sak, og utfallet lagres i koe.innkommende_behandling.
Topic-ID-en normaliseres med én regel for UUID med bindestreker (#906).

Del av #819. Del av #906.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dv5urHiKKqmKQ6HZQiZEdd
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370).</t>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370), og som `server/hendelser.ts` kaller for en ny topic fra TE i innboksen (KT-U6, #819).</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2467,12 +2467,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Saken kan være opprettet fra en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_behandling.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Sakstittelen i `sak_opprettet` kan være tittelen på en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
+          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). En sak fra en topic i innboksen får ingen jobb; den kobles til topicen (W-1b.1, #819). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741).</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Behandlingen kommer i W-1b.</t>
+          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3468,12 +3468,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Raden kan ikke endres eller slettes; en kommentar tilbake til topicen (W-1b.2) endrer ikke utfallet.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3493,12 +3493,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3518,19 +3518,19 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3550,12 +3550,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3582,12 +3582,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3632,19 +3632,19 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3679,29 +3679,29 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3736,72 +3736,129 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="J60" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3818,7 +3875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H122"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7653,17 +7710,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_med_saker_id</t>
+          <t>innkommende_behandling_id</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -7695,17 +7752,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>sak_catenda_topic_sak_id</t>
+          <t>prosjekt_med_saker_id</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -7737,17 +7794,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>sak_catenda_topic_sak_id</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -7779,17 +7836,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>(vedlegg_id, operasjon)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -7816,22 +7873,22 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon)</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>(vedlegg_id, operasjon)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -7841,7 +7898,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -7851,29 +7908,29 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -7893,29 +7950,29 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -7935,34 +7992,34 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Hendelsen i innboksen utfallet gjelder (W-1b.1, #819). Nøkkelen er primærnøkkelen, så hver hendelse har høyst ett utfall, og en hendelse uten rad er ikke behandlet.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -7970,108 +8027,120 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Saken hendelsen ga, bare med utfallet `sak_opprettet` (KT-U6). Med et annet utfall er `sak_id` tom, så nøkkelen gjelder ikke, og `prosjekt_id` er prosjektet koblingen ga, eller tom når prosjektet er ukjent.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G104" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G105" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -8087,34 +8156,34 @@
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -8122,41 +8191,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G107" s="2" t="inlineStr"/>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_av</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -8164,26 +8229,22 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G108" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -8193,12 +8254,12 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -8206,14 +8267,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G109" s="2" t="inlineStr"/>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
+          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>
       </c>
     </row>
@@ -8225,22 +8282,22 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_team</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -8248,27 +8305,31 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
+          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>lastet_opp_av</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -8293,29 +8354,29 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
+          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -8335,34 +8396,34 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Personen som har fullmakten.</t>
+          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>lastet_opp_team</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -8370,36 +8431,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G113" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G113" s="2" t="inlineStr"/>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -8419,29 +8476,29 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>bruker_id</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -8461,24 +8518,24 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Personen som har fullmakten.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -8503,7 +8560,7 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
         </is>
       </c>
     </row>
@@ -8515,22 +8572,22 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -8538,22 +8595,26 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>forrige_pakke_id</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -8563,7 +8624,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>pakke_id</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -8583,19 +8644,19 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>godkjenner_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -8625,34 +8686,34 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -8660,36 +8721,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G120" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -8709,47 +8766,173 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>godkjenner_id</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Godkjenneren i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
           <t>koe.godkjenningshandling</t>
         </is>
       </c>
-      <c r="B122" s="2" t="inlineStr">
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
         <is>
           <t>aktor_id</t>
         </is>
       </c>
-      <c r="C122" s="2" t="inlineStr">
+      <c r="C125" s="2" t="inlineStr">
         <is>
           <t>koe.app_users</t>
         </is>
       </c>
-      <c r="D122" s="2" t="inlineStr">
+      <c r="D125" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E122" s="2" t="inlineStr">
+      <c r="E125" s="2" t="inlineStr">
         <is>
           <t>Fremmednøkkel</t>
         </is>
       </c>
-      <c r="F122" s="2" t="inlineStr">
+      <c r="F125" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G122" s="2" t="inlineStr">
+      <c r="G125" s="2" t="inlineStr">
         <is>
           <t>NO ACTION</t>
         </is>
       </c>
-      <c r="H122" s="2" t="inlineStr">
+      <c r="H125" s="2" t="inlineStr">
         <is>
           <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>
@@ -8766,7 +8949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11832,6 +12015,288 @@
       <c r="I65" s="2" t="inlineStr">
         <is>
           <t>Hele kroppen, med `event.id` og `event.type` i egne kolonner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>C22.1</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: innlogget bruker</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Appen, lagres ikke</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>GET /v2/user</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Integrasjonens egen Catenda-ID (`egenId`), som skiller topics integrasjonen laget. Lagres ikke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>C22.2</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: team og teammedlemmer</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Appen, lagres ikke</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>GET /v2/projects/{catenda_project_id}/teams/{team_id}/members (sidevis), for hvert kontraktsteam</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/autorisasjon.ts:kontraktssideUtenSesjon; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Forfatterens side og team. Blir `aktor_rolle` og `aktor_team_id` i `sak_opprettet`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>C22.3</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_metadata</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad som ved innlogging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>C22.3</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad som ved innlogging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>C22.3</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_catenda_topic</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad som ved innlogging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>C22.4</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>koe.innkommende_behandling</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:registrerBehandling</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Utfallet, med prosjektet, saken og topicen når de er kjent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
les forfatter, type og tittel fra topicen i Catenda, ikke fra kroppen
Kroppen fra webhooken er ikke signert. Behandlingen bruker nå bare topic-ID-en,
boardet og Catenda-prosjektet fra den, henter topicen med integrasjonens token
og løser identiteten først når forfatteren står i medlemslisten fra Catenda,
med navnet og e-posten derfra. En forfalsket kropp gir ingen sak og ingen endret
brukerrad.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR6RgBo4rGt3G71xkT8kPC
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -8949,7 +8949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12088,7 +12088,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Catenda: team og teammedlemmer</t>
+          <t>Catenda: topics</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -12098,17 +12098,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>GET /v2/projects/{catenda_project_id}/teams/{team_id}/members (sidevis), for hvert kontraktsteam</t>
+          <t>GET /opencde/bcf/3.0/projects/{topic_board_id}/topics/{topic_guid}</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/autorisasjon.ts:kontraktssideUtenSesjon; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Forfatterens side og team. Blir `aktor_rolle` og `aktor_team_id` i `sak_opprettet`.</t>
+          <t>Topicens tittel, type og forfatter (`bimsync_creation_author.user.ref`), med integrasjonens token. Kroppen fra webhooken leses ikke for dem. 404 gir utfallet `ugyldig_hendelse` uten sak.</t>
         </is>
       </c>
     </row>
@@ -12135,34 +12135,34 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Catenda: webhook-varsel</t>
+          <t>Catenda: prosjektmedlemmer</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>Appen, lagres ikke</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Hendelsen i innboksen</t>
+          <t>GET /v2/projects/{catenda_project_id}/members?userType=user (sidevis)</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad som ved innlogging.</t>
+          <t>Om forfatteren er medlem av prosjektet, og navnet og e-posten som sendes til `koe_api.catenda_identitet`. Uten medlemskap løses ingen identitet.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>C22.3</t>
+          <t>C22.4</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -12182,34 +12182,34 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Catenda: webhook-varsel</t>
+          <t>Catenda: team og teammedlemmer</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>Appen, lagres ikke</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Hendelsen i innboksen</t>
+          <t>GET /v2/projects/{catenda_project_id}/teams/{team_id}/members (sidevis), for hvert kontraktsteam</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/autorisasjon.ts:kontraktssideUtenSesjon; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad som ved innlogging.</t>
+          <t>Forfatterens side og team. Blir `aktor_rolle` og `aktor_team_id` i `sak_opprettet`.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>C22.3</t>
+          <t>C22.5</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -12249,14 +12249,14 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad som ved innlogging.</t>
+          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad med navnet og e-posten fra medlemslisten, som ved medlemssynkroniseringen, og bare for et medlem.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>C22.4</t>
+          <t>C22.5</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -12281,20 +12281,114 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
+          <t>koe.hendelse</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad med navnet og e-posten fra medlemslisten, som ved medlemssynkroniseringen, og bare for et medlem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>C22.5</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>koe.sak_catenda_topic</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:behandle; server/kommandoer.ts:opprettSak</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Topicens tittel blir sakstittelen i `sak_opprettet`, og topicen og boardet blir koblingen i `koe.sak_catenda_topic`, skrevet av `koe_api.koble_topic` fra `koe_api.opprett_sak`. Kvitteringen i `koe.kvittering` har en kommando-ID avledet av hendelsen i innboksen. Forfatteren løses til en brukerrad med navnet og e-posten fra medlemslisten, som ved medlemssynkroniseringen, og bare for et medlem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>C22.6</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
           <t>koe.innkommende_behandling</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>Hendelsen i innboksen</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:registrerBehandling</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Utfallet, med prosjektet, saken og topicen når de er kjent.</t>
         </is>

</xml_diff>

<commit_message>
før de nye tabellene, nøklene og kallene til Catenda i datamodellregistrene
Del av #819.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RXo2SrvjDmjpdtTz41sHvT
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Raden kan ikke endres eller slettes; en kommentar tilbake til topicen (W-1b.2) endrer ikke utfallet.</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3493,12 +3493,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3525,12 +3525,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3550,12 +3550,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3575,19 +3575,19 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3632,19 +3632,19 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3689,19 +3689,19 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3736,29 +3736,29 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3803,62 +3803,176 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>avledet</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Som journalen den er regnet fra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr">
+      <c r="K62" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -3875,7 +3989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7752,17 +7866,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_med_saker_id</t>
+          <t>innkommende_forsoek_id</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -7794,17 +7908,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>sak_catenda_topic_sak_id</t>
+          <t>topic_kommentar_id</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>sak_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -7836,17 +7950,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>prosjekt_med_saker_id</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>vedlegg_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -7878,17 +7992,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon)</t>
+          <t>sak_catenda_topic_sak_id</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>(vedlegg_id, operasjon)</t>
+          <t>sak_id</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -7915,22 +8029,22 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>vedlegg_id</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -7940,7 +8054,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -7950,29 +8064,29 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>innkommende_hendelse_id</t>
+          <t>(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon)</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_hendelse</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(vedlegg_id, operasjon)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -7982,7 +8096,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -7992,14 +8106,14 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Hendelsen i innboksen utfallet gjelder (W-1b.1, #819). Nøkkelen er primærnøkkelen, så hver hendelse har høyst ett utfall, og en hendelse uten rad er ikke behandlet.</t>
+          <t>Vernet mot TRUNCATE (#582). `koe.toemmingsvern` har ingen rader, så nøkkelen viser aldri til en rad.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -8024,7 +8138,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -8034,24 +8148,24 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Saken hendelsen ga, bare med utfallet `sak_opprettet` (KT-U6). Med et annet utfall er `sak_id` tom, så nøkkelen gjelder ikke, og `prosjekt_id` er prosjektet koblingen ga, eller tom når prosjektet er ukjent.</t>
+          <t>Saken topicen hører til. `sak_id` er primærnøkkelen, så hver sak har høyst én topic. Sammensatt med `prosjekt_id`, så raden står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -8076,14 +8190,14 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
+          <t>Hendelsen i innboksen utfallet gjelder (W-1b.1, #819). Nøkkelen er primærnøkkelen, så hver hendelse har høyst ett utfall, og en hendelse uten rad er ikke behandlet.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -8108,7 +8222,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -8118,34 +8232,34 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
+          <t>Saken hendelsen ga, bare med utfallet `sak_opprettet` (KT-U6). Med et annet utfall er `sak_id` tom, så nøkkelen gjelder ikke, og `prosjekt_id` er prosjektet koblingen ga, eller tom når prosjektet er ukjent.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -8153,151 +8267,167 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
+          <t>Hendelsen i innboksen forsøket gjelder (W-1b.2, #819). En hendelse kan ha mange forsøk, for behandlingen og for kommentaren.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>innkommende_hendelse_id</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G107" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Brevet dette brevet svarer på eller viser til.</t>
+          <t>Utfallet kommentaren hører til (W-1b.2, #819). Nøkkelen er primærnøkkelen, så hvert utfall har høyst én kvittering.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G108" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
+          <t>Prosjektet som har saker. `prosjekt_id` er primærnøkkelen, så hvert prosjekt står høyst én gang (F-1, #820).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>refererer_til_event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr"/>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
+          <t>Saken bufferen er regnet for. `sak_id` er primærnøkkel, så én buffer per sak. Sammensatt med `prosjekt_id`.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -8305,41 +8435,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G110" s="2" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
+          <t>Teamet avsenderen satt i, i `catenda_id()`-formen. Tom når teamet ikke var entydig (DL-U4).</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_av</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -8347,41 +8473,37 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G111" s="2" t="inlineStr"/>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
+          <t>Brevet dette brevet svarer på eller viser til.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>(event_id, sak_id, prosjekt_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -8389,36 +8511,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G112" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G112" s="2" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
+          <t>Teamet som kan lese notatet. Basen avviser et notat uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>lastet_opp_team</t>
+          <t>refererer_til_event_id</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -8434,29 +8552,29 @@
       <c r="G113" s="2" t="inlineStr"/>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
+          <t>Brevet notatet gjelder, uten fremmednøkkel, så notatet kan slettes uten å røre journalen.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -8476,19 +8594,19 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
+          <t>Saken vedlegget er lastet opp i. Sammensatt med `prosjekt_id`, så vedlegget står i sakens prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>lastet_opp_av</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -8518,29 +8636,29 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Personen som har fullmakten.</t>
+          <t>Den som lastet opp vedlegget, `app_users.id` (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>(bundet_av_event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(event_id, sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -8560,34 +8678,34 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+          <t>Den første hendelsen som viser til vedlegget (arbeidsvalg 4 i #790), i samme sak og prosjekt. Tom for et ubundet vedlegg.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>lastet_opp_team</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -8595,36 +8713,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G117" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G117" s="2" t="inlineStr"/>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Teamet som ser og sletter vedlegget før det er bundet. Basen avviser et vedlegg uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -8644,19 +8758,19 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>bruker_id</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -8686,34 +8800,34 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Personen som har fullmakten.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -8721,32 +8835,36 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -8766,29 +8884,29 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>godkjenner_id</t>
+          <t>forrige_pakke_id</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>pakke_id</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -8808,29 +8926,29 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -8850,34 +8968,34 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -8885,54 +9003,218 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G124" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>godkjenner_id</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>Godkjenneren i steget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
           <t>koe.godkjenningshandling</t>
         </is>
       </c>
-      <c r="B125" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningspakke</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
         <is>
           <t>aktor_id</t>
         </is>
       </c>
-      <c r="C125" s="2" t="inlineStr">
+      <c r="C129" s="2" t="inlineStr">
         <is>
           <t>koe.app_users</t>
         </is>
       </c>
-      <c r="D125" s="2" t="inlineStr">
+      <c r="D129" s="2" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E125" s="2" t="inlineStr">
+      <c r="E129" s="2" t="inlineStr">
         <is>
           <t>Fremmednøkkel</t>
         </is>
       </c>
-      <c r="F125" s="2" t="inlineStr">
+      <c r="F129" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G125" s="2" t="inlineStr">
+      <c r="G129" s="2" t="inlineStr">
         <is>
           <t>NO ACTION</t>
         </is>
       </c>
-      <c r="H125" s="2" t="inlineStr">
+      <c r="H129" s="2" t="inlineStr">
         <is>
           <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>
@@ -8949,7 +9231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12036,7 +12318,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -12083,7 +12365,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -12130,7 +12412,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -12177,7 +12459,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -12224,7 +12506,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -12271,7 +12553,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -12318,7 +12600,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -12365,7 +12647,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall (W-1b.1, #819).</t>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -12390,7 +12672,242 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Utfallet, med prosjektet, saken og topicen når de er kjent.</t>
+          <t>Utfallet, med prosjektet, saken, topicen og boardet når de er kjent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>C22.7</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>C22 Behandlingen av innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>inn</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter jobbene: `behandleEnHendelse` i `server/jobber.ts` tar den eldste hendelsen i `koe.innkommende_hendelse` uten utfall som ikke venter etter et forsøk (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: webhook-varsel</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>koe.innkommende_forsoek</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Hendelsen i innboksen</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:behandleEnHendelse; server/hendelser.ts:registrerForsoek</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Steget `behandling` og feilklassen med meldingen, når Catenda eller basen ikke svarte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>C23.1</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>C23 Kommentaren tilbake til topicen fra innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>ut</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter behandlingen av innboksen: `skrivEnKommentar` i `server/jobber.ts` tar det eldste utfallet i `koe.innkommende_behandling` som skal ha en kommentar, ikke har en kvittering og ikke venter etter et forsøk (W-1b.2, #819).</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: kommentarer</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Appen, lagres ikke</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>GET /opencde/bcf/3.0/projects/{catenda_board_id}/topics/{catenda_topic_id}/comments</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:skrivEnKommentar; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Kommentarene på topicen, med ID og tekst. Står samme tekst der, brukes den kommentarens ID. Lagres ikke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>C23.2</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>C23 Kommentaren tilbake til topicen fra innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>ut</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter behandlingen av innboksen: `skrivEnKommentar` i `server/jobber.ts` tar det eldste utfallet i `koe.innkommende_behandling` som skal ha en kommentar, ikke har en kvittering og ikke venter etter et forsøk (W-1b.2, #819).</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>koe.innkommende_behandling</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: kommentarer</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>POST /opencde/bcf/3.0/projects/{catenda_board_id}/topics/{catenda_topic_id}/comments</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:skrivEnKommentar; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Kommentaren for utfallet (`comment`), bare når samme tekst ikke står på topicen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>C23.3</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>C23 Kommentaren tilbake til topicen fra innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>ut</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter behandlingen av innboksen: `skrivEnKommentar` i `server/jobber.ts` tar det eldste utfallet i `koe.innkommende_behandling` som skal ha en kommentar, ikke har en kvittering og ikke venter etter et forsøk (W-1b.2, #819).</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: kommentarer</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>koe.topic_kommentar</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Svaret fra Catenda</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:skrivEnKommentar; server/hendelser.ts:kvitterKommentar</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>ID-en til kommentaren i Catenda, funnet eller skrevet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>C23.4</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>C23 Kommentaren tilbake til topicen fra innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>ut</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter behandlingen av innboksen: `skrivEnKommentar` i `server/jobber.ts` tar det eldste utfallet i `koe.innkommende_behandling` som skal ha en kommentar, ikke har en kvittering og ikke venter etter et forsøk (W-1b.2, #819).</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: kommentarer</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>koe.innkommende_forsoek</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Svaret fra Catenda, eller at det mangler</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:skrivEnKommentar; server/hendelser.ts:registrerForsoek</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Steget `kommentar` og feilklassen med meldingen, når Catenda eller basen ikke svarte.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
legg til innlogging med Entra ID og identiteten for den (S-1c del 1)
`/api/auth/entra/login` og `/callback` med PKCE og nonce, ID-tokenet
validert mot JWKS, og identiteten løst gjennom `koe_api.entra_identitet`
med en hviteliste over tenanter. Entra-sesjonen gir ingen prosjekttilgang.

Del av #831

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NihFjDYkRdtR2U7uWfKhbU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet` eller `koe_api.entra_identitet`, oppretter brukeren første gang en identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659) og `entraIdentitet` i `server/entra.ts` (S-1c del 1, #831).</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Identitetene til en bruker, unike på leverandør, issuer og subjekt. En Catenda-identitet har issueren og subjektformen basen kontrollerer, så samme person ikke får to brukerrader (AGENTS.md).</t>
+          <t>Identitetene til en bruker, unike på leverandør, issuer og subjekt. En Catenda-identitet og en Entra-identitet har issueren og subjektformen basen kontrollerer, så samme person ikke får to brukerrader (AGENTS.md). For Entra er issueren v2-formen for tenanten og subjektet `oid`, begge i små bokstaver (#831).</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659) og gjennom `koe_api.entra_identitet` fra tilbakekallet for Entra ID (S-1c del 1, #831).</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Ja, for leverandøren `catenda`: subjektet er Catenda-ID-en. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, for leverandøren `catenda`: subjektet er Catenda-ID-en. For `entra` kommer subjektet fra ID-tokenet fra Entra ID. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2100,12 +2100,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.entra_tenant</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene. `id` er prosjektgrensen i alle tabellene med saksdata, uten standardverdi (AGENTS.md). `server/prosjekter.ts` leser prosjektene aktøren er aktivt medlem i med `koe_api.brukerens_prosjekter`, og ett av dem med `koe_api.prosjekt` (#660). Tabellen har ikke `settings` og `created_by` fra PostgreSQL.</t>
+          <t>Tenantene i Entra ID driften har godkjent for innloggingen (S-1c del 1, #831). `koe_api.entra_identitet` avviser en issuer for en tenant som ikke står her. Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten; skriptet sier fra når `--organisasjon` er en annen (#836).</t>
+          <t>Driften, som eier. Lest av `koe_api.entra_identitet` fra `server/entra.ts`.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Navnet oppgis av driften; i Python kan det hentes fra Catenda-prosjektet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (tenant_id). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2145,24 +2145,24 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>koe.app_project_memberships</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660). `koe_api.medlemmer`, også kalt derfra, leser de aktive medlemmene for en aktør med aktivt medlemskap (#820).</t>
+          <t>Prosjektene. `id` er prosjektgrensen i alle tabellene med saksdata, uten standardverdi (AGENTS.md). `server/prosjekter.ts` leser prosjektene aktøren er aktivt medlem i med `koe_api.brukerens_prosjekter`, og ett av dem med `koe_api.prosjekt` (#660). Tabellen har ikke `settings` og `created_by` fra PostgreSQL.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2172,22 +2172,22 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10). `koe_api.sett_leserolle`, kalt fra `server/prosjekter.ts`, setter `viewer_override` for et annet aktivt medlem når aktøren er aktiv admin uten leserolle (#820).</t>
+          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten; skriptet sier fra når `--organisasjon` er en annen (#836).</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Delvis</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Ja, medlemslisten i Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Navnet oppgis av driften; i Python kan det hentes fra Catenda-prosjektet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2197,29 +2197,29 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>grunndata, kopi</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>E-post og visningsnavn.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_project_memberships</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen. `server/autorisasjon.ts` leser prosjektets kontraktsteam med `koe_api.kontraktsteam`, bare for en aktør med aktivt medlemskap uten leserollen (#658).</t>
+          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660). `koe_api.medlemmer`, også kalt derfra, leser de aktive medlemmene for en aktør med aktivt medlemskap (#820).</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2229,22 +2229,22 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764). Byttes Catenda-prosjektet, må teamene oppgis på nytt (#836).</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10). `koe_api.sett_leserolle`, kalt fra `server/prosjekter.ts`, setter `viewer_override` for et annet aktivt medlem når aktøren er aktiv admin uten leserolle (#820).</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Delvis</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, medlemslisten i Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.aktor_team_id (uten fremmednøkkel); koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2254,29 +2254,29 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>grunndata, kopi</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>E-post og visningsnavn.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_project_configs</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660). Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10), og setter Catenda-ID-en i synkroniseringsraden til NULL. Den tomme Catenda-ID-en er ikke lov. `topic_board_id` er boardet for saker som opprettes i appen (KT-U4); uten det avviser `koe_api.opprett_sak` saken (#741). `koe_api.opprett_sak` låser raden før den leses, så en ny sak og en ny registrering eller nye kontraktsteam skrives etter hverandre (#868). Triggeren `koe.catenda_project_configs_endret` setter `updated_at` ved hver endring (#618).</t>
+          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen. `server/autorisasjon.ts` leser prosjektets kontraktsteam med `koe_api.kontraktsteam`, bare for en aktør med aktivt medlemskap uten leserollen (#658).</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet og biblioteket og gjør koblingen aktiv. Mappen og boardet skrives over når de er oppgitt. Ellers står de hvis Catenda-prosjektet er det samme, og fjernes hvis det er byttet. Mappen fjernes også når biblioteket er byttet. Har prosjektet saker, avvises bytte av Catenda-prosjekt, og uten saker krever et bytte nye kontraktsteam (#836).</t>
+          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764). Byttes Catenda-prosjektet, må teamene oppgis på nytt (#836).</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2296,12 +2296,12 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.aktor_team_id (uten fremmednøkkel); koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2328,12 +2328,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_absences</t>
+          <t>koe.catenda_project_configs</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene der innloggingens liste over brukerens Catenda-prosjekter viste at brukeren ikke er med, for en bruker uten medlemskap der (DL-U9). `observed_at` er når innloggingens liste ble hentet, etter basens klokke. En medlemsliste hentet samtidig eller før gir ikke brukeren et nytt medlemskap. Har ingen tabell i PostgreSQL.</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660). Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10), og setter Catenda-ID-en i synkroniseringsraden til NULL. Den tomme Catenda-ID-en er ikke lov. `topic_board_id` er boardet for saker som opprettes i appen (KT-U4); uten det avviser `koe_api.opprett_sak` saken (#741). `koe_api.opprett_sak` låser raden før den leses, så en ny sak og en ny registrering eller nye kontraktsteam skrives etter hverandre (#868). Triggeren `koe.catenda_project_configs_endret` setter `updated_at` ved hver endring (#618).</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Innloggingen kaller modulen fra tilbakekallet i `server/innlogging.ts` (F0b-5b).</t>
+          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet og biblioteket og gjør koblingen aktiv. Mappen og boardet skrives over når de er oppgitt. Ellers står de hvis Catenda-prosjektet er det samme, og fjernes hvis det er byttet. Mappen fjernes også når biblioteket er byttet. Har prosjektet saker, avvises bytte av Catenda-prosjekt, og uten saker krever et bytte nye kontraktsteam (#836).</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2353,12 +2353,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id, user_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2373,24 +2373,24 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med prosjektene brukeren ikke er med i og tidspunktene for innloggingene (`observed_at`, `updated_at`).</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_sync</t>
+          <t>koe.app_membership_absences</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også gjennom `ferskeMedlemmer` for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden ingen Catenda-ID (NULL) og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10, #726). Den tomme Catenda-ID-en er ikke lov.</t>
+          <t>Prosjektene der innloggingens liste over brukerens Catenda-prosjekter viste at brukeren ikke er med, for en bruker uten medlemskap der (DL-U9). `observed_at` er når innloggingens liste ble hentet, etter basens klokke. En medlemsliste hentet samtidig eller før gir ikke brukeren et nytt medlemskap. Har ingen tabell i PostgreSQL.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, og triggeren `koe.catenda_project_configs_kobling_endret` når koblingen endres.</t>
+          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Innloggingen kaller modulen fra tilbakekallet i `server/innlogging.ts` (F0b-5b).</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id, user_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2435,44 +2435,44 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med prosjektene brukeren ikke er med i og tidspunktene for innloggingene (`observed_at`, `updated_at`).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også gjennom `ferskeMedlemmer` for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden ingen Catenda-ID (NULL) og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10, #726). Den tomme Catenda-ID-en er ikke lov.</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, og triggeren `koe.catenda_project_configs_kobling_endret` når koblingen endres.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370), og som `server/hendelser.ts` kaller for en ny topic fra TE i innboksen (KT-U6, #819).</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Saken kan være opprettet fra en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_behandling.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2492,19 +2492,19 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>`created_by` peker på en bruker.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661), og `koe_api.opprett_sak` fra `POST /api/kjerne/saker` (#370).</t>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370), og som `server/hendelser.ts` kaller for en ny topic fra TE i innboksen (KT-U6, #819).</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2524,12 +2524,12 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Sakstittelen i `sak_opprettet` kan være tittelen på en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Delvis. Saken kan være opprettet fra en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel); koe.vedlegg.(bundet_av_event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_behandling.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2549,19 +2549,19 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
+          <t>`created_by` peker på en bruker.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
+          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661), og `koe_api.opprett_sak` fra `POST /api/kjerne/saker` (#370).</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Sakstittelen i `sak_opprettet` kan være tittelen på en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel); koe.vedlegg.(bundet_av_event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2601,49 +2601,49 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>koe.jobb</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). En sak fra en topic i innboksen får ingen jobb; den kobles til topicen (W-1b.1, #819). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
+          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak` og triggeren `koe.leveringsoppdrag_levering`, og endres av `koe_api.hent_jobb`, `koe_api.kvitter_topic`, `koe_api.kvitter_levering`, `koe_api.registrer_jobbfeil` og driftsverktøyet `koe_api.start_jobb_paa_nytt`.</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2653,29 +2653,29 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Sakstittelen kan inneholde personopplysninger.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>koe.jobbforsoek</t>
+          <t>koe.jobb</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med SID-en til innloggingen som startet jobben på nytt (`sid:0x…`, eller `driften uten SID`). Raden endres ikke.</t>
+          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). En sak fra en topic i innboksen får ingen jobb; den kobles til topicen (W-1b.1, #819). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Prosedyrene for jobbkjøreren i `database/migrasjoner/20261018100000_jobber.sql`, og driftsverktøyet `koe_api.start_jobb_paa_nytt`, sist definert i `20261020121000_oppretter_tid_og_oppdragsnoekkel.sql`.</t>
+          <t>`koe_api.opprett_sak` og triggeren `koe.leveringsoppdrag_levering`, og endres av `koe_api.hent_jobb`, `koe_api.kvitter_topic`, `koe_api.kvitter_levering`, `koe_api.registrer_jobbfeil` og driftsverktøyet `koe_api.start_jobb_paa_nytt`.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2695,12 +2695,12 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Nei. Meldingen er fra klienten i `server/catenda.ts`, uten svarkropp. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.forsoek_id (uten fremmednøkkel); koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel); koe.vedleggskvittering.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2720,29 +2720,29 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Innloggingen til den i driften som startet en jobb på nytt.</t>
+          <t>Sakstittelen kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
+          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med SID-en til innloggingen som startet jobben på nytt (`sid:0x…`, eller `driften uten SID`). Raden endres ikke.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661).</t>
+          <t>Prosedyrene for jobbkjøreren i `database/migrasjoner/20261018100000_jobber.sql`, og driftsverktøyet `koe_api.start_jobb_paa_nytt`, sist definert i `20261020121000_oppretter_tid_og_oppdragsnoekkel.sql`.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2752,12 +2752,12 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Meldingen er fra klienten i `server/catenda.ts`, uten svarkropp. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id); unik (id, prosjekt_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.forsoek_id (uten fremmednøkkel); koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel); koe.vedleggskvittering.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -2777,19 +2777,19 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
+          <t>Innloggingen til den i driften som startet en jobb på nytt.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>koe.kvittering</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen per kommando (invariant 4, #418): kommando-ID-en klienten gir, summen av innholdet serveren regner ut, og saken og brevet kommandoen ga. Lagres i samme transaksjon som brevet. Nøkkelen er prosjektet, aktøren og kommando-ID-en, så kvitteringen gjelder aktøren. Samme ID med samme sum gir brevet fra kvitteringen, og samme ID med en annen sum avvises (51410).</t>
+          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`.</t>
+          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661).</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id); unik (id, prosjekt_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2834,19 +2834,19 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Aktørens `app_users.id`.</t>
+          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>koe.brevdokument</t>
+          <t>koe.kvittering</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>PDF-en av brevet i et leveringsoppdrag (#371 del 2, merknaden 12.10): bytene og SHA-256 av dem, lagret én gang per oppdrag før første opplasting. Kjøreren har kontrollert at PDF-en gjengir den frosne brevteksten tro (LV-U2), og laster opp den lagrede. Basen regner summen etter. Raden endres ikke, og bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en.</t>
+          <t>Kvitteringen per kommando (invariant 4, #418): kommando-ID-en klienten gir, summen av innholdet serveren regner ut, og saken og brevet kommandoen ga. Lagres i samme transaksjon som brevet. Nøkkelen er prosjektet, aktøren og kommando-ID-en, så kvitteringen gjelder aktøren. Samme ID med samme sum gir brevet fra kvitteringen, og samme ID med en annen sum avvises (51410).</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts` med PDF-en når samme prosedyre uten PDF ikke gir noen lagret for oppdraget (#795 punkt 4, #805 punkt 5).</t>
+          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2891,19 +2891,19 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Brevteksten kan ha navn på personer i prosjektet.</t>
+          <t>Aktørens `app_users.id`.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.brevdokument</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. `koe_api.bind_vedlegg` binder vedleggene hendelsen viser til, i samme transaksjon som hendelsen (V-2). Når Catenda har kvittert for dokumentet, setter `koe_api.kvitter_vedlegg` innholdet til NULL og beholder filnavnet og summen (LV-U12, V-3). Triggeren `koe.vedlegg_uten_endring` slipper bare gjennom de to endringene.</t>
+          <t>PDF-en av brevet i et leveringsoppdrag (#371 del 2, merknaden 12.10): bytene og SHA-256 av dem, lagret én gang per oppdrag før første opplasting. Kjøreren har kontrollert at PDF-en gjengir den frosne brevteksten tro (LV-U2), og laster opp den lagrede. Basen regner summen etter. Raden endres ikke, og bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`, `koe_api.bind_vedlegg`, kalt fra `server/kommandoer.ts`, og `koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts` med PDF-en når samme prosedyre uten PDF ikke gir noen lagret for oppdraget (#795 punkt 4, #805 punkt 5).</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2948,36 +2948,36 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Filen og filnavnet kan ha navn på personer i prosjektet.</t>
+          <t>Brevteksten kan ha navn på personer i prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (GFK-U1). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
+          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. `koe_api.bind_vedlegg` binder vedleggene hendelsen viser til, i samme transaksjon som hendelsen (V-2). Når Catenda har kvittert for dokumentet, setter `koe_api.kvitter_vedlegg` innholdet til NULL og beholder filnavnet og summen (LV-U12, V-3). Triggeren `koe.vedlegg_uten_endring` slipper bare gjennom de to endringene.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`, `koe_api.bind_vedlegg`, kalt fra `server/kommandoer.ts`, og `koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id, bruker_id); unik (prosjekt_id, plass). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3005,19 +3005,19 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Hvem som har fullmakt, med tittel og beløpsgrense.</t>
+          <t>Filen og filnavnet kan ha navn på personer i prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp som fullmaktene.</t>
+          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (GFK-U1). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, bruker_id); unik (prosjekt_id, plass). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3062,36 +3062,36 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Ingen.</t>
+          <t>Hvem som har fullmakt, med tittel og beløpsgrense.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
+          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp som fullmaktene.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -3119,19 +3119,19 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
+          <t>Ingen.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne i en pakke i kjedens rekkefølge, regnet av `server/fullmakt.ts` da pakken ble laget. Endres ikke.</t>
+          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3176,19 +3176,19 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne (`godkjenner_id`).</t>
+          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser tittelen og grensen godkjenneren hadde da den ble gitt, så den står om fullmakten endres senere (B-04 punkt 2). Endres ikke.</t>
+          <t>Godkjennerne i en pakke i kjedens rekkefølge, regnet av `server/fullmakt.ts` da pakken ble laget. Endres ikke.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3233,19 +3233,19 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
+          <t>Godkjennerne (`godkjenner_id`).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser tittelen og grensen godkjenneren hadde da den ble gitt, så den står om fullmakten endres senere (B-04 punkt 2). Endres ikke.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -3265,12 +3265,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3290,19 +3290,19 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3354,37 +3354,37 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3394,12 +3394,12 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -3411,12 +3411,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_hendelse</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3426,22 +3426,22 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3451,29 +3451,29 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
+          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
+          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3493,12 +3493,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
+          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3518,19 +3518,19 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
+          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_forsoek</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
+          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3550,12 +3550,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
+          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3575,19 +3575,19 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
+          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.topic_kommentar</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
+          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
+          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
+          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3632,19 +3632,19 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3689,19 +3689,19 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3753,12 +3753,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3803,19 +3803,19 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3850,29 +3850,29 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3892,12 +3892,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3907,72 +3907,129 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="J63" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K62" s="2" t="inlineStr">
+      <c r="K63" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>

</xml_diff>

<commit_message>
la driften registrere Entra-identiteten; innloggingen oppretter aldri en bruker
Del av #831

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NihFjDYkRdtR2U7uWfKhbU
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet` eller `koe_api.entra_identitet`, oppretter brukeren første gang en identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659) og `entraIdentitet` i `server/entra.ts` (S-1c del 1, #831).</t>
+          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en Catenda-identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659). En Entra-identitet oppretter aldri en bruker ved innloggingen: driften registrerer den med `koe_drift.registrer_entra_identitet`, som ny bruker eller koblet til en eksisterende (S-1c del 1, #831). `koe_api.entra_identitet` oppdaterer navn og e-post ved innloggingen.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659) og gjennom `koe_api.entra_identitet` fra tilbakekallet for Entra ID (S-1c del 1, #831).</t>
+          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659). En Entra-identitet registreres av driften med `koe_drift.registrer_entra_identitet` og slås bare opp av `koe_api.entra_identitet` ved innloggingen (S-1c del 1, #831).</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Tenantene i Entra ID driften har godkjent for innloggingen (S-1c del 1, #831). `koe_api.entra_identitet` avviser en issuer for en tenant som ikke står her. Kjøretiden har ingen rett på tabellen.</t>
+          <t>Tenantene i Entra ID driften har godkjent for innloggingen (S-1c del 1, #831). `koe_api.entra_identitet` og `koe_drift.registrer_entra_identitet` avviser en tenant som ikke står her. Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
legg til roller, stillingstitler og HR-kopien fra Graph med synkronisering i jobbkjøreren
S-1c del 2 (#831): driften registrerer grensen per rolle og hvilken
stillingstittel som gir hvilken rolle (GFK-U6, GFK-U11, S3). Jobbkjøreren
synkroniserer HR-kopien fra Graph hver time med koe_api.synkroniser_hr,
som registrerer Entra-identiteten for alle med en stilling som gir rolle
(svaret 20.10 i #831) og lar en mistet rolle synes (GFK-U10).

Del av #831.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rdtz2rnWigttjP66Up2wt3
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningshandling.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningspakke.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.godkjenner_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningshandling.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningspakke.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.godkjenner_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.hr_kopi.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2157,12 +2157,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.rolle</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene. `id` er prosjektgrensen i alle tabellene med saksdata, uten standardverdi (AGENTS.md). `server/prosjekter.ts` leser prosjektene aktøren er aktivt medlem i med `koe_api.brukerens_prosjekter`, og ett av dem med `koe_api.prosjekt` (#660). Tabellen har ikke `settings` og `created_by` fra PostgreSQL.</t>
+          <t>Rollene byggherren gir fullmakt etter, med beløpsgrensen i kroner, globalt for byggherren (GFK-U6, GFK-U11; S-1c del 2, #831). Ingen grense er ubegrenset (GFK-U4). Rollen er en kode med a–z og `_`. Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten; skriptet sier fra når `--organisasjon` er en annen (#836).</t>
+          <t>Driften, med `koe_drift.sett_rolle` og `koe_drift.fjern_rolle`.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2182,12 +2182,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Navnet oppgis av driften; i Python kan det hentes fra Catenda-prosjektet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (rolle). Vises til fra: koe.hr_kopi.rolle (fremmednøkkel, ON DELETE NO ACTION); koe.stillingstittel.rolle (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2202,24 +2202,24 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>koe.app_project_memberships</t>
+          <t>koe.stillingstittel</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660). `koe_api.medlemmer`, også kalt derfra, leser de aktive medlemmene for en aktør med aktivt medlemskap (#820).</t>
+          <t>Hvilken stillingstittel (`jobTitle` i Graph) som gir hvilken rolle (S3 i #831). Tittelen må stemme tegn for tegn; nøkkelen er SHA-256 av tittelen, fordi `=` ser bort fra mellomrom til slutt. Kjøretiden leser titlene bare gjennom `koe_api.stillingstitler`.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2229,22 +2229,22 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10). `koe_api.sett_leserolle`, kalt fra `server/prosjekter.ts`, setter `viewer_override` for et annet aktivt medlem når aktøren er aktiv admin uten leserolle (#820).</t>
+          <t>Driften, med `koe_drift.sett_stillingstittel` og `koe_drift.fjern_stillingstittel`. Lest av `koe_api.stillingstitler` og `koe_api.synkroniser_hr` fra `server/hrdata.ts`.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Delvis</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Ja, medlemslisten i Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (noekkel). Viser til: rolle → koe.rolle.rolle (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>grunndata, kopi</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2264,19 +2264,19 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>E-post og visningsnavn.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.hr_kopi</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen. `server/autorisasjon.ts` leser prosjektets kontraktsteam med `koe_api.kontraktsteam`, bare for en aktør med aktivt medlemskap uten leserollen (#658).</t>
+          <t>HR-kopien per bruker fra Graph (S-1c del 2, #831): tenanten, `oid`, rollen, lederens `oid` og når bildet ble hentet. Hver synkronisering skriver hele bildet for tenanten; en person uten en stilling som gir rolle, eller med deaktivert konto, beholder raden uten rolle og leder (GFK-U10). Kjøretiden skriver bare gjennom `koe_api.synkroniser_hr` og har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2286,22 +2286,22 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764). Byttes Catenda-prosjektet, må teamene oppgis på nytt (#836).</t>
+          <t>`koe_api.synkroniser_hr`, kalt av jobbkjøreren gjennom `synkroniserHr` i `server/hrdata.ts`.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Fra Microsoft Graph. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.aktor_team_id (uten fremmednøkkel); koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (bruker_id); unik (tenant_id, oid). Viser til: bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); rolle → koe.rolle.rolle (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2311,29 +2311,29 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>kopi</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Hvem som har en rolle med fullmakt, og hvem som er lederen.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_project_configs</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660). Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10), og setter Catenda-ID-en i synkroniseringsraden til NULL. Den tomme Catenda-ID-en er ikke lov. `topic_board_id` er boardet for saker som opprettes i appen (KT-U4); uten det avviser `koe_api.opprett_sak` saken (#741). `koe_api.opprett_sak` låser raden før den leses, så en ny sak og en ny registrering eller nye kontraktsteam skrives etter hverandre (#868). Triggeren `koe.catenda_project_configs_endret` setter `updated_at` ved hver endring (#618).</t>
+          <t>Prosjektene. `id` er prosjektgrensen i alle tabellene med saksdata, uten standardverdi (AGENTS.md). `server/prosjekter.ts` leser prosjektene aktøren er aktivt medlem i med `koe_api.brukerens_prosjekter`, og ett av dem med `koe_api.prosjekt` (#660). Tabellen har ikke `settings` og `created_by` fra PostgreSQL.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet og biblioteket og gjør koblingen aktiv. Mappen og boardet skrives over når de er oppgitt. Ellers står de hvis Catenda-prosjektet er det samme, og fjernes hvis det er byttet. Mappen fjernes også når biblioteket er byttet. Har prosjektet saker, avvises bytte av Catenda-prosjekt, og uten saker krever et bytte nye kontraktsteam (#836).</t>
+          <t>Driften registrerer prosjektet med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt`; bare `koe_driftsrolle` kan kjøre den (F-1, #820). En ny registrering skriver over navnet og beskrivelsen og gjør prosjektet aktivt, men endrer ikke virksomheten; skriptet sier fra når `--organisasjon` er en annen (#836).</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2353,12 +2353,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Navnet oppgis av driften; i Python kan det hentes fra Catenda-prosjektet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2385,12 +2385,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_absences</t>
+          <t>koe.app_project_memberships</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene der innloggingens liste over brukerens Catenda-prosjekter viste at brukeren ikke er med, for en bruker uten medlemskap der (DL-U9). `observed_at` er når innloggingens liste ble hentet, etter basens klokke. En medlemsliste hentet samtidig eller før gir ikke brukeren et nytt medlemskap. Har ingen tabell i PostgreSQL.</t>
+          <t>Medlemskapet i et prosjekt, fra Catenda. Leserollen er `viewer_override`, som i PostgreSQL. `server/autorisasjon.ts` leser aktørens aktive medlemskap med `koe_api.prosjektmedlemskap` (#658). `koe_api.brukerens_prosjekter` og `koe_api.prosjekt`, kalt fra `server/prosjekter.ts`, leser bare prosjekter der aktøren har et aktivt medlemskap (#660). `koe_api.medlemmer`, også kalt derfra, leser de aktive medlemmene for en aktør med aktivt medlemskap (#820).</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2400,22 +2400,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Innloggingen kaller modulen fra tilbakekallet i `server/innlogging.ts` (F0b-5b).</t>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, skriver medlemslisten fra Catenda og gjør medlemmer som ikke står i den, inaktive. `koe_api.deaktiver_ved_innlogging`, også kalt derfra, gjør brukerens medlemskap inaktivt i koblede prosjekter som ikke står i brukerens liste fra Catenda. `deactivated_at` er når medlemskapet sist ble gjort inaktivt, etter basens klokke; en liste hentet før det gjør det ikke aktivt igjen (DL-U8). For en bruker uten medlemskap fører innloggingen en rad i `koe.app_membership_absences`, og en liste hentet før den gir ikke et nytt medlemskap (DL-U9). Tilgangskontrollen i `server/autorisasjon.ts` og tilbakekallet i `server/innlogging.ts` kaller modulen (F0b-5b). Blir koblingen opphevet, slettet eller endret, gjør triggeren `koe.catenda_project_configs_kobling_endret` alle medlemskapene i prosjektet inaktive med `deactivated_at` satt til tidspunktet for endringen (DL-U10). `koe_api.sett_leserolle`, kalt fra `server/prosjekter.ts`, setter `viewer_override` for et annet aktivt medlem når aktøren er aktiv admin uten leserolle (#820).</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Delvis</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, medlemslisten i Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id, user_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id, user_id); unik (project_id, catenda_subject). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>grunndata, kopi</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2435,19 +2435,19 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med prosjektene brukeren ikke er med i og tidspunktene for innloggingene (`observed_at`, `updated_at`).</t>
+          <t>E-post og visningsnavn.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>koe.app_membership_sync</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også gjennom `ferskeMedlemmer` for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden ingen Catenda-ID (NULL) og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10, #726). Den tomme Catenda-ID-en er ikke lov.</t>
+          <t>Kontraktssiden (TE eller BH) for hvert Catenda-team i et prosjekt. Teamet har `catenda_id()`-formen, som `aktor_team_id` i journalen. `server/autorisasjon.ts` leser prosjektets kontraktsteam med `koe_api.kontraktsteam`, bare for en aktør med aktivt medlemskap uten leserollen (#658).</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, og triggeren `koe.catenda_project_configs_kobling_endret` når koblingen endres.</t>
+          <t>Driften setter teamene med skriptet `server/registrering.ts`, som kontrollerer dem mot Catenda-prosjektet og kaller `koe_drift.sett_kontraktsteam`, direkte eller gjennom `koe_drift.registrer_prosjekt` (F-1, #820). Begge sider må ha minst ett team. Uten saker erstatter listen teamene; står prosjektet i `koe.prosjekt_med_saker`, kan de bare få nye team (svaret 18.10 i #764). Byttes Catenda-prosjektet, må teamene oppgis på nytt (#836).</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2467,12 +2467,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id, team_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.aktor_team_id (uten fremmednøkkel); koe.hendelse.aktor_team_id (uten fremmednøkkel); koe.notat.aktor_team_id (uten fremmednøkkel); koe.vedlegg.lastet_opp_team (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2499,37 +2499,37 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.catenda_project_configs</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
+          <t>Koblingen mellom prosjektet i appen og Catenda-prosjektet, og om den er aktiv (arbeidsvalget 16.10 i #53). Svarer til `catenda_project_configs` i PostgreSQL, uten mappene for webhooken. Synkroniseringen avviser en liste fra et annet Catenda-prosjekt. `server/medlemskap.ts` leser en aktiv kobling med `koe_api.prosjektkobling` (#658, #638), og `koe_api.koblede_prosjekter` gir prosjektene koblet til brukerens Catenda-prosjekter ved innlogging. `koe_api.brukerens_prosjekter`, kalt fra `server/prosjekter.ts`, tar bare med prosjekter med aktiv kobling (#660). Triggeren `koe.catenda_project_configs_kobling_endret` gjør medlemskapene inaktive når koblingen oppheves, slettes eller endres (DL-U10), og setter Catenda-ID-en i synkroniseringsraden til NULL. Den tomme Catenda-ID-en er ikke lov. `topic_board_id` er boardet for saker som opprettes i appen (KT-U4); uten det avviser `koe_api.opprett_sak` saken (#741). `koe_api.opprett_sak` låser raden før den leses, så en ny sak og en ny registrering eller nye kontraktsteam skrives etter hverandre (#868). Triggeren `koe.catenda_project_configs_endret` setter `updated_at` ved hver endring (#618).</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Driften registrerer koblingen med skriptet `server/registrering.ts`, som kaller `koe_drift.registrer_prosjekt` (F-1, #820). En ny registrering skriver over Catenda-prosjektet og biblioteket og gjør koblingen aktiv. Mappen og boardet skrives over når de er oppgitt. Ellers står de hvis Catenda-prosjektet er det samme, og fjernes hvis det er byttet. Mappen fjernes også når biblioteket er byttet. Har prosjektet saker, avvises bytte av Catenda-prosjekt, og uten saker krever et bytte nye kontraktsteam (#836).</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370), og som `server/hendelser.ts` kaller for en ny topic fra TE i innboksen (KT-U6, #819).</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Saken kan være opprettet fra en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_behandling.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (internal_project_id); unik (catenda_project_id). Viser til: internal_project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2539,54 +2539,54 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`created_by` peker på en bruker.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>koe.hendelse</t>
+          <t>koe.app_membership_absences</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
+          <t>Prosjektene der innloggingens liste over brukerens Catenda-prosjekter viste at brukeren ikke er med, for en bruker uten medlemskap der (DL-U9). `observed_at` er når innloggingens liste ble hentet, etter basens klokke. En medlemsliste hentet samtidig eller før gir ikke brukeren et nytt medlemskap. Har ingen tabell i PostgreSQL.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.deaktiver_ved_innlogging`, kalt fra `server/medlemskap.ts`, setter inn raden eller flytter `observed_at` fram. `koe_api.synkroniser_medlemskap` sletter radene i prosjektet med `observed_at` før listen den skriver. Innloggingen kaller modulen fra tilbakekallet i `server/innlogging.ts` (F0b-5b).</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661), og `koe_api.opprett_sak` fra `POST /api/kjerne/saker` (#370).</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Sakstittelen i `sak_opprettet` kan være tittelen på en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel); koe.vedlegg.(bundet_av_event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (project_id, user_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2606,44 +2606,44 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med prosjektene brukeren ikke er med i og tidspunktene for innloggingene (`observed_at`, `updated_at`).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>koe.notat</t>
+          <t>koe.app_membership_sync</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
+          <t>Når medlemslisten for prosjektet sist ble hentet, og fra hvilket Catenda-prosjekt (DL-U7). En eldre liste skriver ikke over en nyere. Alderen leses av `koe_api.medlemsliste_alder` (B-04 punkt 4), kalt fra `server/autorisasjon.ts` etter at koblingen er kontrollert (#638 punkt 2), også gjennom `ferskeMedlemmer` for hvert prosjekt i lista i `server/prosjekter.ts` (#660). Svarer til `app_membership_sync` i PostgreSQL. Etter at koblingen er opphevet, slettet eller endret, har raden ingen Catenda-ID (NULL) og tidspunktet for endringen, så ingen liste fra det koblede prosjektet finnes, og en liste hentet før endringen ikke skrives (DL-U10, #726). Den tomme Catenda-ID-en er ikke lov.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.synkroniser_medlemskap`, kalt fra `server/medlemskap.ts`, og triggeren `koe.catenda_project_configs_kobling_endret` når koblingen endres.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Tidspunktet er når hentingen fra Catenda begynte. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (project_id). Viser til: project_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2653,54 +2653,54 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>koe.jobb</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). En sak fra en topic i innboksen får ingen jobb; den kobles til topicen (W-1b.1, #819). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sak`, sammen med `sak_opprettet`, kalt fra `opprettSak` i `server/kommandoer.ts`, som `POST /api/kjerne/saker` kaller (#370), og som `server/hendelser.ts` kaller for en ny topic fra TE i innboksen (KT-U6, #819).</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_sak` og triggeren `koe.leveringsoppdrag_levering`, og endres av `koe_api.hent_jobb`, `koe_api.kvitter_topic`, `koe_api.kvitter_levering`, `koe_api.registrer_jobbfeil` og driftsverktøyet `koe_api.start_jobb_paa_nytt`.</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Saken kan være opprettet fra en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (sak_id, prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); created_by → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningspakke.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_behandling.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.kjernebuffer.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.sak_catenda_topic.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2720,44 +2720,44 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Sakstittelen kan inneholde personopplysninger.</t>
+          <t>`created_by` peker på en bruker.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>koe.jobbforsoek</t>
+          <t>koe.hendelse</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med SID-en til innloggingen som startet jobben på nytt (`sid:0x…`, eller `driften uten SID`). Raden endres ikke.</t>
+          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sak` skriver `sak_opprettet` og `koe_api.skriv_hendelse` de andre brevene, kalt fra `server/kommandoer.ts`. `koe_api.skriv_hendelse` kalles fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661), og `koe_api.opprett_sak` fra `POST /api/kjerne/saker` (#370).</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Prosedyrene for jobbkjøreren i `database/migrasjoner/20261018100000_jobber.sql`, og driftsverktøyet `koe_api.start_jobb_paa_nytt`, sist definert i `20261020121000_oppretter_tid_og_oppdragsnoekkel.sql`.</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Nei. Meldingen er fra klienten i `server/catenda.ts`, uten svarkropp. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Sakstittelen i `sak_opprettet` kan være tittelen på en topic i Catenda (KT-U6, C22). Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.forsoek_id (uten fremmednøkkel); koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel); koe.vedleggskvittering.forsoek_id (uten fremmednøkkel).</t>
+          <t>Nøkler: primærnøkkel (event_id); unik (event_id, sak_id, prosjekt_id); unik (sak_id, versjon). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel). Vises til fra: koe.kvittering.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringsoppdrag.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.notat.refererer_til_event_id (uten fremmednøkkel); koe.vedlegg.(bundet_av_event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -2777,19 +2777,19 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Innloggingen til den i driften som startet en jobb på nytt.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `data` kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringsoppdrag</t>
+          <t>koe.notat</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
+          <t>Interne notater, skjermet på teamet (AGENTS.md). Ikke et kontraktsvarsel, og kan endres og slettes (MS-05).</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id); unik (id, prosjekt_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (notat_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel); refererer_til_event_id → koe.hendelse.event_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2829,34 +2829,34 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
+          <t>`aktor_id` peker på en bruker. Fritekst i `tekst` og `kommentar`.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>koe.kvittering</t>
+          <t>koe.jobb</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen per kommando (invariant 4, #418): kommando-ID-en klienten gir, summen av innholdet serveren regner ut, og saken og brevet kommandoen ga. Lagres i samme transaksjon som brevet. Nøkkelen er prosjektet, aktøren og kommando-ID-en, så kvitteringen gjelder aktøren. Samme ID med samme sum gir brevet fra kvitteringen, og samme ID med en annen sum avvises (51410).</t>
+          <t>Jobbene jobbkjøreren gjør etter commit (B-07, arbeidsvalget 18.10 i #741). En sak fra appen får jobben `catenda_topic` i samme transaksjon, med boardet, Catenda-prosjektet og sakstittelen frosset (KT-U3, invariant 6). En sak fra en topic i innboksen får ingen jobb; den kobles til topicen (W-1b.1, #819). Et brev med tekst fra appen får jobben `levering` for leveringsoppdraget, lagt inn av triggeren `koe.leveringsoppdrag_levering` (#371). Jobben har en lease mens den gjøres, og tilstanden `venter`, `utfoert` eller `parkert`. Bare kjøreveien, `koe_jobbkjoerer`, ser og endrer jobbene; kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`.</t>
+          <t>`koe_api.opprett_sak` og triggeren `koe.leveringsoppdrag_levering`, og endres av `koe_api.hent_jobb`, `koe_api.kvitter_topic`, `koe_api.kvitter_levering`, `koe_api.registrer_jobbfeil` og driftsverktøyet `koe_api.start_jobb_paa_nytt`.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2866,12 +2866,12 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. ID-ene til Catenda-prosjektet og boardet. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (jobb_id); unik indeks (lease) WHERE ([lease] IS NOT NULL); unik indeks (leveringsoppdrag_id) WHERE ([leveringsoppdrag_id] IS NOT NULL); unik indeks (sak_id) WHERE ([jobbtype]=N'catenda_topic'). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); siste_forsoek → koe.jobbforsoek.forsoek_id (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.jobbforsoek.jobb_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2891,29 +2891,29 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Aktørens `app_users.id`.</t>
+          <t>Sakstittelen kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>koe.brevdokument</t>
+          <t>koe.jobbforsoek</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>PDF-en av brevet i et leveringsoppdrag (#371 del 2, merknaden 12.10): bytene og SHA-256 av dem, lagret én gang per oppdrag før første opplasting. Kjøreren har kontrollert at PDF-en gjengir den frosne brevteksten tro (LV-U2), og laster opp den lagrede. Basen regner summen etter. Raden endres ikke, og bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en.</t>
+          <t>Hvert forsøk, hver feil, hver kvittering og hver omstart av en jobb for seg (LV-U1, invariant 7 og 8). Forsøket har leasens ID og lagres når utfallet er kjent: `utfoert`, `feilet`, `usikkert`, `avvist`, `kobling_endret` eller `startet_paa_nytt`, med SID-en til innloggingen som startet jobben på nytt (`sid:0x…`, eller `driften uten SID`). Raden endres ikke.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts` med PDF-en når samme prosedyre uten PDF ikke gir noen lagret for oppdraget (#795 punkt 4, #805 punkt 5).</t>
+          <t>Prosedyrene for jobbkjøreren i `database/migrasjoner/20261018100000_jobber.sql`, og driftsverktøyet `koe_api.start_jobb_paa_nytt`, sist definert i `20261020121000_oppretter_tid_og_oppdragsnoekkel.sql`.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2923,12 +2923,12 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Meldingen er fra klienten i `server/catenda.ts`, uten svarkropp. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (forsoek_id). Viser til: jobb_id → koe.jobb.jobb_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.forsoek_id (uten fremmednøkkel); koe.jobb.siste_forsoek (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.forsoek_id (uten fremmednøkkel); koe.vedleggskvittering.forsoek_id (uten fremmednøkkel).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2948,19 +2948,19 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Brevteksten kan ha navn på personer i prosjektet.</t>
+          <t>Innloggingen til den i driften som startet en jobb på nytt.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>koe.vedlegg</t>
+          <t>koe.leveringsoppdrag</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. `koe_api.bind_vedlegg` binder vedleggene hendelsen viser til, i samme transaksjon som hendelsen (V-2). Når Catenda har kvittert for dokumentet, setter `koe_api.kvitter_vedlegg` innholdet til NULL og beholder filnavnet og summen (LV-U12, V-3). Triggeren `koe.vedlegg_uten_endring` slipper bare gjennom de to endringene.</t>
+          <t>Leveringsoppdraget for et brev (LV-U1, B-03), frosset i samme transaksjon som brevet. Den sammensatte fremmednøkkelen holder det i brevets sak og prosjekt.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`, `koe_api.bind_vedlegg`, kalt fra `server/kommandoer.ts`, og `koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.skriv_hendelse`, med brevet `dokument_registrert` i samme transaksjon, kalt fra `skrivHendelse` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer` (#661).</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei, men oppdraget gjelder en levering til Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik (dokumentnoekkel); unik (event_id); unik (id, prosjekt_id). Viser til: (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.brevdokument.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.jobb.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.leveringskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.(leveringsoppdrag_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -3005,36 +3005,36 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Filen og filnavnet kan ha navn på personer i prosjektet.</t>
+          <t>Innholdet er brevet og kan inneholde personopplysninger.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.kvittering</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (GFK-U1). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
+          <t>Kvitteringen per kommando (invariant 4, #418): kommando-ID-en klienten gir, summen av innholdet serveren regner ut, og saken og brevet kommandoen ga. Lagres i samme transaksjon som brevet. Nøkkelen er prosjektet, aktøren og kommando-ID-en, så kvitteringen gjelder aktøren. Samme ID med samme sum gir brevet fra kvitteringen, og samme ID med en annen sum avvises (51410).</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`.</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id, bruker_id); unik (prosjekt_id, plass). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, aktor_id, kommando_id); unik (event_id). Viser til: aktor_id → koe.app_users.id (uten fremmednøkkel); (event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -3062,36 +3062,36 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Hvem som har fullmakt, med tittel og beløpsgrense.</t>
+          <t>Aktørens `app_users.id`.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.brevdokument</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp som fullmaktene.</t>
+          <t>PDF-en av brevet i et leveringsoppdrag (#371 del 2, merknaden 12.10): bytene og SHA-256 av dem, lagret én gang per oppdrag før første opplasting. Kjøreren har kontrollert at PDF-en gjengir den frosne brevteksten tro (LV-U2), og laster opp den lagrede. Basen regner summen etter. Raden endres ikke, og bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.lagre_brevdokument`, kalt av jobbkjøreren i `server/jobber.ts` med PDF-en når samme prosedyre uten PDF ikke gir noen lagret for oppdraget (#795 punkt 4, #805 punkt 5).</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.brevdokument_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -3119,19 +3119,19 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Ingen.</t>
+          <t>Brevteksten kan ha navn på personer i prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.vedlegg</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
+          <t>Mellomlageret for vedlegg (V-1, del av #790): filen, filnavnet, størrelsen og SHA-256 av bytene, som basen regner etter. Filen ligger her til Catenda har kvittert for den (spørsmål 1 A i #790, 18.10). Et ubundet vedlegg er et utkast som bare teamet som lastet det opp, ser og sletter. Når en hendelse viser til det, får det `bundet_av_event_id` og ses av begge kontraktssider; et bundet vedlegg slettes ikke. `koe_api.bind_vedlegg` binder vedleggene hendelsen viser til, i samme transaksjon som hendelsen (V-2). Når Catenda har kvittert for dokumentet, setter `koe_api.kvitter_vedlegg` innholdet til NULL og beholder filnavnet og summen (LV-U12, V-3). Triggeren `koe.vedlegg_uten_endring` slipper bare gjennom de to endringene.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
+          <t>`koe_api.lagre_vedlegg` og `koe_api.slett_vedlegg`, kalt fra `server/vedlegg.ts`, `koe_api.bind_vedlegg`, kalt fra `server/kommandoer.ts`, og `koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_av → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); (bundet_av_event_id, sak_id, prosjekt_id) → koe.hendelse.(event_id, sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); lastet_opp_team → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); koe.vedleggskvittering.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3176,36 +3176,36 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
+          <t>Filen og filnavnet kan ha navn på personer i prosjektet.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.fullmakt</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne i en pakke i kjedens rekkefølge, regnet av `server/fullmakt.ts` da pakken ble laget. Endres ikke.</t>
+          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (GFK-U1). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id, bruker_id); unik (prosjekt_id, plass). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3233,36 +3233,36 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne (`godkjenner_id`).</t>
+          <t>Hvem som har fullmakt, med tittel og beløpsgrense.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser tittelen og grensen godkjenneren hadde da den ble gitt, så den står om fullmakten endres senere (B-04 punkt 2). Endres ikke.</t>
+          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp som fullmaktene.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3290,19 +3290,19 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
+          <t>Ingen.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -3322,12 +3322,12 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3347,19 +3347,19 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
+          <t>Godkjennerne i en pakke i kjedens rekkefølge, regnet av `server/fullmakt.ts` da pakken ble laget. Endres ikke.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3379,12 +3379,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3404,44 +3404,44 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Godkjennerne (`godkjenner_id`).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser tittelen og grensen godkjenneren hadde da den ble gitt, så den står om fullmakten endres senere (B-04 punkt 2). Endres ikke.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3451,54 +3451,54 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_hendelse</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3518,44 +3518,44 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
+          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -3575,19 +3575,19 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_forsoek</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,22 +3597,22 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3622,29 +3622,29 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.topic_kommentar</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
+          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
+          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
+          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3689,19 +3689,19 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3746,19 +3746,19 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3803,19 +3803,19 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3835,12 +3835,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3867,12 +3867,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3892,12 +3892,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3907,29 +3907,29 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3949,12 +3949,12 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3974,62 +3974,233 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>koe.toemmingsvern</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Nei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>koe.kjernebuffer</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Ingen skriver ennå (#53, del 3).</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>avledet</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>uavklart</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Som journalen den er regnet fra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -4046,7 +4217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H129"/>
+  <dimension ref="A1:H132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9274,6 +9445,132 @@
       <c r="H129" s="2" t="inlineStr">
         <is>
           <t>Den som godkjente, returnerte eller trakk pakken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>koe.stillingstittel</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>rolle</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>koe.rolle</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>rolle</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Rollen stillingstittelen gir (S3 i #831).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>koe.hr_kopi</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>bruker_id</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Brukeren HR-kopien gjelder. Synkroniseringen registrerer Entra-identiteten når den mangler (svaret 20.10 i #831).</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>koe.hr_kopi</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>rolle</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>koe.rolle</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>rolle</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>mange til én</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Rollen personen har etter siste synkronisering, eller ingen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
legg til driftsprosedyren som kobler Catenda-identiteten til HR-brukeren
koe_drift.koble_catenda_identitet registrerer en Catenda-identitet på en
bruker med Entra-identitet. Står identiteten på en bruker som bare har
medlemskap, fravær og sesjoner, flyttes den, og den brukeren slettes;
ellers avvises koblingen (#1002).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NApQhxr4aktDczumkjcwDj
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en Catenda-identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659). En Entra-identitet oppretter aldri en bruker ved innloggingen: driften registrerer den med `koe_drift.registrer_entra_identitet`, som ny bruker eller koblet til en eksisterende (S-1c del 1, #831). `koe_api.entra_identitet` oppdaterer navn og e-post ved innloggingen.</t>
+          <t>`koe.resolve_identity`, kalt gjennom `koe_api.catenda_identitet`, oppretter brukeren første gang en Catenda-identitet sees. Tilbakekallet fra innloggingen kaller den fra `catendaIdentitet` i `server/innlogging.ts` (F0b-5a, #659). En Entra-identitet oppretter aldri en bruker ved innloggingen: driften registrerer den med `koe_drift.registrer_entra_identitet`, som ny bruker eller koblet til en eksisterende (S-1c del 1, #831). `koe_api.entra_identitet` oppdaterer navn og e-post ved innloggingen. `koe_drift.koble_catenda_identitet` kobler en Catenda-identitet til en bruker med Entra-identitet og sletter brukeren identiteten stod på, når den bare har medlemskap, fravær og sesjoner (#1002).</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659). En Entra-identitet registreres av driften med `koe_drift.registrer_entra_identitet` og slås bare opp av `koe_api.entra_identitet` ved innloggingen (S-1c del 1, #831).</t>
+          <t>`koe.resolve_identity`, sammen med brukeren, kalt gjennom `koe_api.catenda_identitet` fra tilbakekallet i `server/innlogging.ts` (F0b-5a, #659). En Entra-identitet registreres av driften med `koe_drift.registrer_entra_identitet` og slås bare opp av `koe_api.entra_identitet` ved innloggingen (S-1c del 1, #831). Driften kobler en Catenda-identitet til en bruker med Entra-identitet med `koe_drift.koble_catenda_identitet`, som flytter identiteten bare når brukeren den stod på, ikke er brukt utover medlemskap, fravær og sesjoner; det er den eneste slettingen triggeren slipper gjennom (#1002).</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">

</xml_diff>

<commit_message>
avled godkjenningskjeden av hierarkiet i HR-kopien og fas ut koe.fullmakt
Del av #831 og #1003.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158HhZDn5qTmkwaNqMeMX7Z
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningshandling.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningspakke.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.godkjenner_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.hr_kopi.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_identities.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_absences.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_sessions.user_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningshandling.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningspakke.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.godkjenner_id (fremmednøkkel, ON DELETE NO ACTION); koe.hendelse.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.hr_kopi.bruker_id (fremmednøkkel, ON DELETE NO ACTION); koe.kvittering.aktor_id (uten fremmednøkkel); koe.notat.aktor_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.created_by (fremmednøkkel, ON DELETE NO ACTION); koe.vedlegg.lastet_opp_av (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rollene byggherren gir fullmakt etter, med beløpsgrensen i kroner, globalt for byggherren (GFK-U6, GFK-U11; S-1c del 2, #831). Ingen grense er ubegrenset (GFK-U4). Rollen er en kode med a–z og `_`. Kjøretiden har ingen rett på tabellen.</t>
+          <t>Rollene byggherren gir fullmakt etter, med beløpsgrensen i kroner, globalt for byggherren (GFK-U6, GFK-U11; S-1c del 2, #831). Ingen grense er ubegrenset (GFK-U4). Rollen er en kode med a–z og `_`. Kjøretiden har ingen rett på tabellen. `koe_api.godkjenningskjede` leser grensen når kjeden avledes, og `koe_api.registrer_godkjenningshandling` fryser rollen og grensen i godkjenningen (S-1c del 3).</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>HR-kopien per bruker fra Graph (S-1c del 2, #831): tenanten, `oid`, rollen, lederens `oid` og når bildet ble hentet. Hver synkronisering skriver hele bildet for tenanten; en person uten en stilling som gir rolle, eller med deaktivert konto, beholder raden uten rolle og leder (GFK-U10). Kjøretiden skriver bare gjennom `koe_api.synkroniser_hr` og har ingen rett på tabellen.</t>
+          <t>HR-kopien per bruker fra Graph (S-1c del 2, #831): tenanten, `oid`, rollen, lederens `oid` og når bildet ble hentet. Hver synkronisering skriver hele bildet for tenanten; en person uten en stilling som gir rolle, eller med deaktivert konto, beholder raden uten rolle og leder (GFK-U10). Kjøretiden skriver bare gjennom `koe_api.synkroniser_hr` og har ingen rett på tabellen. Godkjenningskjeden avledes av lederne i kopien (GFK-U8) i `koe_api.godkjenningskjede`, og en rad leses bare når den er hentet for under 24 timer siden og tenanten er godkjent (S-1c del 3).</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.fullmakt.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3183,12 +3183,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Byggherrens fullmakter i prosjektet (S-1a, #818): personen, tittelen, grensen i kroner (ingen grense er ubegrenset) og plassen i godkjenningskjeden. Driften setter dem opp etter skriftlig bestilling fra byggherren, og appen viser ikke hvem som har endret dem (GFK-U1). Kjøretiden leser dem bare gjennom `koe_api.fullmakter`, som byggherren.</t>
+          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
+          <t>Driften, som eier. Lest av `koe_api.dagmulktssats` fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id, bruker_id); unik (prosjekt_id, plass). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION); bruker_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3233,36 +3233,36 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Hvem som har fullmakt, med tittel og beløpsgrense.</t>
+          <t>Ingen.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Dagmulktssatsen i prosjektet, som fristdagene verdsettes med i fullmakten (GFK-06). Uten rad mangler satsen, og fristdagene kan ikke verdsettes (B-06). Driften setter den opp som fullmaktene.</t>
+          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, verdien kjeden ble avledet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Driften, som eier. Lest av `koe_api.fullmakter` fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3290,19 +3290,19 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Ingen.</t>
+          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
+          <t>Godkjennerne i en pakke i kjedens rekkefølge, avledet av hierarkiet i `koe.hr_kopi` da pakken ble laget (GFK-U8, GFK-U10). Endres ikke.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3347,19 +3347,19 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
+          <t>Godkjennerne (`godkjenner_id`).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne i en pakke i kjedens rekkefølge, regnet av `server/fullmakt.ts` da pakken ble laget. Endres ikke.</t>
+          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser rollen (`fullmakt_tittel`) og grensen godkjenneren hadde i `koe.rolle` da den ble gitt, så den står om rollen endres senere (B-04 punkt 2). Endres ikke.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
+          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3404,19 +3404,19 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne (`godkjenner_id`).</t>
+          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser tittelen og grensen godkjenneren hadde da den ble gitt, så den står om fullmakten endres senere (B-04 punkt 2). Endres ikke.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3436,12 +3436,12 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3461,19 +3461,19 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3525,37 +3525,37 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3565,12 +3565,12 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -3582,12 +3582,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,22 +3597,22 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
+          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nei</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3622,29 +3622,29 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_hendelse</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
+          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
+          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3689,19 +3689,19 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
+          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
+          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
+          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
+          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3746,19 +3746,19 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
+          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_forsoek</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
+          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
+          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
+          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3803,19 +3803,19 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>koe.topic_kommentar</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3835,12 +3835,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3860,19 +3860,19 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3892,12 +3892,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3924,12 +3924,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3974,19 +3974,19 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -4021,29 +4021,29 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.app_sessions</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -4063,12 +4063,12 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -4078,29 +4078,29 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.app_oauth_attempts</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -4120,12 +4120,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -4144,63 +4144,6 @@
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
-        <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>koe.app_oauth_attempts</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>SQL Server</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>teknisk</t>
-        </is>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>i bruk</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -4217,7 +4160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H132"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8951,7 +8894,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.dagmulktssats</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -8986,29 +8929,29 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet fullmakten gjelder i. Driften setter den opp (GFK-U1).</t>
+          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>koe.fullmakt</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -9028,29 +8971,29 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Personen som har fullmakten.</t>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>koe.dagmulktssats</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>prosjekt_id</t>
+          <t>forrige_pakke_id</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>koe.projects</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>pakke_id</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -9070,7 +9013,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Prosjektet satsen gjelder i. Uten rad mangler satsen (B-06).</t>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
         </is>
       </c>
     </row>
@@ -9082,17 +9025,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -9112,7 +9055,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
         </is>
       </c>
     </row>
@@ -9124,22 +9067,22 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -9147,36 +9090,32 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G122" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
+          <t>koe.godkjenningssteg</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
           <t>koe.godkjenningspakke</t>
         </is>
       </c>
-      <c r="B123" s="2" t="inlineStr">
-        <is>
-          <t>aktor_id</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t>koe.app_users</t>
-        </is>
-      </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -9196,34 +9135,34 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>godkjenner_id</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -9231,17 +9170,21 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G124" s="2" t="inlineStr"/>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Godkjenneren i steget.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -9276,29 +9219,29 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
+          <t>koe.godkjenningshandling</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>(pakke_id, steg)</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
           <t>koe.godkjenningssteg</t>
         </is>
       </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>godkjenner_id</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>koe.app_users</t>
-        </is>
-      </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(pakke_id, steg)</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -9318,7 +9261,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
         </is>
       </c>
     </row>
@@ -9330,17 +9273,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -9360,29 +9303,29 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.stillingstittel</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>rolle</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.rolle</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>rolle</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -9402,19 +9345,19 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Rollen stillingstittelen gir (S3 i #831).</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.hr_kopi</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>bruker_id</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -9434,7 +9377,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -9444,14 +9387,14 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Den som godkjente, returnerte eller trakk pakken.</t>
+          <t>Brukeren HR-kopien gjelder. Synkroniseringen registrerer Entra-identiteten når den mangler (svaret 20.10 i #831).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>koe.stillingstittel</t>
+          <t>koe.hr_kopi</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -9485,90 +9428,6 @@
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
-        <is>
-          <t>Rollen stillingstittelen gir (S3 i #831).</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="2" t="inlineStr">
-        <is>
-          <t>koe.hr_kopi</t>
-        </is>
-      </c>
-      <c r="B131" s="2" t="inlineStr">
-        <is>
-          <t>bruker_id</t>
-        </is>
-      </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t>koe.app_users</t>
-        </is>
-      </c>
-      <c r="D131" s="2" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E131" s="2" t="inlineStr">
-        <is>
-          <t>Fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t>én til én</t>
-        </is>
-      </c>
-      <c r="G131" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
-      <c r="H131" s="2" t="inlineStr">
-        <is>
-          <t>Brukeren HR-kopien gjelder. Synkroniseringen registrerer Entra-identiteten når den mangler (svaret 20.10 i #831).</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>koe.hr_kopi</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>rolle</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>koe.rolle</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>rolle</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr">
-        <is>
-          <t>Fremmednøkkel</t>
-        </is>
-      </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>mange til én</t>
-        </is>
-      </c>
-      <c r="G132" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
-      <c r="H132" s="2" t="inlineStr">
         <is>
           <t>Rollen personen har etter siste synkronisering, eller ingen.</t>
         </is>

</xml_diff>

<commit_message>
legg til sakslisten i TS: koe_api.saksliste og GET /api/projects/<p>/saker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019JcUQpmaKbsXwmbdgnhzyv
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting.</t>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting. Sakslisten leser sakene i prosjektet med journalen gjennom `koe_api.saksliste`, under radsikkerheten, fra `server/saksliste.ts` (#1022).</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4).</t>
+          <t>Journalen: ett dokument per brev, med teksten slik den ble sendt. En trigger avviser endring og sletting. Teamet står bare når det er entydig (DL-U4). Sakslisten leser hendelsene i prosjektet gjennom `koe_api.saksliste` og regner statusen og tallene i kjernen ved lesing; ingen oppsummering lagres (#1022).</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">

</xml_diff>

<commit_message>
stopp kontraktsteamene i catenda_admin.py og vis til TS-verktøyet
`contract-teams` og `register --bh/--te` skrev kontraktsteamene uten
bekreftelsen etter DL-U14. Begge avvises nå med exit 2 og en melding som
viser til `server/registrering.ts`. `AuthRepository.set_contract_teams`
hadde ingen andre kallere og er fjernet; den levende testen kaller
`koe_set_contract_teams` direkte. Dataflyten C18 og C19 og
`catenda_contract_teams` i tabellregisteret viser til TS-skriptet.

Closes #1072

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016fzG12hExTZELCRJW5pcUB
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Av `koe_set_contract_teams` og `koe_register_project`, som drift kaller gjennom `scripts/catenda_admin.py`. Etter B-02 punkt 4 er det bare drift som skal gjøre dette.</t>
+          <t>Av `koe_set_contract_teams` og `koe_register_project`. Ingen kode i repoet kaller dem med team lenger: `scripts/catenda_admin.py` avviser `--bh` og `--te` og viser til `server/registrering.ts`, som skriver kontraktsteamene i SQL Server (#1072). Etter B-02 punkt 4 er det bare drift som skal gjøre dette.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/catenda_admin.py:cmd_register; backend/repositories/auth_repository.py:AuthRepository.register_project; databasefunksjon:koe_register_project; databasefunksjon:koe_set_contract_teams</t>
+          <t>server/registrering.ts:kjoer; server/registrering.ts:catendaTeam; server/registrering.ts:registrer</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -12390,7 +12390,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py contract-teams` med `--bh` og `--te`.</t>
+          <t>`server/registrering.ts kontraktsteam` med `--bh`, `--te` og `--en-totalentreprenoer`.</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -12410,7 +12410,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/catenda_admin.py:cmd_contract_teams; backend/repositories/auth_repository.py:AuthRepository.set_contract_teams; databasefunksjon:koe_set_contract_teams</t>
+          <t>server/registrering.ts:kjoer; server/registrering.ts:catendaTeam; server/registrering.ts:settKontraktsteam</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">

</xml_diff>

<commit_message>
rett funnene fra code-review i #1100
Pilene for kontraktsteamene går til koe.catenda_contract_teams, C18 nevner
TS-skriptet som utløser for teamene, contract-teams viser meldingen også
når --bh står først, og meldingen har KOE_DRIFT_TILKOBLING og viser til
teams for PostgreSQL-teamene.

Del av #1072

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016fzG12hExTZELCRJW5pcUB
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Av `koe_set_contract_teams` og `koe_register_project`. Ingen kode i repoet kaller dem med team lenger: `scripts/catenda_admin.py` avviser `--bh` og `--te` og viser til `server/registrering.ts`, som skriver kontraktsteamene i SQL Server (#1072). Etter B-02 punkt 4 er det bare drift som skal gjøre dette.</t>
+          <t>Av `koe_set_contract_teams` og `koe_register_project`. Ingen driftskommando kaller dem med team lenger: `scripts/catenda_admin.py` avviser `--bh` og `--te` og viser til `server/registrering.ts`, som skriver kontraktsteamene i SQL Server (#1072). Bare de levende testene gir `koe_register_project` team. Etter B-02 punkt 4 er det bare drift som skal gjøre dette.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Ja. `team_id` er en Catenda-ID. Dataflyt: fra Catenda i C18, C19 (arket Dataflyt).</t>
+          <t>Ja. `team_id` er en Catenda-ID. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Delvis. Team-ID-en kommer fra Catenda; kontraktssiden settes av driften. Dataflyt: fra Catenda i C18, C19 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12249,7 +12249,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py register`.</t>
+          <t>`scripts/catenda_admin.py register`; teamene bare `server/registrering.ts registrer` med `--bh` og `--te`.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -12296,7 +12296,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py register`.</t>
+          <t>`scripts/catenda_admin.py register`; teamene bare `server/registrering.ts registrer` med `--bh` og `--te`.</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -12306,7 +12306,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -12343,7 +12343,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>`scripts/catenda_admin.py register`.</t>
+          <t>`scripts/catenda_admin.py register`; teamene bare `server/registrering.ts registrer` med `--bh` og `--te`.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>catenda_contract_teams</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">

</xml_diff>

<commit_message>
oppdater datamodellen og EO-dokumentet etter at frontenden ikke kaller EO-rutene
Retter også kommentarene i diffen til norsk og fjerner endringshistorikken i
projects.ts (reviewet av #1109).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2cFeTDKgbg33Q6zTH5m8p
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -11544,7 +11544,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/forsering/&lt;sak_id&gt;/relaterte` og `/kontekst`, og `GET /api/endringsordre/&lt;sak_id&gt;/relaterte` og `/kontekst`.</t>
+          <t>`GET /api/forsering/&lt;sak_id&gt;/relaterte` og `/kontekst`, og `GET /api/endringsordre/&lt;sak_id&gt;/relaterte` og `/kontekst`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -11591,7 +11591,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/forsering/&lt;sak_id&gt;/relaterte` og `/kontekst`, og `GET /api/endringsordre/&lt;sak_id&gt;/relaterte` og `/kontekst`.</t>
+          <t>`GET /api/forsering/&lt;sak_id&gt;/relaterte` og `/kontekst`, og `GET /api/endringsordre/&lt;sak_id&gt;/relaterte` og `/kontekst`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -11826,7 +11826,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`.</t>
+          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -11873,7 +11873,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`.</t>
+          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -11920,7 +11920,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`.</t>
+          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`.</t>
+          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -12014,7 +12014,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`.</t>
+          <t>`POST /api/endringsordre/opprett`, utstedelse etter godkjenning, og `POST /api/endringsordre/&lt;sak_id&gt;/koe` og `DELETE …/koe/&lt;koe_sak_id&gt;`. Frontenden kaller ikke rutene.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">

</xml_diff>

<commit_message>
før forfatterkontrollen for kommentaren inn i dataflyten C23 (#972)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KV14x4MArz2v57zB5EugKn
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -9444,7 +9444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12959,7 +12959,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Catenda: kommentarer</t>
+          <t>Catenda: innlogget bruker</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>GET /opencde/bcf/3.0/projects/{catenda_board_id}/topics/{catenda_topic_id}/comments</t>
+          <t>GET /v2/user</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -12979,7 +12979,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>Kommentarene på topicen, med ID og tekst. Står samme tekst der, brukes den kommentarens ID. Lagres ikke.</t>
+          <t>Integrasjonens brukernavn (`username`), som skiller kommentarer integrasjonen skrev. Lagres ikke.</t>
         </is>
       </c>
     </row>
@@ -13006,17 +13006,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>Catenda: kommentarer</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Catenda: kommentarer</t>
+          <t>Appen, lagres ikke</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>POST /opencde/bcf/3.0/projects/{catenda_board_id}/topics/{catenda_topic_id}/comments</t>
+          <t>GET /opencde/bcf/3.0/projects/{catenda_board_id}/topics/{catenda_topic_id}/comments</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Kommentaren for utfallet (`comment`), bare når samme tekst ikke står på topicen.</t>
+          <t>Kommentarene på topicen, med ID, tekst og forfatter (`author`). Har integrasjonens brukernavn skrevet samme tekst der, brukes den kommentarens ID. Lagres ikke.</t>
         </is>
       </c>
     </row>
@@ -13053,27 +13053,27 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
+          <t>koe.innkommende_behandling</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
           <t>Catenda: kommentarer</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>koe.topic_kommentar</t>
-        </is>
-      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Svaret fra Catenda</t>
+          <t>POST /opencde/bcf/3.0/projects/{catenda_board_id}/topics/{catenda_topic_id}/comments</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>server/jobber.ts:skrivEnKommentar; server/hendelser.ts:kvitterKommentar</t>
+          <t>server/jobber.ts:skrivEnKommentar; server/catenda.ts:innboksintegrasjon; server/catenda.ts:CatendaOAuth</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>ID-en til kommentaren i Catenda, funnet eller skrevet.</t>
+          <t>Kommentaren for utfallet (`comment`), bare når integrasjonen ikke har skrevet samme tekst på topicen.</t>
         </is>
       </c>
     </row>
@@ -13105,20 +13105,67 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
+          <t>koe.topic_kommentar</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Svaret fra Catenda</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>server/jobber.ts:skrivEnKommentar; server/hendelser.ts:kvitterKommentar</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>ID-en til kommentaren i Catenda, funnet eller skrevet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>C23.5</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>C23 Kommentaren tilbake til topicen fra innboksen i TS-serveren</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>ut</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Løkka i jobbkjøreren, etter behandlingen av innboksen: `skrivEnKommentar` i `server/jobber.ts` tar det eldste utfallet i `koe.innkommende_behandling` som skal ha en kommentar, ikke har en kvittering og ikke venter etter et forsøk (W-1b.2, #819).</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Catenda: kommentarer</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
           <t>koe.innkommende_forsoek</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>Svaret fra Catenda, eller at det mangler</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>server/jobber.ts:skrivEnKommentar; server/hendelser.ts:registrerForsoek</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="I79" s="2" t="inlineStr">
         <is>
           <t>Steget `kommentar` og feilklassen med meldingen, når Catenda eller basen ikke svarte.</t>
         </is>

</xml_diff>

<commit_message>
avvis en Catenda-tittel PDF-en ikke kan vise, og kommenter tegnene
En topic fra TE med et tegn i tittelen som brev-PDF-en ikke kan vise, gir
utfallet tittel_kan_ikke_vises og en kommentar i topicen med tegnene. En
senere endring av topicen (issue.modified) er et nytt forsøk på
opprettelsen når tittelen er avvist før (arbeidsvalgene 22.10 i #1138).

Migrasjonen legger utfallet til i CHECK-en, gir neste_kommentar meldingen
og legger til oppslaget koe_api.tittel_avvist_for_topic.

Del av #1138

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B35sTxns8bMgChAPtUfwP7
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -3644,7 +3644,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet.</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board. Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet. En topic fra TE med et tegn i tittelen som PDF-en av brevet ikke kan vise, får `tittel_kan_ikke_vises` med tegnene i `melding`, og en senere endring av topicen er da et nytt forsøk på opprettelsen (`koe_api.tittel_avvist_for_topic`, arbeidsvalgene 22.10 i #1138).</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er en fast feiltekst fra serveren.</t>
+          <t>Nei. `melding` er en fast feiltekst fra serveren, for `tittel_kan_ikke_vises` med tegnene fra topicens tittel.</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
+          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) og `tittel_kan_ikke_vises` (arbeidsvalgene 22.10 i #1138) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">

</xml_diff>

<commit_message>
avgjør prosjektgrensen og kvitteringen uavhengig av kontraktssiden
To prosedyrer i koe_api kjører som koe_grenseoppslag, en bruker uten
innlogging som filterpredikatene på koe.sak_metadata og koe.kvittering
slipper gjennom for et aktivt medlem i prosjektet i konteksten.
krevProsjekttilgang avgjør da prosjektgrensen før siden, som i Flask, og
innboksen leser kvitteringen med bare aktøren og prosjektet.

Del av #1106.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PatsFuvFJYMMTgQ1FUpwBa
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting. Sakslisten leser sakene i prosjektet med journalen gjennom `koe_api.saksliste`, under radsikkerheten, fra `server/saksliste.ts` (#1022).</t>
+          <t>Saksregisteret: saken, prosjektet og sakstypen. En trigger avviser endring og sletting. Sakslisten leser sakene i prosjektet med journalen gjennom `koe_api.saksliste`, under radsikkerheten, fra `server/saksliste.ts` (#1022). Tilgangskontrollen leser om sakene det vises til er i prosjektet, uavhengig av siden, med `koe_api.saker_i_prosjektet` fra `server/autorisasjon.ts` (#1106).</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`.</t>
+          <t>`koe_api.skriv_hendelse` og `koe_api.opprett_sak`, og leses av `koe_api.kvittering`, kalt fra `skrivHendelse` og `opprettSak` i `server/kommandoer.ts`, fra `POST /api/kjerne/saker` og `POST /api/kjerne/saker/&lt;sak_id&gt;/kommandoer`. Innboksen leser saken i kvitteringen uavhengig av siden med `koe_api.kvittert_sak`, fra `kvittertSak` i `server/kommandoer.ts` (#1106).</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">

</xml_diff>

<commit_message>
godta boardet i sakens topickobling og gjør registrer_behandling idempotent før boardkontrollen
Etter /code-review high på #1207: et topicboard byttet mellom oppslaget og
lagringen ga ukjent_prosjekt for en sak som alt var opprettet. Prosedyren
godtar nå også boardet i koe.sak_catenda_topic for saken og topicen, og
gjør ingenting når hendelsen alt har et utfall. dataflyt.toml leser email.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8vJXa66E6bDodRgUdQZqS
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -3644,7 +3644,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board; prosedyren godtar bare topicboardet til prosjektet med utfallet (punkt 8 i #972). Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet. En topic fra TE med et tegn i tittelen som PDF-en av brevet ikke kan vise, får `tittel_kan_ikke_vises` med tegnene i `melding`, og en senere endring av topicen er da et nytt forsøk på opprettelsen, til topicen har fått en sak (`koe_api.tittel_avvist_for_topic`, arbeidsvalgene 22.10 i #1138).</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board; prosedyren godtar bare topicboardet til prosjektet med utfallet, eller boardet i topickoblingen til saken med utfallet (punkt 8 i #972). Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet. En topic fra TE med et tegn i tittelen som PDF-en av brevet ikke kan vise, får `tittel_kan_ikke_vises` med tegnene i `melding`, og en senere endring av topicen er da et nytt forsøk på opprettelsen, til topicen har fått en sak (`koe_api.tittel_avvist_for_topic`, arbeidsvalgene 22.10 i #1138).</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -12979,7 +12979,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>Integrasjonens brukernavn (`username`), som skiller kommentarer integrasjonen skrev. Lagres ikke.</t>
+          <t>Integrasjonens e-post (`email`), som er `author` på kommentarene integrasjonen skrev (#972). Lagres ikke.</t>
         </is>
       </c>
     </row>
@@ -13026,7 +13026,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Kommentarene på topicen, med ID, tekst og forfatter (`author`). Har integrasjonens brukernavn skrevet samme tekst der, brukes den kommentarens ID. Lagres ikke.</t>
+          <t>Kommentarene på topicen, med ID, tekst og forfatter (`author`). Har integrasjonens e-post skrevet samme tekst der, brukes den kommentarens ID. Lagres ikke.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
lagre navnene på byggherren og totalentreprenøren i TS-stien og gi dem i prosjektet (#1398)
Ny tabell koe.kontraktsparter, satt av driften med kommandoen
kontraktsparter i server/registrering.ts gjennom koe_drift.sett_kontraktsparter.
GET /api/projects/:id leser dem med koe_api.kontraktsparter innenfor
medlemskapet og gir dem i settings.contract. Arbeidsvalgene 30.10 i #1398.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/datamodell/tabellbeskrivelse.xlsx
+++ b/docs/datamodell/tabellbeskrivelse.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Vises til fra: koe.app_membership_absences.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_membership_sync.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.app_project_memberships.project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_contract_teams.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.catenda_project_configs.internal_project_id (fremmednøkkel, ON DELETE NO ACTION); koe.dagmulktssats.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.kontraktsparter.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); koe.sak_metadata.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3240,29 +3240,29 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.kontraktsparter</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, verdien kjeden ble avledet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
+          <t>Navnene på byggherren og totalentreprenøren i prosjektet (#1398). Ett prosjekt er én kontrakt (DL-U14). Begge navnene settes sammen, og uten rad har prosjektet ingen navn. Et sendt brev fryser navnene det viste (LV-U1, #1173).</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Driftsskriptet `server/registrering.ts kontraktsparter`. Lest av `koe_api.kontraktsparter` fra `server/prosjekter.ts` (`GET /api/projects/:id`, `settings.contract`).</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Nei</t>
-        </is>
-      </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>transaksjon</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3290,19 +3290,19 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
+          <t>Ingen. Navnene er virksomheter.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne i en pakke i kjedens rekkefølge, avledet av hierarkiet i `koe.hr_kopi` da pakken ble laget (GFK-U8, GFK-U10). Endres ikke.</t>
+          <t>Et svar fra byggherren til intern godkjenning (S-1a, #818): brevet, grunnlaget fullmakten ble regnet av, verdien kjeden ble avledet av, saksbehandleren og teamet. Pakken er et utkast som bare teamet som laget den, ser, og uten team finnes den ikke (AGENTS.md). Den endres ikke; en ny pakke kan erstatte en returnert eller trukket.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id); unik (pakke_id, prosjekt_id, aktor_team_id); unik indeks (forrige_pakke_id) WHERE ([forrige_pakke_id] IS NOT NULL). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forrige_pakke_id → koe.godkjenningspakke.pakke_id (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION); aktor_team_id → koe.catenda_contract_teams.team_id (uten fremmednøkkel). Vises til fra: koe.godkjenningshandling.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); koe.godkjenningssteg.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3347,19 +3347,19 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Godkjennerne (`godkjenner_id`).</t>
+          <t>Saksbehandleren (`aktor_id`) og innholdet i svaret.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser rollen (`fullmakt_tittel`) og grensen godkjenneren hadde i `koe.rolle` da den ble gitt, så den står om rollen endres senere (B-04 punkt 2). Endres ikke.</t>
+          <t>Godkjennerne i en pakke i kjedens rekkefølge, avledet av hierarkiet i `koe.hr_kopi` da pakken ble laget (GFK-U8, GFK-U10). Endres ikke.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
+          <t>`koe_api.lag_godkjenningspakke`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, steg); unik (pakke_id, godkjenner_id). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); godkjenner_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.godkjenningshandling.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3404,19 +3404,19 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
+          <t>Godkjennerne (`godkjenner_id`).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>koe.leveringskvittering</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
+          <t>Hver godkjenning, retur og trekking av en pakke, i rekkefølge. En godkjenning fryser rollen (`fullmakt_tittel`) og grensen godkjenneren hadde i `koe.rolle` da den ble gitt, så den står om rollen endres senere (B-04 punkt 2). Endres ikke.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.registrer_godkjenningshandling`, kalt fra `server/godkjenning.ts`.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3436,12 +3436,12 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (pakke_id, loepenr); unik indeks (pakke_id) WHERE ([handling]&lt;&gt;N'godkjent'); unik indeks (pakke_id, steg) WHERE ([handling]=N'godkjent'). Viser til: (pakke_id, prosjekt_id, aktor_team_id) → koe.godkjenningspakke.(pakke_id, prosjekt_id, aktor_team_id) (fremmednøkkel, ON DELETE NO ACTION); (pakke_id, steg) → koe.godkjenningssteg.(pakke_id, steg) (fremmednøkkel, ON DELETE NO ACTION); aktor_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.(godkjenningshandling_pakke_id, godkjenningshandling_loepenr) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3461,19 +3461,19 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Den som handlet (`aktor_id`) og begrunnelsen for en retur.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>koe.vedleggskvittering</t>
+          <t>koe.leveringskvittering</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
+          <t>Kvitteringen for hver obligatoriske operasjon i leveringen av et brev (#371 del 1, invariant 7): `dokument` når dokumentet ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Brevet er levert når begge radene finnes (B-03, arbeidsvalget 18.10 i #371). Et registrert brev har ingen rader (LV-U11); vedleggene kvitteres i `koe.vedleggskvittering`. Raden har leasen og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. Kjøretiden leser tidspunktet for `dokumentreferanse` som «levert» i visningen av saken (`lesOppdrag` i `server/lager.ts`, #764).</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+          <t>`koe_api.kvitter_dokument` og `koe_api.kvitter_levering`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (leveringsoppdrag_id, operasjon). Viser til: (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, forutsetning) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(leveringskvittering_oppdrag_id, leveringskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3525,37 +3525,37 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_catenda_topic</t>
+          <t>koe.vedleggskvittering</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
+          <t>Kvitteringen for hver operasjon i leveringen av et vedlegg (V-3, del av #790, invariant 7): `dokument` når vedlegget ligger i biblioteket, og `dokumentreferanse` når referansen står på topicen. Kvitteringen gjelder vedlegget, ikke oppdraget, så et vedlegg et senere brev viser til igjen, leveres ikke på nytt. Raden har leasen, oppdraget som leverte og ID-en Catenda ga, og endres ikke. Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad. `koe_api.kvitter_levering` kvitterer leveringen som fullført først når hvert vedlegg i brevet har en referanse.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.kvitter_vedlegg`, kalt av jobbkjøreren i `server/jobber.ts`.</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (vedlegg_id, operasjon). Viser til: vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedlegg_id, forutsetning) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); (leveringsoppdrag_id, prosjekt_id) → koe.leveringsoppdrag.(id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION); forsoek_id → koe.jobbforsoek.forsoek_id (uten fremmednøkkel). Vises til fra: koe.toemmingsvern.(vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3565,12 +3565,12 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>grunndata</t>
+          <t>transaksjon</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -3582,12 +3582,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_hendelse</t>
+          <t>koe.sak_catenda_topic</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
+          <t>Sakens topic i Catenda, med boardet. Én rad per sak, som bare kan legges til: topicen lages etter at saken er lagret, og saksraden er uforanderlig. `koe_api.leveringsmaal` leser den, og leveringsoppdraget fryser topicen, eller null uten rad (F0b-7, #661). Samme topic hører ikke til to saker (#741 punkt 17). En sak fra en topic i Catenda kobles til topicen i transaksjonen som oppretter saken (W-1b.1, #819). Bare kjøreveien, `koe_jobbkjoerer`, kan legge inn en rad.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3597,22 +3597,22 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
+          <t>`koe_api.kvitter_topic`, kalt av jobbkjøreren i `server/jobber.ts` etter at topicen er laget i Catenda (#741), og `koe_api.koble_topic`, kalt bare fra `koe_api.opprett_sak` når saken opprettes fra en topic i innboksen (W-1b.1, #819).</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Nei</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
+          <t>Ja, ID-ene er Catendas. Dataflyt: fra Catenda i C22 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id); unik (catenda_topic_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.sak_catenda_topic_sak_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3622,29 +3622,29 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>grunndata</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_behandling</t>
+          <t>koe.innkommende_hendelse</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board; prosedyren godtar bare topicboardet til prosjektet med utfallet, eller boardet i topickoblingen til saken med utfallet (punkt 8 i #972). Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet. En topic fra TE med et tegn i tittelen som PDF-en av brevet ikke kan vise, får `tittel_kan_ikke_vises` med tegnene i `melding`, og en senere endring av topicen er da et nytt forsøk på opprettelsen, til topicen har fått en sak (`koe_api.tittel_avvist_for_topic`, arbeidsvalgene 22.10 i #1138).</t>
+          <t>Innboksen for webhooken fra Catenda (W-1a, #819). Hver hendelse lagres rå, med kilden, `event.id` og `event.type`, før svaret 200, og samme ID fra samme kilde lagres én gang (INT-02). Prosjektet og saken er ikke avgjort ved mottaket, så tabellen har ingen `prosjekt_id` og ingen radsikkerhet; kjøretiden har ingen rett på den og skriver med `koe_api.motta_hendelse`. Raden kan ikke endres eller slettes. Hendelsene behandles av `server/hendelser.ts`, og utfallet står i `koe.innkommende_behandling` (W-1b.1).</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
+          <t>`koe_api.motta_hendelse`, kalt av webhooken i `server/webhook.ts`.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
+          <t>Ja, hele kroppen er Catendas. Dataflyt: fra Catenda i C21 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id); unik indeks (kilde, hendelse_id). Vises til fra: koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.innkommende_forsoek.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); koe.toemmingsvern.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3689,19 +3689,19 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er en fast feiltekst fra serveren, for `tittel_kan_ikke_vises` med tegnene fra topicens tittel.</t>
+          <t>Ja: kroppen har navnet og e-postadressen til den som laget topicen i Catenda.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>koe.innkommende_forsoek</t>
+          <t>koe.innkommende_behandling</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
+          <t>Utfallet for hver hendelse i innboksen, én rad når behandlingen er ferdig (W-1b.1, #819). En hendelse uten rad er ikke behandlet. Bare en ny topic laget av TE gir en sak, med topicens tittel (KT-U6); en topic fra BH gir ingen sak (KT-U7), og heller ikke en topic som alt hører til en sak eller er laget av integrasjonen (#741 punkt 17). Saken og prosjektet står bare når utfallet er `sak_opprettet`, og prosjektet når koblingen til Catenda-prosjektet og boardet ga det. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_behandling`. Boardet topicen ble slått opp på, står med utfallet, så kommentaren skrives på samme board; prosedyren godtar bare topicboardet til prosjektet med utfallet, eller boardet i topickoblingen til saken med utfallet (punkt 8 i #972). Raden kan ikke endres eller slettes; kommentaren tilbake til topicen (W-1b.2) står i `koe.topic_kommentar` og endrer ikke utfallet. En topic fra TE med et tegn i tittelen som PDF-en av brevet ikke kan vise, får `tittel_kan_ikke_vises` med tegnene i `melding`, og en senere endring av topicen er da et nytt forsøk på opprettelsen, til topicen har fått en sak (`koe_api.tittel_avvist_for_topic`, arbeidsvalgene 22.10 i #1138).</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
+          <t>`koe_api.registrer_behandling`, kalt av `behandleEnHendelse` i `server/jobber.ts` med utfallet fra `server/hendelser.ts`.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
+          <t>Delvis. ID-en til topicen er Catendas. Dataflyt: fra Catenda i C22; til Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_behandling_id (fremmednøkkel, ON DELETE NO ACTION); koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3746,19 +3746,19 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
+          <t>Nei. `melding` er en fast feiltekst fra serveren, for `tittel_kan_ikke_vises` med tegnene fra topicens tittel.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>koe.topic_kommentar</t>
+          <t>koe.innkommende_forsoek</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) og `tittel_kan_ikke_vises` (arbeidsvalgene 22.10 i #1138) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
+          <t>Forsøkene uten utfall for en hendelse i innboksen (W-1b.2, #819), med steget: `behandling` eller `kommentar`. Et forsøk lagres når Catenda eller basen ikke svarte. Hendelsen venter da før neste forsøk, lenger for hvert forsøk (30 s, dobbelt for hvert, høyst en time), og løkka går videre, så én hendelse ikke stenger innboksen (#963). `topic_ikke_funnet` merker forsøkene der Catenda ikke fant topicen; bare de teller mot grensen for `ugyldig_hendelse`. `koe_api.neste_innkommende` og `koe_api.neste_kommentar` hopper over en hendelse som venter. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.registrer_innkommende_forsoek`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
+          <t>`koe_api.registrer_innkommende_forsoek`, kalt av `behandleEnHendelse` og `skrivEnKommentar` i `server/jobber.ts`.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
+          <t>Delvis. `melding` kan være feilmeldingen fra Catenda. Dataflyt: fra Catenda i C22, C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (id). Viser til: innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.innkommende_forsoek_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3803,19 +3803,19 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Nei. `melding` er feilklassen og meldingen fra Catenda eller basen, uten saksdata.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>koe.prosjekt_med_saker</t>
+          <t>koe.topic_kommentar</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
+          <t>Kvitteringen for kommentaren løkka skrev tilbake på topicen i Catenda (W-1b.2, #819), én rad per utfall. Utfallet `sak_opprettet` gir en kommentar med lenke og saksnummer (KT-U6), `topic_fra_bh` (KT-U7) og `sakstype_ikke_stoettet` (arbeidsvalget under OV-U1 i #819) og `tittel_kan_ikke_vises` (arbeidsvalgene 22.10 i #1138) en kommentar om hvorfor ingen sak er opprettet. Kommentarene på topicen leses først, og står teksten der alt, kvitteres den, så samme tekst skrives én gang. Kjøretiden har ingen rett på tabellen og skriver med `koe_api.kvitter_kommentar`. Raden kan ikke endres eller slettes.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
+          <t>`koe_api.kvitter_kommentar`, kalt av `skrivEnKommentar` i `server/jobber.ts` etter at kommentaren er funnet eller skrevet i Catenda.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3835,12 +3835,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Ja, ID-en til kommentaren er Catendas. Dataflyt: fra Catenda i C23 (arket Dataflyt).</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (innkommende_hendelse_id). Viser til: innkommende_hendelse_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.topic_kommentar_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3860,19 +3860,19 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Ingen kjente.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>koe.skrivetidspunkt</t>
+          <t>koe.prosjekt_med_saker</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Prosjektene som har minst én sak. Radsikkerheten skjuler sakene også for eieren, så `koe_drift.sett_kontraktsteam` leser her om kontraktsteamene bare kan få nye team (svaret 18.10 i #764, F-1, #820). Raden kan ikke endres eller slettes. Hadde `koe.sak_metadata` rader da migrasjonen ble anvendt, ble hvert prosjekt ført, fordi sakene ikke kunne leses.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
+          <t>Triggeren `koe.sak_metadata_prosjekt_med_saker`, i samme transaksjon som den første saken i prosjektet.</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3892,12 +3892,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
+          <t>Nøkler: primærnøkkel (prosjekt_id). Viser til: prosjekt_id → koe.projects.id (fremmednøkkel, ON DELETE NO ACTION). Vises til fra: koe.toemmingsvern.prosjekt_med_saker_id (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3924,12 +3924,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>koe.toemmingsvern</t>
+          <t>koe.skrivetidspunkt</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
+          <t>Tidspunktet basen ga for skrivingen i en transaksjon, med økt-ID-en som nøkkel, og transaksjonen og når økta logget inn, fordi transaksjons-ID-en begynner på nytt etter en omstart. `koe_api.skriv_hendelse` godtar bare dette tidspunktet på brevet, i samme transaksjon og økt (DL-U3, svaret 16.10 i #53), og bare i 30 sekunder etter at det ble gitt (#599). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
+          <t>`koe_api.skrivetidspunkt` fører raden, og `koe_api.skriv_hendelse` sletter den i samme transaksjon. Kalt fra `skrivHendelse` i `server/kommandoer.ts`, som ruller tilbake når den ikke skriver. En kaller som committer uten å skrive, etterlater raden; `skrivetidspunkt` erstatter den neste gang samme økt-ID fører et tidspunkt. Tabellen har høyst én rad per økt-ID.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (oekt). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3974,19 +3974,19 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Nei.</t>
+          <t>Ingen kjente.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>koe.kjernebuffer</t>
+          <t>koe.toemmingsvern</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
+          <t>Vernet mot TRUNCATE for de uforanderlige tabellene ingen annen fremmednøkkel viser til (#582). TRUNCATE avfyrer ingen trigger, men avvises for en tabell en fremmednøkkel viser til. En nøkkel en tabell har til seg selv, hindrer ikke TRUNCATE. Tabellen kan ikke ha rader (`toemmingsvern_tom`), og kjøretiden har ingen rett på den.</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Ingen skriver ennå (#53, del 3).</t>
+          <t>Ingen. Migrasjonen lager tabellen, og skranken avviser hver rad.</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: ingen. Viser til: app_identities_id → koe.app_identities.id (fremmednøkkel, ON DELETE NO ACTION); brevdokument_id → koe.brevdokument.leveringsoppdrag_id (fremmednøkkel, ON DELETE NO ACTION); (godkjenningshandling_pakke_id, godkjenningshandling_loepenr) → koe.godkjenningshandling.(pakke_id, loepenr) (fremmednøkkel, ON DELETE NO ACTION); (kvittering_prosjekt_id, kvittering_aktor_id, kvittering_kommando_id) → koe.kvittering.(prosjekt_id, aktor_id, kommando_id) (fremmednøkkel, ON DELETE NO ACTION); (leveringskvittering_oppdrag_id, leveringskvittering_operasjon) → koe.leveringskvittering.(leveringsoppdrag_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION); innkommende_hendelse_id → koe.innkommende_hendelse.id (fremmednøkkel, ON DELETE NO ACTION); innkommende_behandling_id → koe.innkommende_behandling.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); innkommende_forsoek_id → koe.innkommende_forsoek.id (fremmednøkkel, ON DELETE NO ACTION); topic_kommentar_id → koe.topic_kommentar.innkommende_hendelse_id (fremmednøkkel, ON DELETE NO ACTION); prosjekt_med_saker_id → koe.prosjekt_med_saker.prosjekt_id (fremmednøkkel, ON DELETE NO ACTION); sak_catenda_topic_sak_id → koe.sak_catenda_topic.sak_id (fremmednøkkel, ON DELETE NO ACTION); vedlegg_id → koe.vedlegg.vedlegg_id (fremmednøkkel, ON DELETE NO ACTION); (vedleggskvittering_vedlegg_id, vedleggskvittering_operasjon) → koe.vedleggskvittering.(vedlegg_id, operasjon) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -4021,29 +4021,29 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>avledet</t>
+          <t>teknisk</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>uavklart</t>
+          <t>i bruk</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Som journalen den er regnet fra.</t>
+          <t>Nei.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>koe.app_sessions</t>
+          <t>koe.kjernebuffer</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+          <t>Visningen kjernen regner ut av journalen, med versjonene den er regnet med (B-10). Ingen regel og ingen bindende kommando leser den.</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+          <t>Ingen skriver ennå (#53, del 3).</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -4063,12 +4063,12 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+          <t>Nei Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+          <t>Nøkler: primærnøkkel (sak_id). Viser til: (sak_id, prosjekt_id) → koe.sak_metadata.(sak_id, prosjekt_id) (fremmednøkkel, ON DELETE NO ACTION).</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -4078,72 +4078,129 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>teknisk</t>
+          <t>avledet</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>i bruk</t>
+          <t>uavklart</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+          <t>Som journalen den er regnet fra.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>koe.app_sessions</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Innloggingssesjoner. Lagrer SHA-256 av sesjonstokenet, CSRF-tokenet og når sesjonen utløper, 8 timer etter opprettelsen. Svarer til `app_sessions` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>`koe_api.opprett_sesjon` oppretter, `koe_api.slett_sesjon` sletter og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av tilbakekallet og utloggingen i `server/innlogging.ts` (F0b-5a, #659).</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Nei</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Nei. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Nøkler: primærnøkkel (token_hash). Viser til: user_id → koe.app_users.id (fremmednøkkel, ON DELETE NO ACTION).</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>teknisk</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>i bruk</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Knyttet til en bruker gjennom `user_id`, med når sesjonen ble opprettet (`created_at`) og når den utløper (`expires_at`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
           <t>koe.app_oauth_attempts</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Påbegynte innlogginger mot Catenda (OAuth). Lagrer SHA-256 av staten og av nettlesertokenet, returstien og når forsøket utløper, 600 sekunder etter opprettelsen. Svarer til `app_oauth_attempts` i PostgreSQL (B-19, #656). Kjøretiden har ingen rett på tabellen.</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>`koe_api.opprett_innloggingsforsoek` oppretter, `koe_api.bruk_innloggingsforsoek` sletter raden når den brukes, og `koe_api.rydd_utloepte` sletter utløpte rader. Kalt fra `server/sesjon.ts`, av innloggingen og tilbakekallet i `server/innlogging.ts` (F0b-5a, #659).</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>Nei</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Nei, men raden hører til en innlogging hos Catenda. Dataflyt: ingen kall til Catenda skriver eller leser tabellen.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>Nøkler: primærnøkkel (state_hash). Ingen relasjoner til andre tabeller.</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>SQL Server</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>teknisk</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>i bruk</t>
         </is>
       </c>
-      <c r="K65" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>Ingen kjente; bare hasher og en returadresse.</t>
         </is>
@@ -4160,7 +4217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H130"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8936,22 +8993,22 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.kontraktsparter</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>prosjekt_id</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>koe.sak_metadata</t>
+          <t>koe.projects</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>(sak_id, prosjekt_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -8961,7 +9018,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>mange til én</t>
+          <t>én til én</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -8971,7 +9028,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
+          <t>Prosjektet navnene gjelder i. Uten rad har prosjektet ingen navn på partene (#1398).</t>
         </is>
       </c>
     </row>
@@ -8983,17 +9040,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>forrige_pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.sak_metadata</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>pakke_id</t>
+          <t>(sak_id, prosjekt_id)</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -9013,7 +9070,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
+          <t>Saken svaret i pakken gjelder, i samme prosjekt.</t>
         </is>
       </c>
     </row>
@@ -9025,17 +9082,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>forrige_pakke_id</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>pakke_id</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -9055,7 +9112,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Saksbehandleren som utarbeidet svaret.</t>
+          <t>Pakken som ble returnert eller trukket, og som denne erstatter.</t>
         </is>
       </c>
     </row>
@@ -9067,22 +9124,22 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>aktor_team_id</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>koe.catenda_contract_teams</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>team_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Uten fremmednøkkel</t>
+          <t>Fremmednøkkel</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -9090,37 +9147,41 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G122" s="2" t="inlineStr"/>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
+          <t>Saksbehandleren som utarbeidet svaret.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>aktor_team_id</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.catenda_contract_teams</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>team_id</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Fremmednøkkel</t>
+          <t>Uten fremmednøkkel</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -9128,14 +9189,10 @@
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G123" s="2" t="inlineStr">
-        <is>
-          <t>NO ACTION</t>
-        </is>
-      </c>
+      <c r="G123" s="2" t="inlineStr"/>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
+          <t>Teamet som ser pakken. Basen avviser en pakke uten team (AGENTS.md).</t>
         </is>
       </c>
     </row>
@@ -9147,17 +9204,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>godkjenner_id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -9177,29 +9234,29 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Godkjenneren i steget.</t>
+          <t>Pakken steget hører til, med samme prosjekt og team, så radsikkerheten leser dem i steget.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningshandling</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>godkjenner_id</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningspakke</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
@@ -9219,7 +9276,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
+          <t>Godkjenneren i steget.</t>
         </is>
       </c>
     </row>
@@ -9231,17 +9288,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>koe.godkjenningssteg</t>
+          <t>koe.godkjenningspakke</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>(pakke_id, steg)</t>
+          <t>(pakke_id, prosjekt_id, aktor_team_id)</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -9261,7 +9318,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
+          <t>Pakken handlingen gjelder, med samme prosjekt og team.</t>
         </is>
       </c>
     </row>
@@ -9273,17 +9330,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>aktor_id</t>
+          <t>(pakke_id, steg)</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.godkjenningssteg</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>(pakke_id, steg)</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -9303,29 +9360,29 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Den som godkjente, returnerte eller trakk pakken.</t>
+          <t>Steget som er godkjent eller returnert. En trekking har ikke steg.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>koe.stillingstittel</t>
+          <t>koe.godkjenningshandling</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>rolle</t>
+          <t>aktor_id</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>koe.rolle</t>
+          <t>koe.app_users</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>rolle</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -9345,29 +9402,29 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Rollen stillingstittelen gir (S3 i #831).</t>
+          <t>Den som godkjente, returnerte eller trakk pakken.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>koe.hr_kopi</t>
+          <t>koe.stillingstittel</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>bruker_id</t>
+          <t>rolle</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>koe.app_users</t>
+          <t>koe.rolle</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>rolle</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -9377,7 +9434,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>én til én</t>
+          <t>mange til én</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -9387,7 +9444,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Brukeren HR-kopien gjelder. Synkroniseringen registrerer Entra-identiteten når den mangler (svaret 20.10 i #831).</t>
+          <t>Rollen stillingstittelen gir (S3 i #831).</t>
         </is>
       </c>
     </row>
@@ -9399,35 +9456,77 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
+          <t>bruker_id</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>koe.app_users</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Fremmednøkkel</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>én til én</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>NO ACTION</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Brukeren HR-kopien gjelder. Synkroniseringen registrerer Entra-identiteten når den mangler (svaret 20.10 i #831).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>koe.hr_kopi</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
           <t>rolle</t>
         </is>
       </c>
-      <c r="C130" s="2" t="inlineStr">
+      <c r="C131" s="2" t="inlineStr">
         <is>
           <t>koe.rolle</t>
         </is>
       </c>
-      <c r="D130" s="2" t="inlineStr">
+      <c r="D131" s="2" t="inlineStr">
         <is>
           <t>rolle</t>
         </is>
       </c>
-      <c r="E130" s="2" t="inlineStr">
+      <c r="E131" s="2" t="inlineStr">
         <is>
           <t>Fremmednøkkel</t>
         </is>
       </c>
-      <c r="F130" s="2" t="inlineStr">
+      <c r="F131" s="2" t="inlineStr">
         <is>
           <t>mange til én</t>
         </is>
       </c>
-      <c r="G130" s="2" t="inlineStr">
+      <c r="G131" s="2" t="inlineStr">
         <is>
           <t>NO ACTION</t>
         </is>
       </c>
-      <c r="H130" s="2" t="inlineStr">
+      <c r="H131" s="2" t="inlineStr">
         <is>
           <t>Rollen personen har etter siste synkronisering, eller ingen.</t>
         </is>

</xml_diff>